<commit_message>
Add and classify ReconVLA
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Ra078d83f57944d9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rc632b7f507494fa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R044287c5419b4ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R1670bed94b0e42b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rbe2f9d4ce39b43af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R93f4beeda8d74d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R39e67a1570be4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R94f30f9d000040e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R85f281c7f6e64a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R86ee3682b76940e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Ra925f705a993474b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R2f2db1c47bd64a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc69743c2062a4de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R90fd38ad14c74b69"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -384,7 +384,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:Z78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:Z79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="26">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -418,7 +418,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:AU66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:AU67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="47">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -4134,7 +4134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b919a0a6a874e11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae73188e4af4fb4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7430,7 +7430,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7641a7b927524ea7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbda72b59aaa42f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7781,7 +7781,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca0e250dc37451d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7b89ee07ff4da0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8527,7 +8527,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd68244e1786e49b6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0cf507806594083"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14285,6 +14285,86 @@
         <x:v>02_Papers/10_Benchmark_Dataset/Open_X-Embodiment.md</x:v>
       </x:c>
     </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>D078</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>ReconVLA: Reconstructive Vision-Language-Action Model as Effective Robot Perceiver</x:v>
+      </x:c>
+      <x:c r="C79" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Method Paper</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>AAAI</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Official Conference Paper (AAAI-26 Technical Track on Intelligent Robotics)</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>VLA; Robot Manipulation; Generalization; Diffusion</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>Visual Grounding / Robot Perception / Gaze-Region Reconstruction</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>VLA; Robot Manipulation; Visual Grounding; Robot Perception; Implicit Grounding; Gaze-Region Reconstruction; Generalization; Diffusion Transformer</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>https://arxiv.org/abs/2508.10333</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>https://zionchow.github.io/ReconVLA/</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>https://github.com/OpenHelix-Team/ReconVLA</x:v>
+      </x:c>
+      <x:c r="O79" t="str">
+        <x:v>Released</x:v>
+      </x:c>
+      <x:c r="P79" t="str">
+        <x:v>Partial — source datasets and preprocessing instructions are public; compiled pretraining dataset release not verified</x:v>
+      </x:c>
+      <x:c r="Q79" t="str">
+        <x:v>Unknown — no author-released ReconVLA checkpoint located</x:v>
+      </x:c>
+      <x:c r="R79" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S79" t="str">
+        <x:v>Single Arm / Parallel Gripper</x:v>
+      </x:c>
+      <x:c r="T79" t="str">
+        <x:v>AAAI Proceedings / author project page / official GitHub</x:v>
+      </x:c>
+      <x:c r="U79" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="V79" t="str">
+        <x:v>Special Attention: Yes. Abstract-level / 未精读. Official repository includes training, evaluation, and preprocessing code; code was not run locally.</x:v>
+      </x:c>
+      <x:c r="W79" t="str">
+        <x:v>Official AAAI proceedings, arXiv, author project page, and official repository verified; CCF A verified on current official CCF list</x:v>
+      </x:c>
+      <x:c r="X79" t="str">
+        <x:v>2026-09-20</x:v>
+      </x:c>
+      <x:c r="Y79" t="str">
+        <x:v>VLA</x:v>
+      </x:c>
+      <x:c r="Z79" t="str">
+        <x:v>02_Papers/01_VLA/ReconVLA.md</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="D2:D78">
@@ -14305,7 +14385,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51b4725aeaf4284"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32a7cae7933340e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23712,6 +23792,149 @@
         <x:v>Bimanual</x:v>
       </x:c>
     </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>A066</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>ReconVLA: Reconstructive Vision-Language-Action Model as Effective Robot Perceiver</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
+        <x:v>Wenxuan Song; Ziyang Zhou; Han Zhao; Jiayi Chen; Pengxiang Ding; Haodong Yan; Yuxin Huang; Feilong Tang; Donglin Wang; Haoang Li</x:v>
+      </x:c>
+      <x:c r="D67" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>AAAI</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>Official Conference Paper</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>Method Paper</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>VLA; Robot Manipulation; Generalization; Diffusion</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>Visual Grounding / Robot Perception / Gaze-Region Reconstruction</x:v>
+      </x:c>
+      <x:c r="K67" t="str">
+        <x:v>VLA; Robot Manipulation; Visual Grounding; Robot Perception; Implicit Grounding; Gaze-Region Reconstruction; Generalization; Diffusion Transformer</x:v>
+      </x:c>
+      <x:c r="L67" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921</x:v>
+      </x:c>
+      <x:c r="M67" t="str">
+        <x:v>10.1609/aaai.v40i22.38921</x:v>
+      </x:c>
+      <x:c r="N67" t="str">
+        <x:v>https://arxiv.org/abs/2508.10333</x:v>
+      </x:c>
+      <x:c r="O67" t="str">
+        <x:v>https://zionchow.github.io/ReconVLA/</x:v>
+      </x:c>
+      <x:c r="P67" t="str">
+        <x:v>https://github.com/OpenHelix-Team/ReconVLA</x:v>
+      </x:c>
+      <x:c r="Q67" t="str">
+        <x:v>Released</x:v>
+      </x:c>
+      <x:c r="R67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="S67" t="str">
+        <x:v>Unknown — no author-released ReconVLA checkpoint located</x:v>
+      </x:c>
+      <x:c r="T67" t="str">
+        <x:v>Partial — source datasets and preprocessing instructions are public; compiled pretraining dataset release not verified</x:v>
+      </x:c>
+      <x:c r="U67" t="str">
+        <x:v>Franka Panda (CALVIN simulation); real-world platform not confirmed at abstract level</x:v>
+      </x:c>
+      <x:c r="V67" t="str">
+        <x:v>Single Arm / Parallel Gripper</x:v>
+      </x:c>
+      <x:c r="W67" t="str">
+        <x:v>Single Arm</x:v>
+      </x:c>
+      <x:c r="X67" t="str">
+        <x:v>Parallel Gripper</x:v>
+      </x:c>
+      <x:c r="Y67" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z67" t="str">
+        <x:v>BridgeData V2; LIBERO; CALVIN (source datasets); curated 100k+ trajectories / 2M samples reported</x:v>
+      </x:c>
+      <x:c r="AA67" t="str">
+        <x:v>CALVIN; real-world manipulation tasks</x:v>
+      </x:c>
+      <x:c r="AB67" t="str">
+        <x:v>Yes (CALVIN)</x:v>
+      </x:c>
+      <x:c r="AC67" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="AD67" t="str">
+        <x:v>Official AAAI proceedings, arXiv, author project page, and official repository verified; CCF A verified on current official CCF list</x:v>
+      </x:c>
+      <x:c r="AE67" t="str">
+        <x:v>2026-09-20</x:v>
+      </x:c>
+      <x:c r="AF67" t="str">
+        <x:v>Special Attention: Yes. Abstract-level / 未精读. Code status reflects static verification of training, evaluation, and preprocessing implementation; no local run.</x:v>
+      </x:c>
+      <x:c r="AG67" t="str">
+        <x:v>CCF A Conference</x:v>
+      </x:c>
+      <x:c r="AH67" t="str">
+        <x:v>Official Conference Paper</x:v>
+      </x:c>
+      <x:c r="AI67" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AJ67" t="str">
+        <x:v>Discovery / 未读</x:v>
+      </x:c>
+      <x:c r="AK67" t="str">
+        <x:v>02_Papers/01_VLA/ReconVLA.md</x:v>
+      </x:c>
+      <x:c r="AL67" t="str">
+        <x:v>Strict CCF A</x:v>
+      </x:c>
+      <x:c r="AM67" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921; https://arxiv.org/abs/2508.10333; https://zionchow.github.io/ReconVLA/; https://github.com/OpenHelix-Team/ReconVLA</x:v>
+      </x:c>
+      <x:c r="AN67" t="str">
+        <x:v>Abstract-level / 未精读</x:v>
+      </x:c>
+      <x:c r="AO67" t="str">
+        <x:v>Current VLA models often allocate dispersed visual attention and fail to focus precisely on task target regions.</x:v>
+      </x:c>
+      <x:c r="AP67" t="str">
+        <x:v>Introduces reconstructive VLA with implicit grounding and a robot pretraining dataset of 100k+ trajectories and 2M samples.</x:v>
+      </x:c>
+      <x:c r="AQ67" t="str">
+        <x:v>A diffusion transformer reconstructs gaze regions from VLA visual outputs, encouraging fine-grained target-region representations and accurate visual attention.</x:v>
+      </x:c>
+      <x:c r="AR67" t="str">
+        <x:v>Official paper reports CALVIN simulation and real-world experiments supporting precise manipulation, long-horizon performance, and generalization to unseen targets.</x:v>
+      </x:c>
+      <x:c r="AS67" t="str">
+        <x:v>Relevant to VLA perception, target grounding, manipulation precision, and generalization; useful as an auxiliary reconstruction objective reference.</x:v>
+      </x:c>
+      <x:c r="AT67" t="str">
+        <x:v>Current official CCF Artificial Intelligence list checked 2026-09-20: AAAI is A</x:v>
+      </x:c>
+      <x:c r="AU67" t="str">
+        <x:v>VLA</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="10">
     <x:dataValidation type="list" sqref="F2:F51">
@@ -23747,7 +23970,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b19e9f710234bbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7130ba24d5064a71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25286,7 +25509,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc92d01c7d4074a4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09688c328b794cf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Verify and update Sim2Real-VLA
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R94f30f9d000040e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R85f281c7f6e64a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R86ee3682b76940e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Ra925f705a993474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R2f2db1c47bd64a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc69743c2062a4de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R90fd38ad14c74b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rf20c5345323f4b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rf343ef705194437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Ra883011712f24cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rd2861bec75884cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R77a93c54c2f046d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rcd7c79e334b644ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rfcc63173bb0a44bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4134,7 +4134,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae73188e4af4fb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27857e2f4e0948b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7430,7 +7430,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbda72b59aaa42f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R948e4587c85b4c39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7781,7 +7781,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7b89ee07ff4da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5992c9c785d49d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8527,7 +8527,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0cf507806594083"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc16559e87cc441f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14385,7 +14385,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32a7cae7933340e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1286900ceee44021"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23970,7 +23970,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7130ba24d5064a71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99b6d246eb1e427d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24154,7 +24154,7 @@
         <x:v>Official Conference Paper</x:v>
       </x:c>
       <x:c r="H2" s="23" t="str">
-        <x:v>Unknown (project standard conflict; official CCF row pending)</x:v>
+        <x:v>Unknown (current official CCF directory checked; no authoritative ICLR A row located in accessible current listing)</x:v>
       </x:c>
       <x:c r="I2" s="23" t="str">
         <x:v>VLA / Robot Manipulation / Sim2Real</x:v>
@@ -24166,16 +24166,16 @@
         <x:v>VLA; Sim2Real; Robot Manipulation; Synthetic Data; Generalization; Bimanual; Dexterous; Long-horizon</x:v>
       </x:c>
       <x:c r="L2" s="23" t="str">
-        <x:v>Synthetic-only VLA training usually transfers unreliably to real manipulation.</x:v>
+        <x:v>Synthetic-only VLA training often fails to transfer reliably to real manipulation; the paper targets this Sim2Real gap.</x:v>
       </x:c>
       <x:c r="M2" s="23" t="str">
-        <x:v>Dual-system VLA with chain-of-affordances planning and tokenized low-level action execution; automated synthetic skill generation and real-world evaluation.</x:v>
+        <x:v>Dual-system VLA with high-level chain-of-affordances planning, low-level tokenized action execution/validation, and automated synthetic manipulation-skill generation.</x:v>
       </x:c>
       <x:c r="N2" s="23" t="str">
         <x:v>Filter manipulation-irrelevant variation and retain motion-critical affordance structure for zero-shot transfer.</x:v>
       </x:c>
       <x:c r="O2" s="23" t="str">
-        <x:v>https://openreview.net/pdf?id=H4SyKHjd4c</x:v>
+        <x:v>https://openreview.net/pdf/a4174c2964dc0df03c26c311b73e0a2e43de2929.pdf</x:v>
       </x:c>
       <x:c r="P2" s="23" t="str">
         <x:v>https://edem-ai.github.io/sim2realvla.github.io/</x:v>
@@ -24184,16 +24184,16 @@
         <x:v>https://github.com/DexForce/EmbodiChain</x:v>
       </x:c>
       <x:c r="R2" s="23" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Partial (official project links the paper implementation as an integration into EmbodiChain; no standalone paper repository)</x:v>
       </x:c>
       <x:c r="S2" s="23" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="T2" s="23" t="str">
-        <x:v>Automated synthetic manipulation-skill data; release status Unknown</x:v>
+        <x:v>Automated synthetic manipulation-skill data; complete public release not confirmed</x:v>
       </x:c>
       <x:c r="U2" s="23" t="str">
-        <x:v>Multiple platforms shown by official project; exact model names pending full-paper verification</x:v>
+        <x:v>Multiple real-world setups are shown; exact hardware inventory not extracted at abstract/project level</x:v>
       </x:c>
       <x:c r="V2" s="23" t="str">
         <x:v>Single Arm / Bimanual / Dexterous Hand</x:v>
@@ -24211,13 +24211,13 @@
         <x:v>Discovery / 未读</x:v>
       </x:c>
       <x:c r="AA2" s="23" t="str">
-        <x:v>ICLR 2026 publication confirmed by official ICLR proceedings and accepted OpenReview PDF; code integration is partial</x:v>
+        <x:v>ICLR 2026 publication verified through official ICLR Downloads/Proceedings listing, accepted OpenReview PDF, author project page, and author publication list; code remains Partial integration.</x:v>
       </x:c>
       <x:c r="AB2" s="53" t="str">
-        <x:v>2026-09-19</x:v>
+        <x:v>2026-09-21</x:v>
       </x:c>
       <x:c r="AC2" s="23" t="str">
-        <x:v>Do not place in strict CCF_A_Library until the project's CCF seventh-edition mapping conflict is resolved.</x:v>
+        <x:v>Current official CCF directory was checked; ICLR A status was not authoritatively located, so CCF remains Unknown and the paper stays in Robotics Core / Important Papers.</x:v>
       </x:c>
       <x:c r="AD2" s="23" t="str">
         <x:v>02_Papers/05_Sim2Real/Sim2Real-VLA.md</x:v>
@@ -24226,19 +24226,19 @@
         <x:v>Robotics Core / Important Papers</x:v>
       </x:c>
       <x:c r="AF2" s="23" t="str">
-        <x:v>Official ICLR proceedings; accepted OpenReview PDF; official project page; official GitHub</x:v>
+        <x:v>ICLR Downloads/Proceedings; accepted OpenReview PDF; official project page; official EmbodiChain repository; author publication list; current official CCF directory</x:v>
       </x:c>
       <x:c r="AG2" s="23" t="str">
-        <x:v>Abstract-level</x:v>
+        <x:v>Abstract-level / 未精读</x:v>
       </x:c>
       <x:c r="AH2" s="23" t="str">
-        <x:v>Official project reports six manipulation tasks and real-world domain shifts.</x:v>
+        <x:v>Official project reports six robot manipulation tasks spanning single-arm, dual-arm, hand-over and pan-opening/placement settings, plus domain-gap conditions; exact full-paper benchmark table not re-extracted.</x:v>
       </x:c>
       <x:c r="AI2" s="23" t="str">
         <x:v>Directly relevant to VLA, synthetic data, generalization, dual-arm manipulation and real-world deployment.</x:v>
       </x:c>
       <x:c r="AJ2" s="23" t="str">
-        <x:v>CCF seventh edition: exact official row pending unless separately evidenced</x:v>
+        <x:v>CCF 7th edition current official directory checked 2026-09-21; no authoritative ICLR A row located in accessible current listing</x:v>
       </x:c>
       <x:c r="AK2" s="23" t="str">
         <x:v>Sim2Real</x:v>
@@ -25509,7 +25509,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09688c328b794cf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f35a59480584259"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Enrich papers batch 01
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R1d95b3a7d4474096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rddee10ba73044373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Re80d8134d58640f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R04bb7aeaa529491b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R4a34d64120bd4927"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R0a167107ef62482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R953a19614fa24be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rb78e0de66ebe4bc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R0fa1462e67ef4140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R807b83bc92554f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R55565df31e6c4a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R5ca2525dc163414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rce41f18a12ab45ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rbe6574d9f21c4cf3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="PapersTable" displayName="PapersTable" ref="A1:AT5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="46">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PapersTable" displayName="PapersTable" ref="A1:AZ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="52">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -348,6 +348,12 @@
     <x:tableColumn id="44" name="Remaining Unsolved Problem"/>
     <x:tableColumn id="45" name="Relevance to Our Project"/>
     <x:tableColumn id="46" name="Tags"/>
+    <x:tableColumn id="47" name="Evidence Quality"/>
+    <x:tableColumn id="48" name="Idea Clues"/>
+    <x:tableColumn id="49" name="Ablation Study"/>
+    <x:tableColumn id="50" name="Failure Cases"/>
+    <x:tableColumn id="51" name="Citation Source Identifier"/>
+    <x:tableColumn id="52" name="Evidence Sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -399,8 +405,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AO79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="41">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AU79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="47">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -442,14 +448,20 @@
     <x:tableColumn id="39" name="Remaining Unsolved Problem"/>
     <x:tableColumn id="40" name="Relevance to Our Project"/>
     <x:tableColumn id="41" name="Tags"/>
+    <x:tableColumn id="42" name="Evidence Quality"/>
+    <x:tableColumn id="43" name="Idea Clues"/>
+    <x:tableColumn id="44" name="Ablation Study"/>
+    <x:tableColumn id="45" name="Failure Cases"/>
+    <x:tableColumn id="46" name="Citation Source Identifier"/>
+    <x:tableColumn id="47" name="Evidence Sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BH67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="60">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BN67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="66">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="作者 Authors"/>
@@ -510,14 +522,20 @@
     <x:tableColumn id="58" name="Limitations"/>
     <x:tableColumn id="59" name="Remaining Unsolved Problem"/>
     <x:tableColumn id="60" name="Tags"/>
+    <x:tableColumn id="61" name="Evidence Quality"/>
+    <x:tableColumn id="62" name="Idea Clues"/>
+    <x:tableColumn id="63" name="Ablation Study"/>
+    <x:tableColumn id="64" name="Failure Cases"/>
+    <x:tableColumn id="65" name="Citation Source Identifier"/>
+    <x:tableColumn id="66" name="Evidence Sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:AW14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="49">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BC14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="55">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
     <x:tableColumn id="3" name="Authors"/>
@@ -567,6 +585,12 @@
     <x:tableColumn id="47" name="Main Results"/>
     <x:tableColumn id="48" name="Limitations"/>
     <x:tableColumn id="49" name="Remaining Unsolved Problem"/>
+    <x:tableColumn id="50" name="Evidence Quality"/>
+    <x:tableColumn id="51" name="Idea Clues"/>
+    <x:tableColumn id="52" name="Ablation Study"/>
+    <x:tableColumn id="53" name="Failure Cases"/>
+    <x:tableColumn id="54" name="Citation Source Identifier"/>
+    <x:tableColumn id="55" name="Evidence Sources"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -939,6 +963,24 @@
       <x:c r="AT1" t="str">
         <x:v>Tags</x:v>
       </x:c>
+      <x:c r="AU1" t="str">
+        <x:v>Evidence Quality</x:v>
+      </x:c>
+      <x:c r="AV1" t="str">
+        <x:v>Idea Clues</x:v>
+      </x:c>
+      <x:c r="AW1" t="str">
+        <x:v>Ablation Study</x:v>
+      </x:c>
+      <x:c r="AX1" t="str">
+        <x:v>Failure Cases</x:v>
+      </x:c>
+      <x:c r="AY1" t="str">
+        <x:v>Citation Source Identifier</x:v>
+      </x:c>
+      <x:c r="AZ1" t="str">
+        <x:v>Evidence Sources</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="350" customHeight="1">
       <x:c r="A2" t="str">
@@ -1077,6 +1119,24 @@
       </x:c>
       <x:c r="AT2" t="str">
         <x:v>Multimodal / Generalization</x:v>
+      </x:c>
+      <x:c r="AU2" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="AV2" t="str">
+        <x:v>Idea Clue 1: adapt affordance-prior reasoning and active impedance correction to ordinary-gripper bimanual contact tasks. Evidence: APR and AIA ablation gains plus explicit hardware failure cases. Why relevant: actionable path for current real-robot manipulation.</x:v>
+      </x:c>
+      <x:c r="AW2" t="str">
+        <x:v>Reported ablations isolate OCI, MLM, APR, COT and AIA; APR is the largest training-task gain in the cited ablation sequence.</x:v>
+      </x:c>
+      <x:c r="AX2" t="str">
+        <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
+      </x:c>
+      <x:c r="AY2" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4402727730</x:v>
+      </x:c>
+      <x:c r="AZ2" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="150" customHeight="1">
@@ -1186,6 +1246,24 @@
       <x:c r="AT3" t="str">
         <x:v>Residual Learning / Sim-to-Real</x:v>
       </x:c>
+      <x:c r="AU3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV3" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AW3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AX3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AY3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AZ3" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" t="str">
@@ -1294,6 +1372,24 @@
       <x:c r="AT4" t="str">
         <x:v>Diffusion / Contact-rich Manipulation</x:v>
       </x:c>
+      <x:c r="AU4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV4" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AW4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AX4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AY4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AZ4" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
       <x:c r="A5" t="str">
@@ -1401,6 +1497,24 @@
       </x:c>
       <x:c r="AT5" t="str">
         <x:v>Human Video / VLM</x:v>
+      </x:c>
+      <x:c r="AU5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV5" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AW5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AX5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AY5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AZ5" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4414,7 +4528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48df0fc37dae40bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dcb41bb5dcf4040"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7710,7 +7824,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0ae217572a94489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36f63375e94f492f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8061,7 +8175,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R925c82cc5c2e4e51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c918cd74c44125"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8807,7 +8921,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac20970add604579"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R554fa4d754eb4cc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8971,6 +9085,24 @@
       <x:c r="AO1" t="str">
         <x:v>Tags</x:v>
       </x:c>
+      <x:c r="AP1" t="str">
+        <x:v>Evidence Quality</x:v>
+      </x:c>
+      <x:c r="AQ1" t="str">
+        <x:v>Idea Clues</x:v>
+      </x:c>
+      <x:c r="AR1" t="str">
+        <x:v>Ablation Study</x:v>
+      </x:c>
+      <x:c r="AS1" t="str">
+        <x:v>Failure Cases</x:v>
+      </x:c>
+      <x:c r="AT1" t="str">
+        <x:v>Citation Source Identifier</x:v>
+      </x:c>
+      <x:c r="AU1" t="str">
+        <x:v>Evidence Sources</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -9088,6 +9220,24 @@
       <x:c r="AO2" t="str">
         <x:v>Robot Manipulation; Diffusion Policy / Hierarchical Control</x:v>
       </x:c>
+      <x:c r="AP2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ2" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR2" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS2" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU2" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -9205,6 +9355,24 @@
       <x:c r="AO3" t="str">
         <x:v>bimanual manipulation; decoupled interaction; RoboTwin</x:v>
       </x:c>
+      <x:c r="AP3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ3" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU3" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -9322,6 +9490,24 @@
       <x:c r="AO4" t="str">
         <x:v>bimanual; diffusion; teleoperation; human demonstration</x:v>
       </x:c>
+      <x:c r="AP4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ4" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU4" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -9441,6 +9627,24 @@
       <x:c r="AO5" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ5" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -9558,6 +9762,24 @@
       <x:c r="AO6" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ6" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -9675,6 +9897,24 @@
       <x:c r="AO7" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ7" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -9790,6 +10030,24 @@
       <x:c r="AO8" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ8" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -9907,6 +10165,24 @@
       <x:c r="AO9" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ9" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -10022,6 +10298,24 @@
       <x:c r="AO10" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ10" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -10141,6 +10435,24 @@
       <x:c r="AO11" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ11" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -10258,6 +10570,24 @@
         <x:v>Unknown / Needs Project-Specific Review</x:v>
       </x:c>
       <x:c r="AO12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AP12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ12" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -10379,6 +10709,24 @@
       <x:c r="AO13" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ13" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -10496,6 +10844,24 @@
       <x:c r="AO14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ14" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR14" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS14" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -10613,6 +10979,24 @@
         <x:v>Unknown / Needs Project-Specific Review</x:v>
       </x:c>
       <x:c r="AO15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AP15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ15" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR15" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS15" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU15" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -10730,6 +11114,24 @@
       <x:c r="AO16" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ16" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR16" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS16" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -10845,6 +11247,24 @@
       <x:c r="AO17" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ17" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR17" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS17" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -10960,6 +11380,24 @@
       <x:c r="AO18" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ18" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR18" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS18" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -11077,6 +11515,24 @@
       <x:c r="AO19" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ19" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR19" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS19" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -11192,6 +11648,24 @@
       <x:c r="AO20" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ20" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR20" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS20" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -11309,6 +11783,24 @@
       <x:c r="AO21" t="str">
         <x:v>Robot Manipulation; Diffusion Policy / Primitive Skills</x:v>
       </x:c>
+      <x:c r="AP21" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ21" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR21" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS21" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT21" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU21" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -11426,6 +11918,24 @@
       <x:c r="AO22" t="str">
         <x:v>Imitation Learning; Multi-Task / Foresight</x:v>
       </x:c>
+      <x:c r="AP22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ22" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR22" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS22" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU22" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -11543,6 +12053,24 @@
       <x:c r="AO23" t="str">
         <x:v>Robot Manipulation; Long-Horizon / Visual-Tactile Policy</x:v>
       </x:c>
+      <x:c r="AP23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ23" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR23" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS23" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU23" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -11660,6 +12188,24 @@
       <x:c r="AO24" t="str">
         <x:v>Robot Manipulation; Humanoid / Generalization</x:v>
       </x:c>
+      <x:c r="AP24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ24" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR24" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS24" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU24" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -11775,6 +12321,24 @@
       <x:c r="AO25" t="str">
         <x:v>Dexterous Manipulation; Human Demonstrations / Motion Prior</x:v>
       </x:c>
+      <x:c r="AP25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ25" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR25" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS25" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU25" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -11892,6 +12456,24 @@
       <x:c r="AO26" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ26" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR26" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS26" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -12009,6 +12591,24 @@
       <x:c r="AO27" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ27" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR27" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS27" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -12126,6 +12726,24 @@
       <x:c r="AO28" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ28" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR28" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS28" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -12243,6 +12861,24 @@
       <x:c r="AO29" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ29" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR29" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS29" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -12360,6 +12996,24 @@
       <x:c r="AO30" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ30" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR30" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS30" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -12477,6 +13131,24 @@
       <x:c r="AO31" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ31" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR31" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS31" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -12594,6 +13266,24 @@
       <x:c r="AO32" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ32" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR32" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS32" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -12711,6 +13401,24 @@
       <x:c r="AO33" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ33" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR33" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS33" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -12828,6 +13536,24 @@
       <x:c r="AO34" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ34" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR34" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS34" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -12945,6 +13671,24 @@
       <x:c r="AO35" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ35" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR35" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS35" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -13062,6 +13806,24 @@
       <x:c r="AO36" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ36" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR36" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS36" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -13179,6 +13941,24 @@
       <x:c r="AO37" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ37" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR37" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS37" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -13296,6 +14076,24 @@
       <x:c r="AO38" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ38" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR38" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS38" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -13413,6 +14211,24 @@
       <x:c r="AO39" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ39" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR39" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS39" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -13528,6 +14344,24 @@
       <x:c r="AO40" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ40" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR40" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS40" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -13643,6 +14477,24 @@
       <x:c r="AO41" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ41" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR41" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS41" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -13758,6 +14610,24 @@
       <x:c r="AO42" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ42" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR42" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS42" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -13873,6 +14743,24 @@
       <x:c r="AO43" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ43" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR43" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS43" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -13988,6 +14876,24 @@
       <x:c r="AO44" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ44" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR44" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS44" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -14103,6 +15009,24 @@
       <x:c r="AO45" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ45" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR45" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS45" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -14220,6 +15144,24 @@
       <x:c r="AO46" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ46" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR46" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS46" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -14337,6 +15279,24 @@
       <x:c r="AO47" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ47" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR47" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS47" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -14454,6 +15414,24 @@
       <x:c r="AO48" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ48" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR48" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS48" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -14571,6 +15549,24 @@
       <x:c r="AO49" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ49" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR49" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS49" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -14688,6 +15684,24 @@
       <x:c r="AO50" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ50" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR50" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS50" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -14805,6 +15819,24 @@
       <x:c r="AO51" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ51" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR51" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS51" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -14922,6 +15954,24 @@
       <x:c r="AO52" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ52" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR52" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS52" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -15039,6 +16089,24 @@
       <x:c r="AO53" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ53" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR53" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS53" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -15156,6 +16224,24 @@
       <x:c r="AO54" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ54" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR54" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS54" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -15273,6 +16359,24 @@
       <x:c r="AO55" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ55" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR55" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS55" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -15390,6 +16494,24 @@
       <x:c r="AO56" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ56" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR56" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS56" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -15507,6 +16629,24 @@
       <x:c r="AO57" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ57" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR57" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS57" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -15630,6 +16770,24 @@
       <x:c r="AO58" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP58" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ58" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR58" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS58" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT58" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU58" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -15753,6 +16911,24 @@
       <x:c r="AO59" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP59" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ59" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR59" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS59" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT59" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU59" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -15874,6 +17050,24 @@
       <x:c r="AO60" t="str">
         <x:v>Bimanual; Benchmark / Synthetic Demonstrations</x:v>
       </x:c>
+      <x:c r="AP60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ60" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR60" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS60" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU60" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -15997,6 +17191,24 @@
       <x:c r="AO61" t="str">
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
+      <x:c r="AP61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ61" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR61" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS61" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU61" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -16120,6 +17332,24 @@
       <x:c r="AO62" t="str">
         <x:v>VLA; Inference Acceleration / Token Caching</x:v>
       </x:c>
+      <x:c r="AP62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ62" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR62" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS62" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU62" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -16243,6 +17473,24 @@
       <x:c r="AO63" t="str">
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
+      <x:c r="AP63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ63" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR63" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS63" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU63" t="str">
+        <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -16366,6 +17614,24 @@
       <x:c r="AO64" t="str">
         <x:v>VLA; World Model / 3D Generation</x:v>
       </x:c>
+      <x:c r="AP64" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="AQ64" t="str">
+        <x:v>Idea Clue 1: compare explicit 3D goal prediction against image-only VLA on dual-arm ordinary-gripper tasks. Evidence: paper motivation and 3D goal image/point-cloud generation. Why relevant: direct test of 3D planning value.</x:v>
+      </x:c>
+      <x:c r="AR64" t="str">
+        <x:v>Not Reported in the accessible proceedings page.</x:v>
+      </x:c>
+      <x:c r="AS64" t="str">
+        <x:v>Not Explicitly Reported in the accessible proceedings page.</x:v>
+      </x:c>
+      <x:c r="AT64" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4392886475</x:v>
+      </x:c>
+      <x:c r="AU64" t="str">
+        <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -16489,6 +17755,24 @@
       <x:c r="AO65" t="str">
         <x:v>VLA; Efficient Model / Pose Prediction</x:v>
       </x:c>
+      <x:c r="AP65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ65" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR65" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS65" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU65" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -16612,6 +17896,24 @@
       <x:c r="AO66" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ66" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR66" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS66" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="58" customHeight="1">
       <x:c r="A67" t="str">
@@ -16733,6 +18035,24 @@
         <x:v>Unknown / Needs Project-Specific Review</x:v>
       </x:c>
       <x:c r="AO67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AP67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ67" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR67" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS67" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU67" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -16856,6 +18176,24 @@
       <x:c r="AO68" t="str">
         <x:v>Robot Manipulation; Consistency Flow Matching / 3D Policy</x:v>
       </x:c>
+      <x:c r="AP68" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ68" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR68" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS68" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT68" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU68" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
       <x:c r="A69" t="str">
@@ -16979,6 +18317,24 @@
       <x:c r="AO69" t="str">
         <x:v>Dexterous Hand; Policy Distillation / Generalization</x:v>
       </x:c>
+      <x:c r="AP69" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ69" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR69" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS69" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT69" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU69" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" t="str">
@@ -17102,6 +18458,24 @@
       <x:c r="AO70" t="str">
         <x:v>Dexterous Hand; Residual RL / VLM Planning</x:v>
       </x:c>
+      <x:c r="AP70" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ70" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR70" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS70" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT70" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU70" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" t="str">
@@ -17225,6 +18599,24 @@
       <x:c r="AO71" t="str">
         <x:v>VLA; Video-Action Model / Generalization</x:v>
       </x:c>
+      <x:c r="AP71" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ71" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR71" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS71" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT71" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU71" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="58" customHeight="1">
       <x:c r="A72" t="str">
@@ -17348,6 +18740,24 @@
       <x:c r="AO72" t="str">
         <x:v>Dexterous Hand; Contact Reasoning / Language-guided Grasp</x:v>
       </x:c>
+      <x:c r="AP72" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ72" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR72" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS72" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT72" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU72" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="58" customHeight="1">
       <x:c r="A73" t="str">
@@ -17471,6 +18881,24 @@
       <x:c r="AO73" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP73" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ73" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR73" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS73" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT73" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU73" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="58" customHeight="1">
       <x:c r="A74" t="str">
@@ -17594,6 +19022,24 @@
       <x:c r="AO74" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP74" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ74" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR74" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS74" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT74" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU74" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="58" customHeight="1">
       <x:c r="A75" t="str">
@@ -17715,6 +19161,24 @@
         <x:v>Unknown / Needs Project-Specific Review</x:v>
       </x:c>
       <x:c r="AO75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AP75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ75" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR75" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS75" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -17836,6 +19300,24 @@
       <x:c r="AO76" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP76" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ76" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR76" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS76" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT76" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU76" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="58" customHeight="1">
       <x:c r="A77" t="str">
@@ -17953,6 +19435,24 @@
         <x:v>Unknown / Needs Project-Specific Review</x:v>
       </x:c>
       <x:c r="AO77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AP77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ77" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR77" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS77" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU77" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -18074,6 +19574,24 @@
       <x:c r="AO78" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AP78" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AQ78" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AR78" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AS78" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="AT78" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AU78" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -18198,6 +19716,24 @@
       </x:c>
       <x:c r="AO79" t="str">
         <x:v>VLA; Robot Manipulation; Visual Grounding; Robot Perception; Implicit Grounding; Gaze-Region Reconstruction; Generalization; Diffusion Transformer</x:v>
+      </x:c>
+      <x:c r="AP79" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="AQ79" t="str">
+        <x:v>Idea Clue 1: test implicit ga</x:v>
+      </x:c>
+      <x:c r="AR79" t="str">
+        <x:v>Not Reported in the official abstract/project evidence rechecked for this batch.</x:v>
+      </x:c>
+      <x:c r="AS79" t="str">
+        <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
+      </x:c>
+      <x:c r="AT79" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W7137985120</x:v>
+      </x:c>
+      <x:c r="AU79" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18220,7 +19756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93483fbba4d46d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf300a6bb39a34b35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18462,6 +19998,24 @@
       <x:c r="BH1" t="str">
         <x:v>Tags</x:v>
       </x:c>
+      <x:c r="BI1" t="str">
+        <x:v>Evidence Quality</x:v>
+      </x:c>
+      <x:c r="BJ1" t="str">
+        <x:v>Idea Clues</x:v>
+      </x:c>
+      <x:c r="BK1" t="str">
+        <x:v>Ablation Study</x:v>
+      </x:c>
+      <x:c r="BL1" t="str">
+        <x:v>Failure Cases</x:v>
+      </x:c>
+      <x:c r="BM1" t="str">
+        <x:v>Citation Source Identifier</x:v>
+      </x:c>
+      <x:c r="BN1" t="str">
+        <x:v>Evidence Sources</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -18636,6 +20190,24 @@
       <x:c r="BH2" t="str">
         <x:v>Robot Manipulation; Diffusion Policy / Hierarchical Control</x:v>
       </x:c>
+      <x:c r="BI2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ2" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK2" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL2" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN2" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -18810,6 +20382,24 @@
       <x:c r="BH3" t="str">
         <x:v>bimanual manipulation; decoupled interaction; RoboTwin</x:v>
       </x:c>
+      <x:c r="BI3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ3" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN3" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -18984,6 +20574,24 @@
       <x:c r="BH4" t="str">
         <x:v>bimanual; diffusion; teleoperation; human demonstration</x:v>
       </x:c>
+      <x:c r="BI4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ4" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN4" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -19158,6 +20766,24 @@
       <x:c r="BH5" t="str">
         <x:v>Robot Manipulation; Diffusion Policy / Primitive Skills</x:v>
       </x:c>
+      <x:c r="BI5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ5" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN5" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -19332,6 +20958,24 @@
       <x:c r="BH6" t="str">
         <x:v>Imitation Learning; Multi-Task / Foresight</x:v>
       </x:c>
+      <x:c r="BI6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ6" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN6" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -19506,6 +21150,24 @@
       <x:c r="BH7" t="str">
         <x:v>Robot Manipulation; Long-Horizon / Visual-Tactile Policy</x:v>
       </x:c>
+      <x:c r="BI7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ7" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN7" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -19680,6 +21342,24 @@
       <x:c r="BH8" t="str">
         <x:v>Robot Manipulation; Humanoid / Generalization</x:v>
       </x:c>
+      <x:c r="BI8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ8" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN8" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -19852,6 +21532,24 @@
       <x:c r="BH9" t="str">
         <x:v>Dexterous Manipulation; Human Demonstrations / Motion Prior</x:v>
       </x:c>
+      <x:c r="BI9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ9" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN9" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -20030,6 +21728,24 @@
       <x:c r="BH10" t="str">
         <x:v>Bimanual; Benchmark / Synthetic Demonstrations</x:v>
       </x:c>
+      <x:c r="BI10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ10" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN10" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -20210,6 +21926,24 @@
       <x:c r="BH11" t="str">
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
+      <x:c r="BI11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ11" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN11" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -20390,6 +22124,24 @@
       <x:c r="BH12" t="str">
         <x:v>VLA; Inference Acceleration / Token Caching</x:v>
       </x:c>
+      <x:c r="BI12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ12" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN12" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -20570,6 +22322,24 @@
       <x:c r="BH13" t="str">
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
+      <x:c r="BI13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ13" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN13" t="str">
+        <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -20750,6 +22520,24 @@
       <x:c r="BH14" t="str">
         <x:v>VLA; World Model / 3D Generation</x:v>
       </x:c>
+      <x:c r="BI14" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="BJ14" t="str">
+        <x:v>Idea Clue 1: compare explicit 3D goal prediction against image-only VLA on dual-arm ordinary-gripper tasks. Evidence: paper motivation and 3D goal image/point-cloud generation. Why relevant: direct test of 3D planning value.</x:v>
+      </x:c>
+      <x:c r="BK14" t="str">
+        <x:v>Not Reported in the accessible proceedings page.</x:v>
+      </x:c>
+      <x:c r="BL14" t="str">
+        <x:v>Not Explicitly Reported in the accessible proceedings page.</x:v>
+      </x:c>
+      <x:c r="BM14" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4392886475</x:v>
+      </x:c>
+      <x:c r="BN14" t="str">
+        <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -20929,6 +22717,24 @@
       </x:c>
       <x:c r="BH15" t="str">
         <x:v>VLA; Efficient Model / Pose Prediction</x:v>
+      </x:c>
+      <x:c r="BI15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ15" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK15" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL15" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN15" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -21108,6 +22914,24 @@
       <x:c r="BH16" t="str">
         <x:v>Robot Manipulation; Consistency Flow Matching / 3D Policy</x:v>
       </x:c>
+      <x:c r="BI16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ16" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK16" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL16" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN16" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -21288,6 +23112,24 @@
       <x:c r="BH17" t="str">
         <x:v>Dexterous Hand; Policy Distillation / Generalization</x:v>
       </x:c>
+      <x:c r="BI17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ17" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK17" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL17" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN17" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -21468,6 +23310,24 @@
       <x:c r="BH18" t="str">
         <x:v>Dexterous Hand; Residual RL / VLM Planning</x:v>
       </x:c>
+      <x:c r="BI18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ18" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK18" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL18" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN18" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -21648,6 +23508,24 @@
       <x:c r="BH19" t="str">
         <x:v>VLA; Video-Action Model / Generalization</x:v>
       </x:c>
+      <x:c r="BI19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ19" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK19" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL19" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN19" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -21828,6 +23706,24 @@
       <x:c r="BH20" t="str">
         <x:v>Dexterous Hand; Contact Reasoning / Language-guided Grasp</x:v>
       </x:c>
+      <x:c r="BI20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ20" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK20" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL20" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN20" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -22010,6 +23906,24 @@
       <x:c r="BH21" t="str">
         <x:v>Multimodal / Generalization</x:v>
       </x:c>
+      <x:c r="BI21" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="BJ21" t="str">
+        <x:v>Idea Clue 1: adapt affordance-prior reasoning and active impedance correction to ordinary-gripper bimanual contact tasks. Evidence: APR and AIA ablation gains plus explicit hardware failure cases. Why relevant: actionable path for current real-robot manipulation.</x:v>
+      </x:c>
+      <x:c r="BK21" t="str">
+        <x:v>Reported ablations isolate OCI, MLM, APR, COT and AIA; APR is the largest training-task gain in the cited ablation sequence.</x:v>
+      </x:c>
+      <x:c r="BL21" t="str">
+        <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
+      </x:c>
+      <x:c r="BM21" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4402727730</x:v>
+      </x:c>
+      <x:c r="BN21" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -22192,6 +24106,24 @@
       <x:c r="BH22" t="str">
         <x:v>Residual Learning / Sim-to-Real</x:v>
       </x:c>
+      <x:c r="BI22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ22" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK22" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL22" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN22" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -22374,6 +24306,24 @@
       <x:c r="BH23" t="str">
         <x:v>Diffusion / Contact-rich Manipulation</x:v>
       </x:c>
+      <x:c r="BI23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ23" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK23" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL23" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN23" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -22556,6 +24506,24 @@
       <x:c r="BH24" t="str">
         <x:v>Human Video / VLM</x:v>
       </x:c>
+      <x:c r="BI24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ24" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK24" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL24" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN24" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -22738,6 +24706,24 @@
       <x:c r="BH25" t="str">
         <x:v>Dexterous Grasping</x:v>
       </x:c>
+      <x:c r="BI25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ25" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK25" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL25" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN25" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Xu_Dexterous_Grasp_Transformer_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -22920,6 +24906,24 @@
       <x:c r="BH26" t="str">
         <x:v>Mobile Manipulation</x:v>
       </x:c>
+      <x:c r="BI26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ26" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK26" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL26" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN26" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wu_MoManipVLA_Transferring_Vision-language-action_Models_for_General_Mobile_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -23102,6 +25106,24 @@
       <x:c r="BH27" t="str">
         <x:v>Action Chunking / Multi-task Policy</x:v>
       </x:c>
+      <x:c r="BI27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ27" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK27" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL27" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN27" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/ff887781480973bd3cb6026feb378d1e-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -23284,6 +25306,24 @@
       <x:c r="BH28" t="str">
         <x:v>Surgical Robotics</x:v>
       </x:c>
+      <x:c r="BI28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ28" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK28" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL28" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN28" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/74c4f2b87b7499d365422152c76fd916-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -23466,6 +25506,24 @@
       <x:c r="BH29" t="str">
         <x:v>Video Demonstration / Reward Learning</x:v>
       </x:c>
+      <x:c r="BI29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ29" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK29" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL29" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN29" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/dcd297696d0bb304ba426b3c5a679c37-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -23648,6 +25706,24 @@
       <x:c r="BH30" t="str">
         <x:v>Long-Horizon / Failure Recovery</x:v>
       </x:c>
+      <x:c r="BI30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ30" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK30" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL30" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN30" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/fad8962279154544ed69bb63eb14d677-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -23830,6 +25906,24 @@
       <x:c r="BH31" t="str">
         <x:v>3D Observation / Contact-rich</x:v>
       </x:c>
+      <x:c r="BI31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ31" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK31" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL31" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN31" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/8e5dc5969a6174fcaaececd890c7f59b-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -24012,6 +26106,24 @@
       <x:c r="BH32" t="str">
         <x:v>Text-conditioned Reward</x:v>
       </x:c>
+      <x:c r="BI32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ32" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK32" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL32" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN32" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/5227ce00add5aa0a12d1c4ee92fcd2dc-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -24194,6 +26306,24 @@
       <x:c r="BH33" t="str">
         <x:v>Human-Robot Domain Adaptation</x:v>
       </x:c>
+      <x:c r="BI33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ33" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK33" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL33" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN33" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhou_Mitigating_the_Human-Robot_Domain_Discrepancy_in_Visual_Pre-training_for_Robotic_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -24376,6 +26506,24 @@
       <x:c r="BH34" t="str">
         <x:v>Grounding / Synthetic Data</x:v>
       </x:c>
+      <x:c r="BI34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ34" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK34" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL34" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN34" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Huang_RoboGround_Robotic_Manipulation_with_Grounded_Vision-Language_Priors_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -24558,6 +26706,24 @@
       <x:c r="BH35" t="str">
         <x:v>Synthetic Data / Scene Generation</x:v>
       </x:c>
+      <x:c r="BI35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ35" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK35" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL35" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN35" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -24740,6 +26906,24 @@
       <x:c r="BH36" t="str">
         <x:v>Lifelong Learning</x:v>
       </x:c>
+      <x:c r="BI36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ36" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK36" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL36" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN36" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Yao_Think_Small_Act_Big_Primitive_Prompt_Learning_for_Lifelong_Robot_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -24922,6 +27106,24 @@
       <x:c r="BH37" t="str">
         <x:v>Failure Recovery / 3D Gaussian Splatting</x:v>
       </x:c>
+      <x:c r="BI37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ37" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK37" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL37" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN37" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/34866；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -25104,6 +27306,24 @@
       <x:c r="BH38" t="str">
         <x:v>Articulated Object / Affordance</x:v>
       </x:c>
+      <x:c r="BI38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ38" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK38" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL38" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN38" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33615；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -25286,6 +27506,24 @@
       <x:c r="BH39" t="str">
         <x:v>Long-Horizon / Mobile Manipulation</x:v>
       </x:c>
+      <x:c r="BI39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ39" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK39" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL39" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN39" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33610；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -25468,6 +27706,24 @@
       <x:c r="BH40" t="str">
         <x:v>World Model / Video Diffusion</x:v>
       </x:c>
+      <x:c r="BI40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ40" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK40" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL40" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN40" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/481c70828a4ff20d31a646cc6cc95f3d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -25650,6 +27906,24 @@
       <x:c r="BH41" t="str">
         <x:v>Human Video / 3D Affordance</x:v>
       </x:c>
+      <x:c r="BI41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ41" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK41" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL41" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN41" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generalizable_3D_Actions_from_In-the-Wild_2D_Human_Videos_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -25832,6 +28106,24 @@
       <x:c r="BH42" t="str">
         <x:v>Visual Chain-of-Thought</x:v>
       </x:c>
+      <x:c r="BI42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ42" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK42" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL42" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN42" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhao_CoT-VLA_Visual_Chain-of-Thought_Reasoning_for_Vision-Language-Action_Models_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -26014,6 +28306,24 @@
       <x:c r="BH43" t="str">
         <x:v>Sim-to-Real / Behavior Cloning</x:v>
       </x:c>
+      <x:c r="BI43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ43" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK43" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL43" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN43" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1185c89347a3f21ffc48c9d083c9437c-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -26196,6 +28506,24 @@
       <x:c r="BH44" t="str">
         <x:v>Long-Horizon / Planning</x:v>
       </x:c>
+      <x:c r="BI44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ44" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK44" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL44" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN44" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b94310e1c7ecb79f1a24adc757f1b89b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -26378,6 +28706,24 @@
       <x:c r="BH45" t="str">
         <x:v>Stochastic Interpolant / Efficiency</x:v>
       </x:c>
+      <x:c r="BI45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ45" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK45" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL45" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN45" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/49eadcc4a329fc6b74b9f8a82b78cbc3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -26560,6 +28906,24 @@
       <x:c r="BH46" t="str">
         <x:v>Mobile Manipulation / Agent</x:v>
       </x:c>
+      <x:c r="BI46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ46" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK46" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL46" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN46" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/bc97207e3979d1cc23109db0be0e8ed2-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -26742,6 +29106,24 @@
       <x:c r="BH47" t="str">
         <x:v>Flow Matching / Visuomotor Policy</x:v>
       </x:c>
+      <x:c r="BI47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ47" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK47" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL47" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN47" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/282c3318be1b047b7bb5ba94fa4f3231-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -26924,6 +29306,24 @@
       <x:c r="BH48" t="str">
         <x:v>Tool Use / Generative Design</x:v>
       </x:c>
+      <x:c r="BI48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ48" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK48" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL48" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN48" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/9fc291fef2f9607a46777d367f900a15-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -27106,6 +29506,24 @@
       <x:c r="BH49" t="str">
         <x:v>3D Manipulation / Multimodal Policy</x:v>
       </x:c>
+      <x:c r="BI49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ49" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK49" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL49" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN49" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/eacc8ae341d15d2c13c02fef88189db3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -27288,6 +29706,24 @@
       <x:c r="BH50" t="str">
         <x:v>Robot Data / Spatial Reasoning</x:v>
       </x:c>
+      <x:c r="BI50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ50" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK50" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL50" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN50" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1f467c3e37abf9f86c78f44c6a27ee7c-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -27470,6 +29906,24 @@
       <x:c r="BH51" t="str">
         <x:v>Task Planning / Demonstrations</x:v>
       </x:c>
+      <x:c r="BI51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ51" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK51" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL51" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN51" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b8358a00e5b870194b974ddf8dd415c3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -27652,6 +30106,24 @@
       <x:c r="BH52" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ52" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK52" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL52" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN52" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Wang_DexH2R_A_Benchmark_for_Dynamic_Dexterous_Grasping_in_Human-to-Robot_Handover_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -27834,6 +30306,24 @@
       <x:c r="BH53" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ53" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK53" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL53" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN53" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhang_BimArt_A_Unified_Approach_for_the_Synthesis_of_3D_Bimanual_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -28016,6 +30506,24 @@
       <x:c r="BH54" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI54" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="BJ54" t="str">
+        <x:v>Idea Clue 1: use part-level language affordances as a perception front-end for bimanual grasp sequencing. Evidence: part-touch/part-grasp metrics and flow pose head. Why relevant: supports target-region and action alignment.</x:v>
+      </x:c>
+      <x:c r="BK54" t="str">
+        <x:v>The paper compares language-enabled DGN2.0* + CLIP against the full VLM/flow model; exact component ablations require supplementary extraction.</x:v>
+      </x:c>
+      <x:c r="BL54" t="str">
+        <x:v>The reported setting focuses on tabletop part-aligned grasps; broader clutter, occlusion and multi-step manipulation are not established by the cited results.</x:v>
+      </x:c>
+      <x:c r="BM54" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4417183400</x:v>
+      </x:c>
+      <x:c r="BN54" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/He_DexVLG_Dexterous_Vision-Language-Grasp_Model_at_Scale_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -28198,6 +30706,24 @@
       <x:c r="BH55" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ55" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK55" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL55" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN55" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generalizable_Hand_Object_Motion_Generation_with_Latent_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -28380,6 +30906,24 @@
       <x:c r="BH56" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ56" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK56" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL56" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN56" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generalizable_Bimanual_Tool-ACtion-Object_Understanding_CVPR_2024_paper.pdf；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -28562,6 +31106,24 @@
       <x:c r="BH57" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ57" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK57" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL57" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN57" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Uppal_SPIN_Simultaneous_Perception_Interaction_and_Navigation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -28744,6 +31306,24 @@
       <x:c r="BH58" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="BJ58" t="str">
+        <x:v>Idea Clue 1: use AnyBimanual as a baseline for ordinary-gripper dual-arm transfer with controlled demonstration budgets. Evidence: 12 RLBench2 + 9 real tasks and limited bimanual demonstrations. Why relevant: directly matches current bimanual project.</x:v>
+      </x:c>
+      <x:c r="BK58" t="str">
+        <x:v>The accessible arXiv text describes the separate skill-manager and visual-aligner contributions; full ablation numbers were not re-extracted in this batch.</x:v>
+      </x:c>
+      <x:c r="BL58" t="str">
+        <x:v>The paper identifies observation discrepancy between unimanual and bimanual systems as a transfer risk; detailed failure cases require appendix extraction.</x:v>
+      </x:c>
+      <x:c r="BM58" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W4405254485</x:v>
+      </x:c>
+      <x:c r="BN58" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Lu_AnyBimanual_Transferring_Unimanual_Policy_for_General_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -28926,6 +31506,24 @@
       <x:c r="BH59" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI59" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="BJ59" t="str">
+        <x:v>Idea Clue 1: borrow FAAS-style functional action grouping for dual-arm gripper role transfer. Evidence: unified cross-hand action coordinates. Why relevant: possible bridge from dexterous data to ordinary-gripper control.</x:v>
+      </x:c>
+      <x:c r="BK59" t="str">
+        <x:v>Not Reported in the accessible official abstract evidence.</x:v>
+      </x:c>
+      <x:c r="BL59" t="str">
+        <x:v>Cross-hand and retargeting edge cases are not detailed in the accessible abstract; full supplementary review is needed.</x:v>
+      </x:c>
+      <x:c r="BM59" t="str">
+        <x:v>OpenAlex Work: Unknown</x:v>
+      </x:c>
+      <x:c r="BN59" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Zhang_UniDex_A_Robot_Foundation_Suite_for_Universal_Dexterous_Hand_Control_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -29108,6 +31706,24 @@
       <x:c r="BH60" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ60" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK60" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL60" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN60" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhao_TASTE-Rob_Advancing_Video_Generation_of_Task-Oriented_Hand-Object_Interaction_for_Generalizable_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -29290,6 +31906,24 @@
       <x:c r="BH61" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ61" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK61" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL61" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN61" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38874；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -29472,6 +32106,24 @@
       <x:c r="BH62" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ62" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK62" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL62" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN62" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/e4ef7454447baa15a424314e6284441b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -29654,6 +32306,24 @@
       <x:c r="BH63" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ63" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK63" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL63" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN63" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38313；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -29836,6 +32506,24 @@
       <x:c r="BH64" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI64" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ64" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK64" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL64" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM64" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN64" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/40127；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -30018,6 +32706,24 @@
       <x:c r="BH65" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BJ65" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="BK65" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BL65" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BM65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BN65" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28266；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -30200,6 +32906,24 @@
       <x:c r="BH66" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BI66" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="BJ66" t="str">
+        <x:v>Idea Clue 1: evaluate predicted left/right/both affordances as a front-end for dual-arm task planning. Evidence: explicit hand-taxonomy decoder. Why relevant: actionable perception before VLA action generation.</x:v>
+      </x:c>
+      <x:c r="BK66" t="str">
+        <x:v>VLM-based versus CLIP-based affordance predictor is reported; exact ablation numbers require table extraction.</x:v>
+      </x:c>
+      <x:c r="BL66" t="str">
+        <x:v>The paper notes ambiguity/multi-modality of valid interaction regions; exact failure examples require figure-level review.</x:v>
+      </x:c>
+      <x:c r="BM66" t="str">
+        <x:v>OpenAlex Work: Unknown</x:v>
+      </x:c>
+      <x:c r="BN66" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Heidinger_2HandedAfforder_Learning_Precise_Actionable_Bimanual_Affordances_from_Human_Videos_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
@@ -30381,6 +33105,24 @@
       </x:c>
       <x:c r="BH67" t="str">
         <x:v>VLA; Robot Manipulation; Visual Grounding; Robot Perception; Implicit Grounding; Gaze-Region Reconstruction; Generalization; Diffusion Transformer</x:v>
+      </x:c>
+      <x:c r="BI67" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="BJ67" t="str">
+        <x:v>Idea Clue 1: test implicit ga</x:v>
+      </x:c>
+      <x:c r="BK67" t="str">
+        <x:v>Not Reported in the official abstract/project evidence rechecked for this batch.</x:v>
+      </x:c>
+      <x:c r="BL67" t="str">
+        <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
+      </x:c>
+      <x:c r="BM67" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W7137985120</x:v>
+      </x:c>
+      <x:c r="BN67" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -30418,7 +33160,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re18b2744b4b14791"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc302613323ef40fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30614,6 +33356,24 @@
       <x:c r="AW1" t="str">
         <x:v>Remaining Unsolved Problem</x:v>
       </x:c>
+      <x:c r="AX1" t="str">
+        <x:v>Evidence Quality</x:v>
+      </x:c>
+      <x:c r="AY1" t="str">
+        <x:v>Idea Clues</x:v>
+      </x:c>
+      <x:c r="AZ1" t="str">
+        <x:v>Ablation Study</x:v>
+      </x:c>
+      <x:c r="BA1" t="str">
+        <x:v>Failure Cases</x:v>
+      </x:c>
+      <x:c r="BB1" t="str">
+        <x:v>Citation Source Identifier</x:v>
+      </x:c>
+      <x:c r="BC1" t="str">
+        <x:v>Evidence Sources</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="62" customHeight="1">
       <x:c r="A2" t="str">
@@ -30763,6 +33523,24 @@
       <x:c r="AW2" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX2" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="AY2" t="str">
+        <x:v>Idea Clue 1: use affordance-conditioned dual-arm skill transfer as a controlled baseline for real gripper experiments. Evidence: official six-task and domain-gap evaluation. Why relevant: directly matches bimanual + sim2real direction.</x:v>
+      </x:c>
+      <x:c r="AZ2" t="str">
+        <x:v>Not Reported in the sources rechecked for this batch.</x:v>
+      </x:c>
+      <x:c r="BA2" t="str">
+        <x:v>Domain-gap evaluation explicitly tests background, object, table and combined shifts; exact failure cases require full-paper appendix extraction.</x:v>
+      </x:c>
+      <x:c r="BB2" t="str">
+        <x:v>OpenAlex Work: https://openalex.org/W? title match was not high-confidence for this title; Citation Count remains Unknown.</x:v>
+      </x:c>
+      <x:c r="BC2" t="str">
+        <x:v>Official ICLR Downloads/Proceedings; accepted OpenReview PDF; official project page; official EmbodiChain repository; author publication list; current official CCF directory</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" t="str">
@@ -30912,6 +33690,24 @@
       <x:c r="AW3" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY3" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA3" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:v>RSS official proceedings abstract</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" t="str">
@@ -31061,6 +33857,24 @@
       <x:c r="AW4" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY4" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA4" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC4" t="str">
+        <x:v>RSS official proceedings abstract</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" t="str">
@@ -31210,6 +34024,24 @@
       <x:c r="AW5" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY5" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA5" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC5" t="str">
+        <x:v>RSS official proceedings</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" t="str">
@@ -31359,6 +34191,24 @@
       <x:c r="AW6" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY6" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA6" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC6" t="str">
+        <x:v>RSS official proceedings abstract</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" t="str">
@@ -31508,6 +34358,24 @@
       <x:c r="AW7" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY7" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA7" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC7" t="str">
+        <x:v>IEEE Xplore abstract; official project page</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" t="str">
@@ -31657,6 +34525,24 @@
       <x:c r="AW8" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY8" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA8" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC8" t="str">
+        <x:v>IEEE Xplore abstract</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" t="str">
@@ -31806,6 +34692,24 @@
       <x:c r="AW9" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY9" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA9" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC9" t="str">
+        <x:v>IEEE Xplore abstract</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" t="str">
@@ -31954,6 +34858,24 @@
       </x:c>
       <x:c r="AW10" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
+      </x:c>
+      <x:c r="AX10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY10" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA10" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC10" t="str">
+        <x:v>IEEE Xplore abstract</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -32082,6 +35004,24 @@
       <x:c r="AW11" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY11" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA11" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" t="str">
@@ -32205,6 +35145,24 @@
       <x:c r="AW12" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY12" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA12" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" t="str">
@@ -32328,6 +35286,24 @@
       <x:c r="AW13" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
+      <x:c r="AX13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY13" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA13" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" t="str">
@@ -32450,6 +35426,24 @@
       </x:c>
       <x:c r="AW14" t="str">
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
+      </x:c>
+      <x:c r="AX14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY14" t="str">
+        <x:v>Unknown / Needs Evidence</x:v>
+      </x:c>
+      <x:c r="AZ14" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BA14" t="str">
+        <x:v>Unknown / Not Explicitly Reported</x:v>
+      </x:c>
+      <x:c r="BB14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BC14" t="str">
+        <x:v>Unknown</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32469,7 +35463,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7fe16fb3c4f419a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8743da78aa834f11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Sync enrichment metadata and progress
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rb78e0de66ebe4bc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R0fa1462e67ef4140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R807b83bc92554f01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R55565df31e6c4a84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R5ca2525dc163414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rce41f18a12ab45ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rbe6574d9f21c4cf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R57908c5da2c148be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R63c2aa156b054ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rad8dabf4aaca4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R88127d74d18b4b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R96875125680b43a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R0bb1bfd8b552455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R2b735d1032b646c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PapersTable" displayName="PapersTable" ref="A1:AZ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="PapersTable" displayName="PapersTable" ref="A1:AZ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="52">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -405,7 +405,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AU79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AU79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="47">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -460,7 +460,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BN67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BN67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="66">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -534,7 +534,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BC14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BC14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="55">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1247,19 +1247,19 @@
         <x:v>Residual Learning / Sim-to-Real</x:v>
       </x:c>
       <x:c r="AU3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AV3" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AW3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AX3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AZ3" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -1373,22 +1373,22 @@
         <x:v>Diffusion / Contact-rich Manipulation</x:v>
       </x:c>
       <x:c r="AU4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AV4" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AW4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AX4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AZ4" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
@@ -1499,19 +1499,19 @@
         <x:v>Human Video / VLM</x:v>
       </x:c>
       <x:c r="AU5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AV5" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AW5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AX5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AZ5" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -4528,7 +4528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8dcb41bb5dcf4040"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f40b01cc37a4f7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7824,7 +7824,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36f63375e94f492f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf782efb0e6bf495e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8175,7 +8175,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09c918cd74c44125"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd847cc0db2e4d6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8921,7 +8921,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R554fa4d754eb4cc4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re26aaa9f1a724d70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9221,19 +9221,19 @@
         <x:v>Robot Manipulation; Diffusion Policy / Hierarchical Control</x:v>
       </x:c>
       <x:c r="AP2" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ2" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR2" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS2" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT2" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -9356,19 +9356,19 @@
         <x:v>bimanual manipulation; decoupled interaction; RoboTwin</x:v>
       </x:c>
       <x:c r="AP3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ3" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -9491,19 +9491,19 @@
         <x:v>bimanual; diffusion; teleoperation; human demonstration</x:v>
       </x:c>
       <x:c r="AP4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ4" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -9628,19 +9628,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ5" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU5" t="str">
         <x:v>Unknown</x:v>
@@ -9763,19 +9763,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ6" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU6" t="str">
         <x:v>Unknown</x:v>
@@ -9898,19 +9898,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ7" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU7" t="str">
         <x:v>Unknown</x:v>
@@ -10031,19 +10031,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ8" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU8" t="str">
         <x:v>Unknown</x:v>
@@ -10166,19 +10166,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ9" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU9" t="str">
         <x:v>Unknown</x:v>
@@ -10299,19 +10299,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ10" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU10" t="str">
         <x:v>Unknown</x:v>
@@ -10436,19 +10436,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ11" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU11" t="str">
         <x:v>Unknown</x:v>
@@ -10573,19 +10573,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ12" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU12" t="str">
         <x:v>Unknown</x:v>
@@ -10710,19 +10710,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ13" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU13" t="str">
         <x:v>Unknown</x:v>
@@ -10845,19 +10845,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ14" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR14" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS14" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU14" t="str">
         <x:v>Unknown</x:v>
@@ -10982,19 +10982,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP15" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ15" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR15" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS15" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT15" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU15" t="str">
         <x:v>Unknown</x:v>
@@ -11115,19 +11115,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP16" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ16" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR16" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS16" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT16" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU16" t="str">
         <x:v>Unknown</x:v>
@@ -11248,19 +11248,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ17" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR17" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS17" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU17" t="str">
         <x:v>Unknown</x:v>
@@ -11381,19 +11381,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP18" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ18" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR18" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS18" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT18" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU18" t="str">
         <x:v>Unknown</x:v>
@@ -11516,19 +11516,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP19" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ19" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR19" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS19" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT19" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU19" t="str">
         <x:v>Unknown</x:v>
@@ -11649,19 +11649,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP20" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ20" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR20" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS20" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT20" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU20" t="str">
         <x:v>Unknown</x:v>
@@ -11784,19 +11784,19 @@
         <x:v>Robot Manipulation; Diffusion Policy / Primitive Skills</x:v>
       </x:c>
       <x:c r="AP21" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ21" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR21" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS21" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT21" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU21" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
@@ -11919,19 +11919,19 @@
         <x:v>Imitation Learning; Multi-Task / Foresight</x:v>
       </x:c>
       <x:c r="AP22" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ22" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR22" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS22" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT22" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU22" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
@@ -12054,19 +12054,19 @@
         <x:v>Robot Manipulation; Long-Horizon / Visual-Tactile Policy</x:v>
       </x:c>
       <x:c r="AP23" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ23" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR23" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS23" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT23" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU23" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
@@ -12189,19 +12189,19 @@
         <x:v>Robot Manipulation; Humanoid / Generalization</x:v>
       </x:c>
       <x:c r="AP24" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ24" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR24" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS24" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT24" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU24" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
@@ -12322,19 +12322,19 @@
         <x:v>Dexterous Manipulation; Human Demonstrations / Motion Prior</x:v>
       </x:c>
       <x:c r="AP25" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ25" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR25" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS25" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT25" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU25" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
@@ -12457,19 +12457,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP26" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ26" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR26" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS26" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT26" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU26" t="str">
         <x:v>Unknown</x:v>
@@ -12592,19 +12592,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP27" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ27" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR27" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS27" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT27" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU27" t="str">
         <x:v>Unknown</x:v>
@@ -12727,22 +12727,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP28" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ28" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR28" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS28" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT28" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU28" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>https://proceedings.mlr.press/v270/</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
@@ -12862,19 +12862,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP29" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ29" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR29" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS29" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT29" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU29" t="str">
         <x:v>Unknown</x:v>
@@ -12997,19 +12997,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP30" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ30" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR30" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS30" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT30" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU30" t="str">
         <x:v>Unknown</x:v>
@@ -13132,19 +13132,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP31" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ31" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR31" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS31" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT31" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU31" t="str">
         <x:v>Unknown</x:v>
@@ -13267,19 +13267,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP32" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ32" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR32" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS32" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT32" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU32" t="str">
         <x:v>Unknown</x:v>
@@ -13402,19 +13402,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP33" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ33" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR33" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS33" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT33" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU33" t="str">
         <x:v>Unknown</x:v>
@@ -13537,19 +13537,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP34" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ34" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR34" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS34" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT34" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU34" t="str">
         <x:v>Unknown</x:v>
@@ -13672,19 +13672,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP35" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ35" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR35" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS35" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT35" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU35" t="str">
         <x:v>Unknown</x:v>
@@ -13807,19 +13807,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP36" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ36" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR36" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS36" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT36" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU36" t="str">
         <x:v>Unknown</x:v>
@@ -13942,19 +13942,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP37" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ37" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR37" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS37" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT37" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU37" t="str">
         <x:v>Unknown</x:v>
@@ -14077,19 +14077,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP38" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ38" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR38" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS38" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT38" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU38" t="str">
         <x:v>Unknown</x:v>
@@ -14212,22 +14212,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP39" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ39" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR39" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS39" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT39" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU39" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>https://proceedings.mlr.press/v270/</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
@@ -14345,19 +14345,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP40" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ40" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR40" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS40" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT40" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU40" t="str">
         <x:v>Unknown</x:v>
@@ -14478,19 +14478,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP41" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ41" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR41" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS41" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT41" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU41" t="str">
         <x:v>Unknown</x:v>
@@ -14611,19 +14611,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP42" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ42" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR42" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS42" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT42" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU42" t="str">
         <x:v>Unknown</x:v>
@@ -14744,19 +14744,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP43" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ43" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR43" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS43" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT43" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU43" t="str">
         <x:v>Unknown</x:v>
@@ -14877,19 +14877,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP44" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ44" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR44" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS44" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT44" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU44" t="str">
         <x:v>Unknown</x:v>
@@ -15010,19 +15010,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP45" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ45" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR45" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS45" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT45" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU45" t="str">
         <x:v>Unknown</x:v>
@@ -15145,19 +15145,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP46" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ46" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR46" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS46" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT46" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU46" t="str">
         <x:v>Unknown</x:v>
@@ -15280,19 +15280,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP47" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ47" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR47" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS47" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT47" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU47" t="str">
         <x:v>Unknown</x:v>
@@ -15415,19 +15415,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP48" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ48" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR48" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS48" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT48" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU48" t="str">
         <x:v>Unknown</x:v>
@@ -15550,19 +15550,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP49" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ49" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR49" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS49" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT49" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU49" t="str">
         <x:v>Unknown</x:v>
@@ -15685,19 +15685,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP50" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ50" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR50" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS50" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT50" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU50" t="str">
         <x:v>Unknown</x:v>
@@ -15820,19 +15820,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP51" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ51" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR51" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS51" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT51" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU51" t="str">
         <x:v>Unknown</x:v>
@@ -15955,19 +15955,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP52" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ52" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR52" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS52" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT52" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU52" t="str">
         <x:v>Unknown</x:v>
@@ -16090,19 +16090,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP53" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ53" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR53" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS53" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT53" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU53" t="str">
         <x:v>Unknown</x:v>
@@ -16225,19 +16225,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP54" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ54" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR54" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS54" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT54" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU54" t="str">
         <x:v>Unknown</x:v>
@@ -16360,19 +16360,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP55" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ55" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR55" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS55" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT55" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU55" t="str">
         <x:v>Unknown</x:v>
@@ -16495,19 +16495,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP56" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ56" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR56" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS56" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT56" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU56" t="str">
         <x:v>Unknown</x:v>
@@ -16630,19 +16630,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP57" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ57" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR57" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS57" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT57" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU57" t="str">
         <x:v>Unknown</x:v>
@@ -16771,19 +16771,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP58" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ58" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR58" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS58" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT58" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU58" t="str">
         <x:v>Unknown</x:v>
@@ -16912,19 +16912,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP59" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ59" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR59" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS59" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT59" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU59" t="str">
         <x:v>Unknown</x:v>
@@ -17051,19 +17051,19 @@
         <x:v>Bimanual; Benchmark / Synthetic Demonstrations</x:v>
       </x:c>
       <x:c r="AP60" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ60" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR60" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS60" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT60" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU60" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -17192,19 +17192,19 @@
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
       <x:c r="AP61" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ61" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR61" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS61" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT61" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU61" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -17333,19 +17333,19 @@
         <x:v>VLA; Inference Acceleration / Token Caching</x:v>
       </x:c>
       <x:c r="AP62" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ62" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR62" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS62" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT62" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -17474,19 +17474,19 @@
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
       <x:c r="AP63" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ63" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR63" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS63" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT63" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU63" t="str">
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
@@ -17756,22 +17756,22 @@
         <x:v>VLA; Efficient Model / Pose Prediction</x:v>
       </x:c>
       <x:c r="AP65" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ65" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR65" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS65" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT65" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU65" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
@@ -17897,19 +17897,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP66" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ66" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR66" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS66" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT66" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU66" t="str">
         <x:v>Unknown</x:v>
@@ -18038,19 +18038,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP67" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ67" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR67" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS67" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT67" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU67" t="str">
         <x:v>Unknown</x:v>
@@ -18177,22 +18177,22 @@
         <x:v>Robot Manipulation; Consistency Flow Matching / 3D Policy</x:v>
       </x:c>
       <x:c r="AP68" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ68" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR68" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS68" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT68" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU68" t="str">
-        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617；官方摘要/论文集元数据</x:v>
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
@@ -18318,19 +18318,19 @@
         <x:v>Dexterous Hand; Policy Distillation / Generalization</x:v>
       </x:c>
       <x:c r="AP69" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ69" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR69" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS69" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT69" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU69" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -18459,19 +18459,19 @@
         <x:v>Dexterous Hand; Residual RL / VLM Planning</x:v>
       </x:c>
       <x:c r="AP70" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ70" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR70" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS70" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT70" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU70" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -18600,19 +18600,19 @@
         <x:v>VLA; Video-Action Model / Generalization</x:v>
       </x:c>
       <x:c r="AP71" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ71" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR71" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS71" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT71" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU71" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -18741,19 +18741,19 @@
         <x:v>Dexterous Hand; Contact Reasoning / Language-guided Grasp</x:v>
       </x:c>
       <x:c r="AP72" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ72" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR72" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS72" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT72" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU72" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -18882,19 +18882,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP73" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ73" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR73" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS73" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT73" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU73" t="str">
         <x:v>Unknown</x:v>
@@ -19023,19 +19023,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP74" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ74" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR74" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS74" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT74" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU74" t="str">
         <x:v>Unknown</x:v>
@@ -19164,19 +19164,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP75" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ75" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR75" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS75" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT75" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU75" t="str">
         <x:v>Unknown</x:v>
@@ -19301,19 +19301,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP76" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ76" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR76" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS76" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT76" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU76" t="str">
         <x:v>Unknown</x:v>
@@ -19438,19 +19438,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP77" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ77" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR77" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS77" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT77" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU77" t="str">
         <x:v>Unknown</x:v>
@@ -19575,19 +19575,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP78" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AQ78" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AR78" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AS78" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT78" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU78" t="str">
         <x:v>Unknown</x:v>
@@ -19756,7 +19756,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf300a6bb39a34b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a2910e42e24495"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20191,19 +20191,19 @@
         <x:v>Robot Manipulation; Diffusion Policy / Hierarchical Control</x:v>
       </x:c>
       <x:c r="BI2" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ2" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK2" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL2" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM2" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -20383,19 +20383,19 @@
         <x:v>bimanual manipulation; decoupled interaction; RoboTwin</x:v>
       </x:c>
       <x:c r="BI3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ3" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -20575,19 +20575,19 @@
         <x:v>bimanual; diffusion; teleoperation; human demonstration</x:v>
       </x:c>
       <x:c r="BI4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ4" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -20767,19 +20767,19 @@
         <x:v>Robot Manipulation; Diffusion Policy / Primitive Skills</x:v>
       </x:c>
       <x:c r="BI5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ5" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN5" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
@@ -20959,19 +20959,19 @@
         <x:v>Imitation Learning; Multi-Task / Foresight</x:v>
       </x:c>
       <x:c r="BI6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ6" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN6" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
@@ -21151,19 +21151,19 @@
         <x:v>Robot Manipulation; Long-Horizon / Visual-Tactile Policy</x:v>
       </x:c>
       <x:c r="BI7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ7" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN7" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
@@ -21343,19 +21343,19 @@
         <x:v>Robot Manipulation; Humanoid / Generalization</x:v>
       </x:c>
       <x:c r="BI8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ8" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN8" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
@@ -21533,19 +21533,19 @@
         <x:v>Dexterous Manipulation; Human Demonstrations / Motion Prior</x:v>
       </x:c>
       <x:c r="BI9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ9" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN9" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
@@ -21729,19 +21729,19 @@
         <x:v>Bimanual; Benchmark / Synthetic Demonstrations</x:v>
       </x:c>
       <x:c r="BI10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ10" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN10" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -21927,19 +21927,19 @@
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
       <x:c r="BI11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ11" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN11" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -22125,19 +22125,19 @@
         <x:v>VLA; Inference Acceleration / Token Caching</x:v>
       </x:c>
       <x:c r="BI12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ12" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN12" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -22323,19 +22323,19 @@
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
       <x:c r="BI13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ13" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN13" t="str">
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
@@ -22719,22 +22719,22 @@
         <x:v>VLA; Efficient Model / Pose Prediction</x:v>
       </x:c>
       <x:c r="BI15" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ15" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK15" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL15" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM15" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN15" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -22915,22 +22915,22 @@
         <x:v>Robot Manipulation; Consistency Flow Matching / 3D Policy</x:v>
       </x:c>
       <x:c r="BI16" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ16" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK16" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL16" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM16" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN16" t="str">
-        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617；官方摘要/论文集元数据</x:v>
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
@@ -23113,19 +23113,19 @@
         <x:v>Dexterous Hand; Policy Distillation / Generalization</x:v>
       </x:c>
       <x:c r="BI17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ17" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK17" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL17" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN17" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -23311,19 +23311,19 @@
         <x:v>Dexterous Hand; Residual RL / VLM Planning</x:v>
       </x:c>
       <x:c r="BI18" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ18" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK18" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL18" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM18" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN18" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -23509,19 +23509,19 @@
         <x:v>VLA; Video-Action Model / Generalization</x:v>
       </x:c>
       <x:c r="BI19" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ19" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK19" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL19" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM19" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN19" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -23707,19 +23707,19 @@
         <x:v>Dexterous Hand; Contact Reasoning / Language-guided Grasp</x:v>
       </x:c>
       <x:c r="BI20" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ20" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK20" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL20" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM20" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN20" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -24107,19 +24107,19 @@
         <x:v>Residual Learning / Sim-to-Real</x:v>
       </x:c>
       <x:c r="BI22" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ22" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK22" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL22" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM22" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN22" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -24307,22 +24307,22 @@
         <x:v>Diffusion / Contact-rich Manipulation</x:v>
       </x:c>
       <x:c r="BI23" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ23" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK23" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL23" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM23" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN23" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
@@ -24507,19 +24507,19 @@
         <x:v>Human Video / VLM</x:v>
       </x:c>
       <x:c r="BI24" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ24" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK24" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL24" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM24" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN24" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -24707,19 +24707,19 @@
         <x:v>Dexterous Grasping</x:v>
       </x:c>
       <x:c r="BI25" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ25" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK25" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL25" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM25" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN25" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Xu_Dexterous_Grasp_Transformer_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -24907,19 +24907,19 @@
         <x:v>Mobile Manipulation</x:v>
       </x:c>
       <x:c r="BI26" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ26" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK26" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL26" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM26" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN26" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wu_MoManipVLA_Transferring_Vision-language-action_Models_for_General_Mobile_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -25107,19 +25107,19 @@
         <x:v>Action Chunking / Multi-task Policy</x:v>
       </x:c>
       <x:c r="BI27" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ27" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK27" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL27" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM27" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN27" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/ff887781480973bd3cb6026feb378d1e-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -25307,19 +25307,19 @@
         <x:v>Surgical Robotics</x:v>
       </x:c>
       <x:c r="BI28" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ28" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK28" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL28" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM28" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN28" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/74c4f2b87b7499d365422152c76fd916-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -25507,19 +25507,19 @@
         <x:v>Video Demonstration / Reward Learning</x:v>
       </x:c>
       <x:c r="BI29" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ29" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK29" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL29" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM29" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN29" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/dcd297696d0bb304ba426b3c5a679c37-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -25707,19 +25707,19 @@
         <x:v>Long-Horizon / Failure Recovery</x:v>
       </x:c>
       <x:c r="BI30" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ30" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK30" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL30" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM30" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN30" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/fad8962279154544ed69bb63eb14d677-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -25907,19 +25907,19 @@
         <x:v>3D Observation / Contact-rich</x:v>
       </x:c>
       <x:c r="BI31" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ31" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK31" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL31" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM31" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN31" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/8e5dc5969a6174fcaaececd890c7f59b-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -26107,19 +26107,19 @@
         <x:v>Text-conditioned Reward</x:v>
       </x:c>
       <x:c r="BI32" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ32" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK32" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL32" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM32" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN32" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/5227ce00add5aa0a12d1c4ee92fcd2dc-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -26307,22 +26307,22 @@
         <x:v>Human-Robot Domain Adaptation</x:v>
       </x:c>
       <x:c r="BI33" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ33" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK33" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL33" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM33" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN33" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhou_Mitigating_the_Human-Robot_Domain_Discrepancy_in_Visual_Pre-training_for_Robotic_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
@@ -26507,19 +26507,19 @@
         <x:v>Grounding / Synthetic Data</x:v>
       </x:c>
       <x:c r="BI34" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ34" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK34" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL34" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM34" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN34" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Huang_RoboGround_Robotic_Manipulation_with_Grounded_Vision-Language_Priors_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -26707,19 +26707,19 @@
         <x:v>Synthetic Data / Scene Generation</x:v>
       </x:c>
       <x:c r="BI35" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ35" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK35" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL35" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM35" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN35" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -26907,19 +26907,19 @@
         <x:v>Lifelong Learning</x:v>
       </x:c>
       <x:c r="BI36" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ36" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK36" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL36" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM36" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN36" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Yao_Think_Small_Act_Big_Primitive_Prompt_Learning_for_Lifelong_Robot_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -27107,19 +27107,19 @@
         <x:v>Failure Recovery / 3D Gaussian Splatting</x:v>
       </x:c>
       <x:c r="BI37" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ37" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK37" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL37" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM37" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN37" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/34866；官方摘要/论文集元数据</x:v>
@@ -27307,19 +27307,19 @@
         <x:v>Articulated Object / Affordance</x:v>
       </x:c>
       <x:c r="BI38" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ38" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK38" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL38" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM38" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN38" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33615；官方摘要/论文集元数据</x:v>
@@ -27507,19 +27507,19 @@
         <x:v>Long-Horizon / Mobile Manipulation</x:v>
       </x:c>
       <x:c r="BI39" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ39" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK39" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL39" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM39" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN39" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33610；官方摘要/论文集元数据</x:v>
@@ -27707,19 +27707,19 @@
         <x:v>World Model / Video Diffusion</x:v>
       </x:c>
       <x:c r="BI40" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ40" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK40" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL40" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM40" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN40" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/481c70828a4ff20d31a646cc6cc95f3d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -27907,22 +27907,22 @@
         <x:v>Human Video / 3D Affordance</x:v>
       </x:c>
       <x:c r="BI41" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ41" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK41" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL41" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM41" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN41" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generalizable_3D_Actions_from_In-the-Wild_2D_Human_Videos_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generali</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
@@ -28107,22 +28107,22 @@
         <x:v>Visual Chain-of-Thought</x:v>
       </x:c>
       <x:c r="BI42" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ42" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK42" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL42" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM42" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN42" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhao_CoT-VLA_Visual_Chain-of-Thought_Reasoning_for_Vision-Language-Action_Models_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
@@ -28307,19 +28307,19 @@
         <x:v>Sim-to-Real / Behavior Cloning</x:v>
       </x:c>
       <x:c r="BI43" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ43" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK43" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL43" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM43" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN43" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1185c89347a3f21ffc48c9d083c9437c-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -28507,19 +28507,19 @@
         <x:v>Long-Horizon / Planning</x:v>
       </x:c>
       <x:c r="BI44" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ44" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK44" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL44" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM44" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN44" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b94310e1c7ecb79f1a24adc757f1b89b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -28707,19 +28707,19 @@
         <x:v>Stochastic Interpolant / Efficiency</x:v>
       </x:c>
       <x:c r="BI45" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ45" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK45" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL45" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM45" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN45" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/49eadcc4a329fc6b74b9f8a82b78cbc3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -28907,19 +28907,19 @@
         <x:v>Mobile Manipulation / Agent</x:v>
       </x:c>
       <x:c r="BI46" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ46" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK46" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL46" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM46" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN46" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/bc97207e3979d1cc23109db0be0e8ed2-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -29107,19 +29107,19 @@
         <x:v>Flow Matching / Visuomotor Policy</x:v>
       </x:c>
       <x:c r="BI47" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ47" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK47" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL47" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM47" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN47" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/282c3318be1b047b7bb5ba94fa4f3231-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -29307,19 +29307,19 @@
         <x:v>Tool Use / Generative Design</x:v>
       </x:c>
       <x:c r="BI48" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ48" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK48" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL48" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM48" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN48" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/9fc291fef2f9607a46777d367f900a15-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -29507,19 +29507,19 @@
         <x:v>3D Manipulation / Multimodal Policy</x:v>
       </x:c>
       <x:c r="BI49" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ49" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK49" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL49" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM49" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN49" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/eacc8ae341d15d2c13c02fef88189db3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -29707,19 +29707,19 @@
         <x:v>Robot Data / Spatial Reasoning</x:v>
       </x:c>
       <x:c r="BI50" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ50" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK50" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL50" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM50" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN50" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1f467c3e37abf9f86c78f44c6a27ee7c-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -29907,19 +29907,19 @@
         <x:v>Task Planning / Demonstrations</x:v>
       </x:c>
       <x:c r="BI51" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ51" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK51" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL51" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM51" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN51" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b8358a00e5b870194b974ddf8dd415c3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -30107,19 +30107,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI52" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ52" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK52" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL52" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM52" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN52" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Wang_DexH2R_A_Benchmark_for_Dynamic_Dexterous_Grasping_in_Human-to-Robot_Handover_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -30307,22 +30307,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI53" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ53" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK53" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL53" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM53" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN53" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhang_BimArt_A_Unified_Approach_for_the_Synthesis_of_3D_Bimanual_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
@@ -30707,22 +30707,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI55" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ55" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK55" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL55" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM55" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN55" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generalizable_Hand_Object_Motion_Generation_with_Latent_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generali</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
@@ -30907,22 +30907,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI56" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ56" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK56" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL56" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM56" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN56" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generalizable_Bimanual_Tool-ACtion-Object_Understanding_CVPR_2024_paper.pdf；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generali</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
@@ -31107,19 +31107,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI57" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ57" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK57" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL57" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM57" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN57" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Uppal_SPIN_Simultaneous_Perception_Interaction_and_Navigation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -31707,22 +31707,22 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI60" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ60" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK60" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL60" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM60" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN60" t="str">
-        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Zhao_TASTE-Rob_Advancing_Video_Generation_of_Task-Oriented_Hand-Object_Interaction_for_Generalizable_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
+        <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
@@ -31907,19 +31907,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI61" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ61" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK61" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL61" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM61" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN61" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38874；官方摘要/论文集元数据</x:v>
@@ -32107,19 +32107,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI62" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ62" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK62" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL62" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM62" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/e4ef7454447baa15a424314e6284441b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -32307,19 +32307,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI63" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ63" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK63" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL63" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM63" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN63" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38313；官方摘要/论文集元数据</x:v>
@@ -32507,19 +32507,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI64" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ64" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK64" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL64" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM64" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN64" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/40127；官方摘要/论文集元数据</x:v>
@@ -32707,19 +32707,19 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BI65" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="BJ65" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="BK65" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BL65" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM65" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BN65" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28266；官方摘要/论文集元数据</x:v>
@@ -33160,7 +33160,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc302613323ef40fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d151f50ba90484f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33691,22 +33691,22 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY3" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA3" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB3" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC3" t="str">
-        <x:v>RSS official proceedings abstract</x:v>
+        <x:v>https://www.roboticsproceedings.org/rss21/p149.html; https://hnu</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
@@ -33858,19 +33858,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY4" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA4" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB4" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC4" t="str">
         <x:v>RSS official proceedings abstract</x:v>
@@ -34025,19 +34025,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY5" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA5" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB5" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC5" t="str">
         <x:v>RSS official proceedings</x:v>
@@ -34192,19 +34192,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY6" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA6" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB6" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC6" t="str">
         <x:v>RSS official proceedings abstract</x:v>
@@ -34359,19 +34359,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY7" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA7" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB7" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC7" t="str">
         <x:v>IEEE Xplore abstract; official project page</x:v>
@@ -34526,19 +34526,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY8" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA8" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB8" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC8" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -34693,19 +34693,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY9" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA9" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB9" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC9" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -34860,19 +34860,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY10" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA10" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB10" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC10" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -35005,19 +35005,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY11" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA11" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB11" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC11" t="str">
         <x:v>Unknown</x:v>
@@ -35146,19 +35146,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY12" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA12" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB12" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC12" t="str">
         <x:v>Unknown</x:v>
@@ -35287,19 +35287,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY13" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA13" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB13" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC13" t="str">
         <x:v>Unknown</x:v>
@@ -35428,19 +35428,19 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="AY14" t="str">
-        <x:v>Unknown / Needs Evidence</x:v>
+        <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
       </x:c>
       <x:c r="AZ14" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BA14" t="str">
-        <x:v>Unknown / Not Explicitly Reported</x:v>
+        <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB14" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC14" t="str">
         <x:v>Unknown</x:v>
@@ -35463,7 +35463,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8743da78aa834f11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd07c215f6a644228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Sync evidence upgrade statuses
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R57908c5da2c148be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R63c2aa156b054ec2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rad8dabf4aaca4b71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R88127d74d18b4b30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R96875125680b43a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R0bb1bfd8b552455d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R2b735d1032b646c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rd4ae01dd80cd4d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R045ebd6a5fb24004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R255adb3d1f524f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rd38c8746b1a14fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rf744afbc81b541c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rf53b9c3f8f264abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R34449d90d2e84a8a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="PapersTable" displayName="PapersTable" ref="A1:AZ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="52">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="PapersTable" displayName="PapersTable" ref="A1:BD5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="56">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -354,6 +354,10 @@
     <x:tableColumn id="50" name="Failure Cases"/>
     <x:tableColumn id="51" name="Citation Source Identifier"/>
     <x:tableColumn id="52" name="Evidence Sources"/>
+    <x:tableColumn id="53" name="Evidence Upgrade Status"/>
+    <x:tableColumn id="54" name="Supplement Status"/>
+    <x:tableColumn id="55" name="Code Completeness"/>
+    <x:tableColumn id="56" name="Robot Platform Evidence"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -405,8 +409,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AU79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="47">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:AY79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="51">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -454,14 +458,18 @@
     <x:tableColumn id="45" name="Failure Cases"/>
     <x:tableColumn id="46" name="Citation Source Identifier"/>
     <x:tableColumn id="47" name="Evidence Sources"/>
+    <x:tableColumn id="48" name="Evidence Upgrade Status"/>
+    <x:tableColumn id="49" name="Supplement Status"/>
+    <x:tableColumn id="50" name="Code Completeness"/>
+    <x:tableColumn id="51" name="Robot Platform Evidence"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BN67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="66">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="26" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:BR67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="70">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="作者 Authors"/>
@@ -528,14 +536,18 @@
     <x:tableColumn id="64" name="Failure Cases"/>
     <x:tableColumn id="65" name="Citation Source Identifier"/>
     <x:tableColumn id="66" name="Evidence Sources"/>
+    <x:tableColumn id="67" name="Evidence Upgrade Status"/>
+    <x:tableColumn id="68" name="Supplement Status"/>
+    <x:tableColumn id="69" name="Code Completeness"/>
+    <x:tableColumn id="70" name="Robot Platform Evidence"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BC14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="55">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="27" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BG14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="59">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
     <x:tableColumn id="3" name="Authors"/>
@@ -591,6 +603,10 @@
     <x:tableColumn id="53" name="Failure Cases"/>
     <x:tableColumn id="54" name="Citation Source Identifier"/>
     <x:tableColumn id="55" name="Evidence Sources"/>
+    <x:tableColumn id="56" name="Evidence Upgrade Status"/>
+    <x:tableColumn id="57" name="Supplement Status"/>
+    <x:tableColumn id="58" name="Code Completeness"/>
+    <x:tableColumn id="59" name="Robot Platform Evidence"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -981,6 +997,18 @@
       <x:c r="AZ1" t="str">
         <x:v>Evidence Sources</x:v>
       </x:c>
+      <x:c r="BA1" t="str">
+        <x:v>Evidence Upgrade Status</x:v>
+      </x:c>
+      <x:c r="BB1" t="str">
+        <x:v>Supplement Status</x:v>
+      </x:c>
+      <x:c r="BC1" t="str">
+        <x:v>Code Completeness</x:v>
+      </x:c>
+      <x:c r="BD1" t="str">
+        <x:v>Robot Platform Evidence</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="350" customHeight="1">
       <x:c r="A2" t="str">
@@ -1137,6 +1165,18 @@
       </x:c>
       <x:c r="AZ2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
+      <x:c r="BA2" t="str">
+        <x:v>A-Upgraded</x:v>
+      </x:c>
+      <x:c r="BB2" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BC2" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BD2" t="str">
+        <x:v>Unknown</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="150" customHeight="1">
@@ -1264,6 +1304,18 @@
       <x:c r="AZ3" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BA3" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BB3" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BC3" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BD3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" t="str">
@@ -1390,6 +1442,18 @@
       <x:c r="AZ4" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
       </x:c>
+      <x:c r="BA4" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BB4" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BC4" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BD4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
       <x:c r="A5" t="str">
@@ -1515,6 +1579,18 @@
       </x:c>
       <x:c r="AZ5" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
+      </x:c>
+      <x:c r="BA5" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BB5" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BC5" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BD5" t="str">
+        <x:v>Unknown</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4528,7 +4604,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f40b01cc37a4f7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb6b3e8902a14813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7824,7 +7900,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf782efb0e6bf495e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0c56d1d9f95448a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8175,7 +8251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd847cc0db2e4d6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9556a8be6dfd4281"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8921,7 +8997,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re26aaa9f1a724d70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8cc26495f454170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9103,6 +9179,18 @@
       <x:c r="AU1" t="str">
         <x:v>Evidence Sources</x:v>
       </x:c>
+      <x:c r="AV1" t="str">
+        <x:v>Evidence Upgrade Status</x:v>
+      </x:c>
+      <x:c r="AW1" t="str">
+        <x:v>Supplement Status</x:v>
+      </x:c>
+      <x:c r="AX1" t="str">
+        <x:v>Code Completeness</x:v>
+      </x:c>
+      <x:c r="AY1" t="str">
+        <x:v>Robot Platform Evidence</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -9238,6 +9326,18 @@
       <x:c r="AU2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV2" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW2" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -9373,6 +9473,18 @@
       <x:c r="AU3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV3" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW3" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -9508,6 +9620,18 @@
       <x:c r="AU4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV4" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW4" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -9645,6 +9769,18 @@
       <x:c r="AU5" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV5" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW5" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -9780,6 +9916,18 @@
       <x:c r="AU6" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV6" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW6" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -9915,6 +10063,18 @@
       <x:c r="AU7" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV7" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW7" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -10048,6 +10208,18 @@
       <x:c r="AU8" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV8" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW8" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -10183,6 +10355,18 @@
       <x:c r="AU9" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV9" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW9" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -10316,6 +10500,18 @@
       <x:c r="AU10" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV10" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW10" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -10453,6 +10649,18 @@
       <x:c r="AU11" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV11" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW11" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -10588,6 +10796,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV12" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW12" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -10727,6 +10947,18 @@
       <x:c r="AU13" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV13" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW13" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX13" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -10862,6 +11094,18 @@
       <x:c r="AU14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV14" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW14" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -10997,6 +11241,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV15" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW15" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX15" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY15" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -11132,6 +11388,18 @@
       <x:c r="AU16" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV16" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW16" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -11265,6 +11533,18 @@
       <x:c r="AU17" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV17" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW17" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -11398,6 +11678,18 @@
       <x:c r="AU18" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV18" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW18" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -11533,6 +11825,18 @@
       <x:c r="AU19" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV19" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW19" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -11666,6 +11970,18 @@
       <x:c r="AU20" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV20" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW20" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -11801,6 +12117,18 @@
       <x:c r="AU21" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV21" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW21" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX21" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY21" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -11936,6 +12264,18 @@
       <x:c r="AU22" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV22" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW22" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -12071,6 +12411,18 @@
       <x:c r="AU23" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV23" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW23" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -12206,6 +12558,18 @@
       <x:c r="AU24" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV24" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW24" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -12339,6 +12703,18 @@
       <x:c r="AU25" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV25" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW25" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -12474,6 +12850,18 @@
       <x:c r="AU26" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV26" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW26" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -12609,6 +12997,18 @@
       <x:c r="AU27" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV27" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW27" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -12744,6 +13144,18 @@
       <x:c r="AU28" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
       </x:c>
+      <x:c r="AV28" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW28" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -12879,6 +13291,18 @@
       <x:c r="AU29" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV29" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW29" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -13014,6 +13438,18 @@
       <x:c r="AU30" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV30" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW30" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -13149,6 +13585,18 @@
       <x:c r="AU31" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV31" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW31" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -13284,6 +13732,18 @@
       <x:c r="AU32" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV32" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW32" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -13419,6 +13879,18 @@
       <x:c r="AU33" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV33" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW33" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -13554,6 +14026,18 @@
       <x:c r="AU34" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV34" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW34" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -13689,6 +14173,18 @@
       <x:c r="AU35" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV35" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW35" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -13824,6 +14320,18 @@
       <x:c r="AU36" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV36" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW36" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -13959,6 +14467,18 @@
       <x:c r="AU37" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV37" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW37" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -14094,6 +14614,18 @@
       <x:c r="AU38" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV38" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW38" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -14229,6 +14761,18 @@
       <x:c r="AU39" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
       </x:c>
+      <x:c r="AV39" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW39" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -14362,6 +14906,18 @@
       <x:c r="AU40" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV40" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW40" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -14495,6 +15051,18 @@
       <x:c r="AU41" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV41" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW41" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -14628,6 +15196,18 @@
       <x:c r="AU42" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV42" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW42" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -14761,6 +15341,18 @@
       <x:c r="AU43" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV43" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW43" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -14894,6 +15486,18 @@
       <x:c r="AU44" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV44" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW44" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -15027,6 +15631,18 @@
       <x:c r="AU45" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV45" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW45" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -15162,6 +15778,18 @@
       <x:c r="AU46" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV46" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW46" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -15297,6 +15925,18 @@
       <x:c r="AU47" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV47" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW47" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -15432,6 +16072,18 @@
       <x:c r="AU48" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV48" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW48" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -15567,6 +16219,18 @@
       <x:c r="AU49" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV49" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW49" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -15702,6 +16366,18 @@
       <x:c r="AU50" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV50" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW50" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -15837,6 +16513,18 @@
       <x:c r="AU51" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV51" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW51" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -15972,6 +16660,18 @@
       <x:c r="AU52" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV52" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW52" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -16107,6 +16807,18 @@
       <x:c r="AU53" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV53" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW53" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -16242,6 +16954,18 @@
       <x:c r="AU54" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV54" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW54" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -16377,6 +17101,18 @@
       <x:c r="AU55" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV55" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW55" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -16512,6 +17248,18 @@
       <x:c r="AU56" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV56" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW56" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -16647,6 +17395,18 @@
       <x:c r="AU57" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV57" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW57" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -16788,6 +17548,18 @@
       <x:c r="AU58" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV58" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW58" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX58" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY58" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -16929,6 +17701,18 @@
       <x:c r="AU59" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV59" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW59" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX59" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY59" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -17068,6 +17852,18 @@
       <x:c r="AU60" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV60" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW60" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX60" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -17209,6 +18005,18 @@
       <x:c r="AU61" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV61" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW61" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX61" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -17350,6 +18158,18 @@
       <x:c r="AU62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV62" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW62" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX62" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -17491,6 +18311,18 @@
       <x:c r="AU63" t="str">
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV63" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW63" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX63" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="AY63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -17632,6 +18464,18 @@
       <x:c r="AU64" t="str">
         <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV64" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW64" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX64" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="AY64" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -17773,6 +18617,18 @@
       <x:c r="AU65" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
       </x:c>
+      <x:c r="AV65" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW65" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX65" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="AY65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -17914,6 +18770,18 @@
       <x:c r="AU66" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV66" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW66" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX66" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="AY66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="58" customHeight="1">
       <x:c r="A67" t="str">
@@ -18053,6 +18921,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU67" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV67" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW67" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX67" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY67" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -18194,6 +19074,18 @@
       <x:c r="AU68" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
       </x:c>
+      <x:c r="AV68" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW68" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX68" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY68" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
       <x:c r="A69" t="str">
@@ -18335,6 +19227,18 @@
       <x:c r="AU69" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV69" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW69" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX69" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY69" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" t="str">
@@ -18476,6 +19380,18 @@
       <x:c r="AU70" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV70" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW70" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX70" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY70" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" t="str">
@@ -18617,6 +19533,18 @@
       <x:c r="AU71" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV71" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW71" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX71" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="AY71" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="58" customHeight="1">
       <x:c r="A72" t="str">
@@ -18758,6 +19686,18 @@
       <x:c r="AU72" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="AV72" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW72" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX72" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY72" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="58" customHeight="1">
       <x:c r="A73" t="str">
@@ -18899,6 +19839,18 @@
       <x:c r="AU73" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV73" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW73" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX73" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY73" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="58" customHeight="1">
       <x:c r="A74" t="str">
@@ -19040,6 +19992,18 @@
       <x:c r="AU74" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV74" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW74" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX74" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY74" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="75" ht="58" customHeight="1">
       <x:c r="A75" t="str">
@@ -19179,6 +20143,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV75" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW75" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX75" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -19318,6 +20294,18 @@
       <x:c r="AU76" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV76" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW76" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX76" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY76" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="58" customHeight="1">
       <x:c r="A77" t="str">
@@ -19453,6 +20441,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="AU77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AV77" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW77" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX77" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="AY77" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -19592,6 +20592,18 @@
       <x:c r="AU78" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="AV78" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="AW78" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX78" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY78" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -19734,6 +20746,18 @@
       </x:c>
       <x:c r="AU79" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
+      </x:c>
+      <x:c r="AV79" t="str">
+        <x:v>B-Experiment-Not-Extracted</x:v>
+      </x:c>
+      <x:c r="AW79" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="AX79" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="AY79" t="str">
+        <x:v>Franka Panda (CALVIN simulation); real-world platform not confirmed at abstract level</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -19756,7 +20780,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37a2910e42e24495"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fc4c099267640c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20016,6 +21040,18 @@
       <x:c r="BN1" t="str">
         <x:v>Evidence Sources</x:v>
       </x:c>
+      <x:c r="BO1" t="str">
+        <x:v>Evidence Upgrade Status</x:v>
+      </x:c>
+      <x:c r="BP1" t="str">
+        <x:v>Supplement Status</x:v>
+      </x:c>
+      <x:c r="BQ1" t="str">
+        <x:v>Code Completeness</x:v>
+      </x:c>
+      <x:c r="BR1" t="str">
+        <x:v>Robot Platform Evidence</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -20208,6 +21244,18 @@
       <x:c r="BN2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO2" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP2" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR2" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -20400,6 +21448,18 @@
       <x:c r="BN3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO3" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP3" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR3" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -20592,6 +21652,18 @@
       <x:c r="BN4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO4" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP4" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR4" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -20784,6 +21856,18 @@
       <x:c r="BN5" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO5" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP5" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR5" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -20976,6 +22060,18 @@
       <x:c r="BN6" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO6" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP6" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR6" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -21168,6 +22264,18 @@
       <x:c r="BN7" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO7" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP7" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR7" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -21360,6 +22468,18 @@
       <x:c r="BN8" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO8" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP8" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR8" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -21550,6 +22670,18 @@
       <x:c r="BN9" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO9" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP9" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR9" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -21746,6 +22878,18 @@
       <x:c r="BN10" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO10" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP10" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ10" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR10" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -21944,6 +23088,18 @@
       <x:c r="BN11" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO11" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP11" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ11" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -22142,6 +23298,18 @@
       <x:c r="BN12" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO12" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP12" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ12" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -22340,6 +23508,18 @@
       <x:c r="BN13" t="str">
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO13" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP13" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ13" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -22538,6 +23718,18 @@
       <x:c r="BN14" t="str">
         <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO14" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP14" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ14" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -22735,6 +23927,18 @@
       </x:c>
       <x:c r="BN15" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
+      </x:c>
+      <x:c r="BO15" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP15" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR15" t="str">
+        <x:v>Unknown</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -22932,6 +24136,18 @@
       <x:c r="BN16" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
       </x:c>
+      <x:c r="BO16" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP16" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ16" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR16" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -23130,6 +24346,18 @@
       <x:c r="BN17" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO17" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP17" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ17" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR17" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -23328,6 +24556,18 @@
       <x:c r="BN18" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO18" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP18" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ18" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR18" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -23526,6 +24766,18 @@
       <x:c r="BN19" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO19" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP19" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ19" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR19" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -23724,6 +24976,18 @@
       <x:c r="BN20" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO20" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP20" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ20" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR20" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -23924,6 +25188,18 @@
       <x:c r="BN21" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO21" t="str">
+        <x:v>A-Upgraded</x:v>
+      </x:c>
+      <x:c r="BP21" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ21" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR21" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -24124,6 +25400,18 @@
       <x:c r="BN22" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO22" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP22" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ22" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR22" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -24324,6 +25612,18 @@
       <x:c r="BN23" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
       </x:c>
+      <x:c r="BO23" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP23" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ23" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BR23" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -24524,6 +25824,18 @@
       <x:c r="BN24" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO24" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP24" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ24" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR24" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -24724,6 +26036,18 @@
       <x:c r="BN25" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Xu_Dexterous_Grasp_Transformer_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO25" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP25" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ25" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR25" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -24924,6 +26248,18 @@
       <x:c r="BN26" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wu_MoManipVLA_Transferring_Vision-language-action_Models_for_General_Mobile_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO26" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP26" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ26" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR26" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -25124,6 +26460,18 @@
       <x:c r="BN27" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/ff887781480973bd3cb6026feb378d1e-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO27" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP27" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ27" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR27" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -25324,6 +26672,18 @@
       <x:c r="BN28" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/74c4f2b87b7499d365422152c76fd916-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO28" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP28" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ28" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR28" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -25524,6 +26884,18 @@
       <x:c r="BN29" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/dcd297696d0bb304ba426b3c5a679c37-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO29" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP29" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ29" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR29" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -25724,6 +27096,18 @@
       <x:c r="BN30" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/fad8962279154544ed69bb63eb14d677-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO30" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP30" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ30" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR30" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -25924,6 +27308,18 @@
       <x:c r="BN31" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/8e5dc5969a6174fcaaececd890c7f59b-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO31" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP31" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ31" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR31" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -26124,6 +27520,18 @@
       <x:c r="BN32" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/5227ce00add5aa0a12d1c4ee92fcd2dc-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO32" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP32" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ32" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR32" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -26324,6 +27732,18 @@
       <x:c r="BN33" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
+      <x:c r="BO33" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP33" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ33" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -26524,6 +27944,18 @@
       <x:c r="BN34" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Huang_RoboGround_Robotic_Manipulation_with_Grounded_Vision-Language_Priors_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO34" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP34" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ34" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR34" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -26724,6 +28156,18 @@
       <x:c r="BN35" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO35" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP35" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ35" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR35" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -26924,6 +28368,18 @@
       <x:c r="BN36" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Yao_Think_Small_Act_Big_Primitive_Prompt_Learning_for_Lifelong_Robot_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO36" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP36" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ36" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR36" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -27124,6 +28580,18 @@
       <x:c r="BN37" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/34866；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO37" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP37" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ37" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR37" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -27324,6 +28792,18 @@
       <x:c r="BN38" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33615；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO38" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP38" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ38" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR38" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -27524,6 +29004,18 @@
       <x:c r="BN39" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33610；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO39" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP39" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ39" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR39" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -27724,6 +29216,18 @@
       <x:c r="BN40" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/481c70828a4ff20d31a646cc6cc95f3d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO40" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP40" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ40" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR40" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -27924,6 +29428,18 @@
       <x:c r="BN41" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generali</x:v>
       </x:c>
+      <x:c r="BO41" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP41" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ41" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR41" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -28124,6 +29640,18 @@
       <x:c r="BN42" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
+      <x:c r="BO42" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP42" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ42" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR42" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -28324,6 +29852,18 @@
       <x:c r="BN43" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1185c89347a3f21ffc48c9d083c9437c-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO43" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP43" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ43" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR43" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -28524,6 +30064,18 @@
       <x:c r="BN44" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b94310e1c7ecb79f1a24adc757f1b89b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO44" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP44" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ44" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR44" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -28724,6 +30276,18 @@
       <x:c r="BN45" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/49eadcc4a329fc6b74b9f8a82b78cbc3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO45" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP45" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ45" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR45" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -28924,6 +30488,18 @@
       <x:c r="BN46" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/bc97207e3979d1cc23109db0be0e8ed2-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO46" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP46" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ46" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR46" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -29124,6 +30700,18 @@
       <x:c r="BN47" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/282c3318be1b047b7bb5ba94fa4f3231-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO47" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP47" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ47" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR47" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -29324,6 +30912,18 @@
       <x:c r="BN48" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/9fc291fef2f9607a46777d367f900a15-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO48" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP48" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ48" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR48" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -29524,6 +31124,18 @@
       <x:c r="BN49" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/eacc8ae341d15d2c13c02fef88189db3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO49" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP49" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ49" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR49" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -29724,6 +31336,18 @@
       <x:c r="BN50" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1f467c3e37abf9f86c78f44c6a27ee7c-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO50" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP50" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ50" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR50" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -29924,6 +31548,18 @@
       <x:c r="BN51" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b8358a00e5b870194b974ddf8dd415c3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO51" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP51" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ51" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR51" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -30124,6 +31760,18 @@
       <x:c r="BN52" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Wang_DexH2R_A_Benchmark_for_Dynamic_Dexterous_Grasping_in_Human-to-Robot_Handover_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO52" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP52" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ52" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR52" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -30324,6 +31972,18 @@
       <x:c r="BN53" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
+      <x:c r="BO53" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP53" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ53" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR53" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -30524,6 +32184,18 @@
       <x:c r="BN54" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/He_DexVLG_Dexterous_Vision-Language-Grasp_Model_at_Scale_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO54" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BP54" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BR54" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -30724,6 +32396,18 @@
       <x:c r="BN55" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generali</x:v>
       </x:c>
+      <x:c r="BO55" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP55" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ55" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR55" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -30924,6 +32608,18 @@
       <x:c r="BN56" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generali</x:v>
       </x:c>
+      <x:c r="BO56" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP56" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ56" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR56" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -31124,6 +32820,18 @@
       <x:c r="BN57" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Uppal_SPIN_Simultaneous_Perception_Interaction_and_Navigation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO57" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP57" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ57" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR57" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -31324,6 +33032,18 @@
       <x:c r="BN58" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Lu_AnyBimanual_Transferring_Unimanual_Policy_for_General_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO58" t="str">
+        <x:v>A-Upgraded</x:v>
+      </x:c>
+      <x:c r="BP58" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ58" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR58" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -31524,6 +33244,18 @@
       <x:c r="BN59" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Zhang_UniDex_A_Robot_Foundation_Suite_for_Universal_Dexterous_Hand_Control_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO59" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP59" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ59" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR59" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -31724,6 +33456,18 @@
       <x:c r="BN60" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
+      <x:c r="BO60" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP60" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ60" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR60" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -31924,6 +33668,18 @@
       <x:c r="BN61" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38874；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO61" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP61" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ61" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR61" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -32124,6 +33880,18 @@
       <x:c r="BN62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/e4ef7454447baa15a424314e6284441b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO62" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP62" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ62" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR62" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -32324,6 +34092,18 @@
       <x:c r="BN63" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38313；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO63" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP63" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ63" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR63" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -32524,6 +34304,18 @@
       <x:c r="BN64" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/40127；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO64" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP64" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ64" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR64" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -32724,6 +34516,18 @@
       <x:c r="BN65" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28266；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO65" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP65" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ65" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR65" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -32924,6 +34728,18 @@
       <x:c r="BN66" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Heidinger_2HandedAfforder_Learning_Precise_Actionable_Bimanual_Affordances_from_Human_Videos_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
       </x:c>
+      <x:c r="BO66" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BP66" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ66" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BR66" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
@@ -33123,6 +34939,18 @@
       </x:c>
       <x:c r="BN67" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
+      </x:c>
+      <x:c r="BO67" t="str">
+        <x:v>B-Experiment-Not-Extracted</x:v>
+      </x:c>
+      <x:c r="BP67" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BQ67" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BR67" t="str">
+        <x:v>Franka Panda (CALVIN simulation); real-world platform not confirmed at abstract level</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -33160,7 +34988,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d151f50ba90484f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7da2787efe4e06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33374,6 +35202,18 @@
       <x:c r="BC1" t="str">
         <x:v>Evidence Sources</x:v>
       </x:c>
+      <x:c r="BD1" t="str">
+        <x:v>Evidence Upgrade Status</x:v>
+      </x:c>
+      <x:c r="BE1" t="str">
+        <x:v>Supplement Status</x:v>
+      </x:c>
+      <x:c r="BF1" t="str">
+        <x:v>Code Completeness</x:v>
+      </x:c>
+      <x:c r="BG1" t="str">
+        <x:v>Robot Platform Evidence</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="62" customHeight="1">
       <x:c r="A2" t="str">
@@ -33541,6 +35381,18 @@
       <x:c r="BC2" t="str">
         <x:v>Official ICLR Downloads/Proceedings; accepted OpenReview PDF; official project page; official EmbodiChain repository; author publication list; current official CCF directory</x:v>
       </x:c>
+      <x:c r="BD2" t="str">
+        <x:v>B-Experiment-Not-Extracted</x:v>
+      </x:c>
+      <x:c r="BE2" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF2" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BG2" t="str">
+        <x:v>Multiple real-world setups are shown; exact hardware inventory not extracted at abstract/project level</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" t="str">
@@ -33708,6 +35560,18 @@
       <x:c r="BC3" t="str">
         <x:v>https://www.roboticsproceedings.org/rss21/p149.html; https://hnu</x:v>
       </x:c>
+      <x:c r="BD3" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE3" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF3" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG3" t="str">
+        <x:v>Dual robot arms; exact platform pending full-paper check</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" t="str">
@@ -33875,6 +35739,18 @@
       <x:c r="BC4" t="str">
         <x:v>RSS official proceedings abstract</x:v>
       </x:c>
+      <x:c r="BD4" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE4" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF4" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG4" t="str">
+        <x:v>Bimanual gripper system; exact model pending full-paper check</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" t="str">
@@ -34042,6 +35918,18 @@
       <x:c r="BC5" t="str">
         <x:v>RSS official proceedings</x:v>
       </x:c>
+      <x:c r="BD5" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE5" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF5" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG5" t="str">
+        <x:v>Dexterous robotic hand</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" t="str">
@@ -34209,6 +36097,18 @@
       <x:c r="BC6" t="str">
         <x:v>RSS official proceedings abstract</x:v>
       </x:c>
+      <x:c r="BD6" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE6" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF6" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG6" t="str">
+        <x:v>Simulation plus real-world replication</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" t="str">
@@ -34376,6 +36276,18 @@
       <x:c r="BC7" t="str">
         <x:v>IEEE Xplore abstract; official project page</x:v>
       </x:c>
+      <x:c r="BD7" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BE7" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF7" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BG7" t="str">
+        <x:v>Dual robot arms; exact model pending full-paper check</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" t="str">
@@ -34543,6 +36455,18 @@
       <x:c r="BC8" t="str">
         <x:v>IEEE Xplore abstract</x:v>
       </x:c>
+      <x:c r="BD8" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE8" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF8" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG8" t="str">
+        <x:v>Robot arm with visuotactile end effector</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" t="str">
@@ -34710,6 +36634,18 @@
       <x:c r="BC9" t="str">
         <x:v>IEEE Xplore abstract</x:v>
       </x:c>
+      <x:c r="BD9" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE9" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF9" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG9" t="str">
+        <x:v>Multiple robotic arms</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" t="str">
@@ -34876,6 +36812,18 @@
       </x:c>
       <x:c r="BC10" t="str">
         <x:v>IEEE Xplore abstract</x:v>
+      </x:c>
+      <x:c r="BD10" t="str">
+        <x:v>B-Code-Unverified</x:v>
+      </x:c>
+      <x:c r="BE10" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF10" t="str">
+        <x:v>Unavailable</x:v>
+      </x:c>
+      <x:c r="BG10" t="str">
+        <x:v>Multiple hand geometries</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -35022,6 +36970,18 @@
       <x:c r="BC11" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BD11" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BE11" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF11" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BG11" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" t="str">
@@ -35163,6 +37123,18 @@
       <x:c r="BC12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BD12" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BE12" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF12" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BG12" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" t="str">
@@ -35304,6 +37276,18 @@
       <x:c r="BC13" t="str">
         <x:v>Unknown</x:v>
       </x:c>
+      <x:c r="BD13" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BE13" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BG13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" t="str">
@@ -35443,6 +37427,18 @@
         <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC14" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="BD14" t="str">
+        <x:v>B-Fulltext-Unavailable</x:v>
+      </x:c>
+      <x:c r="BE14" t="str">
+        <x:v>Not Checked</x:v>
+      </x:c>
+      <x:c r="BF14" t="str">
+        <x:v>Mostly Complete</x:v>
+      </x:c>
+      <x:c r="BG14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
     </x:row>
@@ -35463,7 +37459,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd07c215f6a644228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb371afc4806b4e43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deep-enrich VLA batch 02
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R701641b7409142a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R1558b6a60fa64e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R70b64d35efd546c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R819c9bf184d84ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rba8f19defe2b4beb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R88f4c2d47b3747c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R82cd8b97fb794536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R2a26ccb80085449a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R3e0a53a2796b4fee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rd3468dd66f94418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R96d1726f960f437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R8f8e965c0b6a40f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rf66c3f58ff424b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rab43dd6ed7cd49db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="PapersTable" displayName="PapersTable" ref="A1:BP5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="68">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="69">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -370,6 +370,7 @@
     <x:tableColumn id="66" name="DOI Status"/>
     <x:tableColumn id="67" name="arXiv Status"/>
     <x:tableColumn id="68" name="Deep Enrichment Status"/>
+    <x:tableColumn id="69" name="Deep Enrichment Completed"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -421,8 +422,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="37" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BK79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="63">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="64">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -486,14 +487,15 @@
     <x:tableColumn id="61" name="DOI Status"/>
     <x:tableColumn id="62" name="arXiv Status"/>
     <x:tableColumn id="63" name="Deep Enrichment Status"/>
+    <x:tableColumn id="64" name="Deep Enrichment Completed"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="38" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CD67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="82">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="83">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="作者 Authors"/>
@@ -576,14 +578,15 @@
     <x:tableColumn id="80" name="DOI Status"/>
     <x:tableColumn id="81" name="arXiv Status"/>
     <x:tableColumn id="82" name="Deep Enrichment Status"/>
+    <x:tableColumn id="83" name="Deep Enrichment Completed"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="39" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BS14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="71">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="72">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
     <x:tableColumn id="3" name="Authors"/>
@@ -655,6 +658,7 @@
     <x:tableColumn id="69" name="DOI Status"/>
     <x:tableColumn id="70" name="arXiv Status"/>
     <x:tableColumn id="71" name="Deep Enrichment Status"/>
+    <x:tableColumn id="72" name="Deep Enrichment Completed"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1093,6 +1097,9 @@
       <x:c r="BP1" t="str">
         <x:v>Deep Enrichment Status</x:v>
       </x:c>
+      <x:c r="BQ1" t="str">
+        <x:v>Deep Enrichment Completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="350" customHeight="1">
       <x:c r="A2" t="str">
@@ -1295,6 +1302,9 @@
       </x:c>
       <x:c r="BP2" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BQ2" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="150" customHeight="1">
@@ -1468,6 +1478,9 @@
       <x:c r="BP3" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BQ3" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" t="str">
@@ -1640,6 +1653,9 @@
       <x:c r="BP4" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BQ4" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
       <x:c r="A5" t="str">
@@ -1811,6 +1827,9 @@
       </x:c>
       <x:c r="BP5" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BQ5" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4824,7 +4843,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f5167e3362547f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab466b1784c74225"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8120,7 +8139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra356fe3872634c89"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284677e1e66c4387"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8471,7 +8490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc51529cf3c46fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c3aa5d73ef94d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9217,7 +9236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R780f6d2c6bd24827"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e7eaae709754c6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9447,6 +9466,9 @@
       <x:c r="BK1" t="str">
         <x:v>Deep Enrichment Status</x:v>
       </x:c>
+      <x:c r="BL1" t="str">
+        <x:v>Deep Enrichment Completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -9628,6 +9650,9 @@
       <x:c r="BK2" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL2" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -9809,6 +9834,9 @@
       <x:c r="BK3" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL3" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -9990,6 +10018,9 @@
       <x:c r="BK4" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL4" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -10173,6 +10204,9 @@
       <x:c r="BK5" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL5" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -10354,6 +10388,9 @@
       <x:c r="BK6" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL6" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -10535,6 +10572,9 @@
       <x:c r="BK7" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL7" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -10714,6 +10754,9 @@
       <x:c r="BK8" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL8" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -10895,6 +10938,9 @@
       <x:c r="BK9" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL9" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -11074,6 +11120,9 @@
       <x:c r="BK10" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL10" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -11257,6 +11306,9 @@
       <x:c r="BK11" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL11" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -11439,6 +11491,9 @@
       </x:c>
       <x:c r="BK12" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL12" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -11623,6 +11678,9 @@
       <x:c r="BK13" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL13" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -11804,6 +11862,9 @@
       <x:c r="BK14" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL14" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -11986,6 +12047,9 @@
       </x:c>
       <x:c r="BK15" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL15" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -12166,6 +12230,9 @@
       <x:c r="BK16" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL16" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -12345,6 +12412,9 @@
       <x:c r="BK17" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL17" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -12461,7 +12531,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP18" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AQ18" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -12479,7 +12549,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV18" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="AW18" t="str">
         <x:v>Not Found</x:v>
@@ -12523,6 +12593,9 @@
       </x:c>
       <x:c r="BK18" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL18" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
@@ -12705,6 +12778,9 @@
       <x:c r="BK19" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL19" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -12884,6 +12960,9 @@
       <x:c r="BK20" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL20" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -13065,6 +13144,9 @@
       <x:c r="BK21" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL21" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -13246,6 +13328,9 @@
       <x:c r="BK22" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL22" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -13427,6 +13512,9 @@
       <x:c r="BK23" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL23" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -13608,6 +13696,9 @@
       <x:c r="BK24" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL24" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -13787,6 +13878,9 @@
       <x:c r="BK25" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL25" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -13968,6 +14062,9 @@
       <x:c r="BK26" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL26" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -14149,6 +14246,9 @@
       <x:c r="BK27" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL27" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -14330,6 +14430,9 @@
       <x:c r="BK28" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL28" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -14511,6 +14614,9 @@
       <x:c r="BK29" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL29" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -14692,6 +14798,9 @@
       <x:c r="BK30" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL30" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -14873,6 +14982,9 @@
       <x:c r="BK31" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL31" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -15054,6 +15166,9 @@
       <x:c r="BK32" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL32" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -15235,6 +15350,9 @@
       <x:c r="BK33" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL33" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -15416,6 +15534,9 @@
       <x:c r="BK34" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL34" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -15597,6 +15718,9 @@
       <x:c r="BK35" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL35" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -15778,6 +15902,9 @@
       <x:c r="BK36" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL36" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -15959,6 +16086,9 @@
       <x:c r="BK37" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL37" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -16140,6 +16270,9 @@
       <x:c r="BK38" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL38" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -16321,6 +16454,9 @@
       <x:c r="BK39" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL39" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -16500,6 +16636,9 @@
       <x:c r="BK40" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL40" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -16679,6 +16818,9 @@
       <x:c r="BK41" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL41" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -16858,6 +17000,9 @@
       <x:c r="BK42" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL42" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -17037,6 +17182,9 @@
       <x:c r="BK43" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL43" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -17216,6 +17364,9 @@
       <x:c r="BK44" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL44" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -17395,6 +17546,9 @@
       <x:c r="BK45" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL45" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -17576,6 +17730,9 @@
       <x:c r="BK46" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL46" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -17757,6 +17914,9 @@
       <x:c r="BK47" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL47" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -17938,6 +18098,9 @@
       <x:c r="BK48" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL48" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -18119,6 +18282,9 @@
       <x:c r="BK49" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL49" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -18300,6 +18466,9 @@
       <x:c r="BK50" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL50" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -18481,6 +18650,9 @@
       <x:c r="BK51" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL51" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -18662,6 +18834,9 @@
       <x:c r="BK52" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL52" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -18843,6 +19018,9 @@
       <x:c r="BK53" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL53" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -19024,6 +19202,9 @@
       <x:c r="BK54" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL54" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -19205,6 +19386,9 @@
       <x:c r="BK55" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL55" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -19386,6 +19570,9 @@
       <x:c r="BK56" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL56" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -19567,6 +19754,9 @@
       <x:c r="BK57" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL57" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -19754,6 +19944,9 @@
       <x:c r="BK58" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL58" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -19941,6 +20134,9 @@
       <x:c r="BK59" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL59" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -20126,6 +20322,9 @@
       <x:c r="BK60" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL60" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -20250,7 +20449,7 @@
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
       <x:c r="AP61" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AQ61" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -20268,7 +20467,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
       <x:c r="AV61" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="AW61" t="str">
         <x:v>Not Found</x:v>
@@ -20312,6 +20511,9 @@
       </x:c>
       <x:c r="BK61" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL61" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
@@ -20500,6 +20702,9 @@
       <x:c r="BK62" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL62" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -20624,7 +20829,7 @@
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
       <x:c r="AP63" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AQ63" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -20642,7 +20847,7 @@
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
       </x:c>
       <x:c r="AV63" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="AW63" t="str">
         <x:v>Not Found</x:v>
@@ -20686,6 +20891,9 @@
       </x:c>
       <x:c r="BK63" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL63" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
@@ -20874,6 +21082,9 @@
       <x:c r="BK64" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL64" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -21061,6 +21272,9 @@
       <x:c r="BK65" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL65" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -21248,6 +21462,9 @@
       <x:c r="BK66" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL66" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="67" ht="58" customHeight="1">
       <x:c r="A67" t="str">
@@ -21434,6 +21651,9 @@
       </x:c>
       <x:c r="BK67" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL67" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="58" customHeight="1">
@@ -21620,6 +21840,9 @@
       <x:c r="BK68" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL68" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
       <x:c r="A69" t="str">
@@ -21807,6 +22030,9 @@
       <x:c r="BK69" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL69" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" t="str">
@@ -21994,6 +22220,9 @@
       <x:c r="BK70" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL70" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" t="str">
@@ -22181,6 +22410,9 @@
       <x:c r="BK71" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL71" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="72" ht="58" customHeight="1">
       <x:c r="A72" t="str">
@@ -22368,6 +22600,9 @@
       <x:c r="BK72" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL72" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="58" customHeight="1">
       <x:c r="A73" t="str">
@@ -22555,6 +22790,9 @@
       <x:c r="BK73" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL73" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="58" customHeight="1">
       <x:c r="A74" t="str">
@@ -22679,7 +22917,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP74" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AQ74" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -22697,7 +22935,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV74" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="AW74" t="str">
         <x:v>Not Found</x:v>
@@ -22741,6 +22979,9 @@
       </x:c>
       <x:c r="BK74" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL74" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="58" customHeight="1">
@@ -22866,7 +23107,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AP75" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AQ75" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -22884,7 +23125,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV75" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="AW75" t="str">
         <x:v>Not Found</x:v>
@@ -22928,6 +23169,9 @@
       </x:c>
       <x:c r="BK75" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL75" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="58" customHeight="1">
@@ -23112,6 +23356,9 @@
       <x:c r="BK76" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL76" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="77" ht="58" customHeight="1">
       <x:c r="A77" t="str">
@@ -23294,6 +23541,9 @@
       </x:c>
       <x:c r="BK77" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL77" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="58" customHeight="1">
@@ -23478,6 +23728,9 @@
       <x:c r="BK78" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BL78" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -23666,6 +23919,9 @@
       </x:c>
       <x:c r="BK79" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BL79" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23688,7 +23944,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60e967459dd747e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123c3f02f61949d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23996,6 +24252,9 @@
       <x:c r="CD1" t="str">
         <x:v>Deep Enrichment Status</x:v>
       </x:c>
+      <x:c r="CE1" t="str">
+        <x:v>Deep Enrichment Completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -24234,6 +24493,9 @@
       <x:c r="CD2" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE2" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -24472,6 +24734,9 @@
       <x:c r="CD3" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE3" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -24710,6 +24975,9 @@
       <x:c r="CD4" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE4" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -24948,6 +25216,9 @@
       <x:c r="CD5" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE5" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -25186,6 +25457,9 @@
       <x:c r="CD6" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE6" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -25424,6 +25698,9 @@
       <x:c r="CD7" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE7" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -25662,6 +25939,9 @@
       <x:c r="CD8" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE8" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -25898,6 +26178,9 @@
       <x:c r="CD9" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE9" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -26140,6 +26423,9 @@
       <x:c r="CD10" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE10" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -26321,7 +26607,7 @@
         <x:v>VLA; 3D Manipulation / Data Efficiency</x:v>
       </x:c>
       <x:c r="BI11" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="BJ11" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -26339,7 +26625,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
       </x:c>
       <x:c r="BO11" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="BP11" t="str">
         <x:v>Not Found</x:v>
@@ -26383,6 +26669,9 @@
       </x:c>
       <x:c r="CD11" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="CE11" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -26628,6 +26917,9 @@
       <x:c r="CD12" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE12" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -26809,7 +27101,7 @@
         <x:v>VLA; Autoregressive Reasoning / Diffusion</x:v>
       </x:c>
       <x:c r="BI13" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="BJ13" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -26827,7 +27119,7 @@
         <x:v>https://proceedings.mlr.press/v267/wen25g.html；官方摘要/论文集元数据</x:v>
       </x:c>
       <x:c r="BO13" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="BP13" t="str">
         <x:v>Not Found</x:v>
@@ -26871,6 +27163,9 @@
       </x:c>
       <x:c r="CD13" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="CE13" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -27116,6 +27411,9 @@
       <x:c r="CD14" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE14" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -27359,6 +27657,9 @@
       </x:c>
       <x:c r="CD15" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="CE15" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
@@ -27602,6 +27903,9 @@
       <x:c r="CD16" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE16" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -27846,6 +28150,9 @@
       <x:c r="CD17" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE17" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -28090,6 +28397,9 @@
       <x:c r="CD18" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE18" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -28334,6 +28644,9 @@
       <x:c r="CD19" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE19" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -28578,6 +28891,9 @@
       <x:c r="CD20" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE20" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -28824,6 +29140,9 @@
       <x:c r="CD21" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE21" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -29070,6 +29389,9 @@
       <x:c r="CD22" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE22" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -29316,6 +29638,9 @@
       <x:c r="CD23" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE23" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -29562,6 +29887,9 @@
       <x:c r="CD24" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE24" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -29808,6 +30136,9 @@
       <x:c r="CD25" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE25" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -30054,6 +30385,9 @@
       <x:c r="CD26" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE26" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -30300,6 +30634,9 @@
       <x:c r="CD27" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE27" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -30546,6 +30883,9 @@
       <x:c r="CD28" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE28" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -30792,6 +31132,9 @@
       <x:c r="CD29" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE29" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -31038,6 +31381,9 @@
       <x:c r="CD30" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE30" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -31284,6 +31630,9 @@
       <x:c r="CD31" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE31" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -31530,6 +31879,9 @@
       <x:c r="CD32" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE32" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -31776,6 +32128,9 @@
       <x:c r="CD33" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE33" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -32022,6 +32377,9 @@
       <x:c r="CD34" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE34" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -32268,6 +32626,9 @@
       <x:c r="CD35" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE35" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -32514,6 +32875,9 @@
       <x:c r="CD36" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE36" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -32760,6 +33124,9 @@
       <x:c r="CD37" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE37" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -33006,6 +33373,9 @@
       <x:c r="CD38" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE38" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -33252,6 +33622,9 @@
       <x:c r="CD39" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE39" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -33498,6 +33871,9 @@
       <x:c r="CD40" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE40" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -33744,6 +34120,9 @@
       <x:c r="CD41" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE41" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -33927,7 +34306,7 @@
         <x:v>Visual Chain-of-Thought</x:v>
       </x:c>
       <x:c r="BI42" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="BJ42" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -33945,7 +34324,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
       </x:c>
       <x:c r="BO42" t="str">
-        <x:v>B-Code-Unverified</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="BP42" t="str">
         <x:v>Not Found</x:v>
@@ -33989,6 +34368,9 @@
       </x:c>
       <x:c r="CD42" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="CE42" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
@@ -34236,6 +34618,9 @@
       <x:c r="CD43" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE43" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -34482,6 +34867,9 @@
       <x:c r="CD44" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE44" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -34728,6 +35116,9 @@
       <x:c r="CD45" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE45" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -34974,6 +35365,9 @@
       <x:c r="CD46" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE46" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -35220,6 +35614,9 @@
       <x:c r="CD47" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE47" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -35466,6 +35863,9 @@
       <x:c r="CD48" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE48" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -35712,6 +36112,9 @@
       <x:c r="CD49" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE49" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -35958,6 +36361,9 @@
       <x:c r="CD50" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE50" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -36204,6 +36610,9 @@
       <x:c r="CD51" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE51" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -36450,6 +36859,9 @@
       <x:c r="CD52" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE52" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -36696,6 +37108,9 @@
       <x:c r="CD53" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE53" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -36942,6 +37357,9 @@
       <x:c r="CD54" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE54" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -37188,6 +37606,9 @@
       <x:c r="CD55" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE55" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -37434,6 +37855,9 @@
       <x:c r="CD56" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE56" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -37680,6 +38104,9 @@
       <x:c r="CD57" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE57" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -37926,6 +38353,9 @@
       <x:c r="CD58" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE58" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -38172,6 +38602,9 @@
       <x:c r="CD59" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE59" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -38418,6 +38851,9 @@
       <x:c r="CD60" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE60" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -38664,6 +39100,9 @@
       <x:c r="CD61" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE61" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -38910,6 +39349,9 @@
       <x:c r="CD62" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE62" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -39156,6 +39598,9 @@
       <x:c r="CD63" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE63" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -39402,6 +39847,9 @@
       <x:c r="CD64" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE64" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -39648,6 +40096,9 @@
       <x:c r="CD65" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE65" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -39894,6 +40345,9 @@
       <x:c r="CD66" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="CE66" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
@@ -40139,6 +40593,9 @@
       </x:c>
       <x:c r="CD67" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="CE67" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -40176,7 +40633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82da15685a574f77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3383174a60b84151"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40438,6 +40895,9 @@
       <x:c r="BS1" t="str">
         <x:v>Deep Enrichment Status</x:v>
       </x:c>
+      <x:c r="BT1" t="str">
+        <x:v>Deep Enrichment Completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="62" customHeight="1">
       <x:c r="A2" t="str">
@@ -40651,6 +41111,9 @@
       <x:c r="BS2" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT2" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" t="str">
@@ -40864,6 +41327,9 @@
       <x:c r="BS3" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT3" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" t="str">
@@ -41077,6 +41543,9 @@
       <x:c r="BS4" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT4" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" t="str">
@@ -41290,6 +41759,9 @@
       <x:c r="BS5" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT5" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" t="str">
@@ -41503,6 +41975,9 @@
       <x:c r="BS6" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT6" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" t="str">
@@ -41716,6 +42191,9 @@
       <x:c r="BS7" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT7" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" t="str">
@@ -41929,6 +42407,9 @@
       <x:c r="BS8" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT8" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" t="str">
@@ -42142,6 +42623,9 @@
       <x:c r="BS9" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT9" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" t="str">
@@ -42354,6 +42838,9 @@
       </x:c>
       <x:c r="BS10" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BT10" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -42483,7 +42970,7 @@
         <x:v>Library Analysis / Research Note: Unknown / Needs Full-Paper Verification</x:v>
       </x:c>
       <x:c r="AX11" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="AY11" t="str">
         <x:v>Unknown / Needs paper-specific evidence; no inference added from title alone.</x:v>
@@ -42501,7 +42988,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="BD11" t="str">
-        <x:v>B-Fulltext-Unavailable</x:v>
+        <x:v>A-Upgraded</x:v>
       </x:c>
       <x:c r="BE11" t="str">
         <x:v>Not Found</x:v>
@@ -42545,6 +43032,9 @@
       </x:c>
       <x:c r="BS11" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BT11" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -42733,6 +43223,9 @@
       <x:c r="BS12" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT12" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" t="str">
@@ -42920,6 +43413,9 @@
       <x:c r="BS13" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
       </x:c>
+      <x:c r="BT13" t="str">
+        <x:v>false</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" t="str">
@@ -43106,6 +43602,9 @@
       </x:c>
       <x:c r="BS14" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
+      </x:c>
+      <x:c r="BT14" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -43125,7 +43624,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96b87176bc384e0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02555f8e754949cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct batch 02 enrichment status sync
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R2a26ccb80085449a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R3e0a53a2796b4fee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rd3468dd66f94418c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R96d1726f960f437f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R8f8e965c0b6a40f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rf66c3f58ff424b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rab43dd6ed7cd49db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R5023eba1be2843cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rc816669bb72649ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R11666bc5d61d4589"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rf79ede85faf24489"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rccafa41268f94673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R20aa7941aa944d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Ref69d14cbb6e41d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="40" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="69">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -422,7 +422,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="41" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="64">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -494,7 +494,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="42" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="83">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -585,7 +585,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="43" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="72">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -4843,7 +4843,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab466b1784c74225"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7eac612cde249c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8139,7 +8139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R284677e1e66c4387"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radca5a9c1f434655"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8490,7 +8490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c3aa5d73ef94d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5f4702ba84a4b7a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9236,7 +9236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e7eaae709754c6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb064adde1aa841e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23944,7 +23944,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123c3f02f61949d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7e7c330c2d54d21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40633,7 +40633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3383174a60b84151"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54c39461032744ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43624,7 +43624,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02555f8e754949cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf485eb76d0dc42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Deep-enrich batch 03: VLA and grounded policies
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R5023eba1be2843cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rc816669bb72649ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R11666bc5d61d4589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rf79ede85faf24489"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rccafa41268f94673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R20aa7941aa944d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Ref69d14cbb6e41d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R2b48adc121074eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rdebf079706ca4e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R1c65c5a34a5a453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R0811c3c2d8644999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R38631e8e5565466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc562fd02888d4b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R676ebc86ceae431c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="69">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -422,7 +422,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="64">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -494,7 +494,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="83">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -585,7 +585,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="72">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -4843,7 +4843,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7eac612cde249c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c3f422684ff480c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8139,7 +8139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radca5a9c1f434655"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b68bed915a04772"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8490,7 +8490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5f4702ba84a4b7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R619b0453d5674480"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9236,7 +9236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb064adde1aa841e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6000c873d1a24c67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23944,7 +23944,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7e7c330c2d54d21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R546fae1cb2be4f0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40633,7 +40633,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54c39461032744ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b0842603324a9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43624,7 +43624,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf485eb76d0dc42ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad226df4586d4d02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Advance enrichment queue and defer blocked papers
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R2b48adc121074eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rdebf079706ca4e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R1c65c5a34a5a453a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R0811c3c2d8644999"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R38631e8e5565466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc562fd02888d4b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R676ebc86ceae431c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R088f20caa81c4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R79c228a70d0e482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R32ac521297054fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R1051e123e15c4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rd6933891c3d94d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Ree6cb4209d1f4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R2480683c407b4386"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="48" name="PapersTable" displayName="PapersTable" ref="A1:BQ5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="69">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="PapersTable" displayName="PapersTable" ref="A1:BR5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="70">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -371,6 +371,7 @@
     <x:tableColumn id="67" name="arXiv Status"/>
     <x:tableColumn id="68" name="Deep Enrichment Status"/>
     <x:tableColumn id="69" name="Deep Enrichment Completed"/>
+    <x:tableColumn id="70" name="Queue Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -422,8 +423,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="49" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BL79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="64">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BM79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="65">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="年份 Year"/>
@@ -488,14 +489,15 @@
     <x:tableColumn id="62" name="arXiv Status"/>
     <x:tableColumn id="63" name="Deep Enrichment Status"/>
     <x:tableColumn id="64" name="Deep Enrichment Completed"/>
+    <x:tableColumn id="65" name="Queue Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="50" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CE67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="83">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CF67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="84">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
     <x:tableColumn id="3" name="作者 Authors"/>
@@ -579,14 +581,15 @@
     <x:tableColumn id="81" name="arXiv Status"/>
     <x:tableColumn id="82" name="Deep Enrichment Status"/>
     <x:tableColumn id="83" name="Deep Enrichment Completed"/>
+    <x:tableColumn id="84" name="Queue Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="51" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BT14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="72">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BU14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="73">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
     <x:tableColumn id="3" name="Authors"/>
@@ -659,6 +662,7 @@
     <x:tableColumn id="70" name="arXiv Status"/>
     <x:tableColumn id="71" name="Deep Enrichment Status"/>
     <x:tableColumn id="72" name="Deep Enrichment Completed"/>
+    <x:tableColumn id="73" name="Queue Status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1100,6 +1104,9 @@
       <x:c r="BQ1" t="str">
         <x:v>Deep Enrichment Completed</x:v>
       </x:c>
+      <x:c r="BR1" t="str">
+        <x:v>Queue Status</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="350" customHeight="1">
       <x:c r="A2" t="str">
@@ -1306,6 +1313,7 @@
       <x:c r="BQ2" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BR2" t="str"/>
     </x:row>
     <x:row r="3" ht="150" customHeight="1">
       <x:c r="A3" t="str">
@@ -1481,6 +1489,7 @@
       <x:c r="BQ3" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BR3" t="str"/>
     </x:row>
     <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" t="str">
@@ -1656,6 +1665,7 @@
       <x:c r="BQ4" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BR4" t="str"/>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
       <x:c r="A5" t="str">
@@ -1831,6 +1841,7 @@
       <x:c r="BQ5" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BR5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="AC6" s="7"/>
@@ -4843,7 +4854,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c3f422684ff480c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d56b28395454f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8139,7 +8150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b68bed915a04772"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ed45e795c4b4da1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8490,7 +8501,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R619b0453d5674480"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36fe4e66a443490e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9236,7 +9247,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6000c873d1a24c67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe8d92f56e3b4a6e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9469,6 +9480,9 @@
       <x:c r="BL1" t="str">
         <x:v>Deep Enrichment Completed</x:v>
       </x:c>
+      <x:c r="BM1" t="str">
+        <x:v>Queue Status</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -9653,6 +9667,7 @@
       <x:c r="BL2" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM2" t="str"/>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -9837,6 +9852,7 @@
       <x:c r="BL3" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM3" t="str"/>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -10021,6 +10037,7 @@
       <x:c r="BL4" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM4" t="str"/>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -10207,6 +10224,7 @@
       <x:c r="BL5" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM5" t="str"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -10391,6 +10409,7 @@
       <x:c r="BL6" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM6" t="str"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -10575,6 +10594,7 @@
       <x:c r="BL7" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM7" t="str"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -10757,6 +10777,7 @@
       <x:c r="BL8" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM8" t="str"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -10941,6 +10962,7 @@
       <x:c r="BL9" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM9" t="str"/>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -11123,6 +11145,7 @@
       <x:c r="BL10" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM10" t="str"/>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -11309,6 +11332,7 @@
       <x:c r="BL11" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM11" t="str"/>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -11495,6 +11519,7 @@
       <x:c r="BL12" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM12" t="str"/>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -11681,6 +11706,7 @@
       <x:c r="BL13" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM13" t="str"/>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -11865,6 +11891,7 @@
       <x:c r="BL14" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM14" t="str"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -12051,6 +12078,7 @@
       <x:c r="BL15" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM15" t="str"/>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" t="str">
@@ -12233,6 +12261,7 @@
       <x:c r="BL16" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM16" t="str"/>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -12415,6 +12444,7 @@
       <x:c r="BL17" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM17" t="str"/>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -12597,6 +12627,7 @@
       <x:c r="BL18" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM18" t="str"/>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -12781,6 +12812,7 @@
       <x:c r="BL19" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM19" t="str"/>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -12963,6 +12995,7 @@
       <x:c r="BL20" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM20" t="str"/>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -13147,6 +13180,7 @@
       <x:c r="BL21" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM21" t="str"/>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -13331,6 +13365,7 @@
       <x:c r="BL22" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM22" t="str"/>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -13515,6 +13550,7 @@
       <x:c r="BL23" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM23" t="str"/>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -13699,6 +13735,7 @@
       <x:c r="BL24" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM24" t="str"/>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -13881,6 +13918,7 @@
       <x:c r="BL25" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM25" t="str"/>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -14065,6 +14103,7 @@
       <x:c r="BL26" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM26" t="str"/>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -14249,6 +14288,7 @@
       <x:c r="BL27" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM27" t="str"/>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -14433,6 +14473,7 @@
       <x:c r="BL28" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM28" t="str"/>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -14617,6 +14658,7 @@
       <x:c r="BL29" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM29" t="str"/>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -14801,6 +14843,7 @@
       <x:c r="BL30" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM30" t="str"/>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -14985,6 +15028,7 @@
       <x:c r="BL31" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM31" t="str"/>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -15169,6 +15213,7 @@
       <x:c r="BL32" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM32" t="str"/>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -15353,6 +15398,7 @@
       <x:c r="BL33" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM33" t="str"/>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -15537,6 +15583,7 @@
       <x:c r="BL34" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM34" t="str"/>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -15721,6 +15768,7 @@
       <x:c r="BL35" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM35" t="str"/>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -15905,6 +15953,7 @@
       <x:c r="BL36" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM36" t="str"/>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -16089,6 +16138,7 @@
       <x:c r="BL37" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM37" t="str"/>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -16273,6 +16323,7 @@
       <x:c r="BL38" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM38" t="str"/>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -16457,6 +16508,7 @@
       <x:c r="BL39" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM39" t="str"/>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -16639,6 +16691,7 @@
       <x:c r="BL40" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM40" t="str"/>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -16821,6 +16874,7 @@
       <x:c r="BL41" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM41" t="str"/>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -17003,6 +17057,7 @@
       <x:c r="BL42" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM42" t="str"/>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -17185,6 +17240,7 @@
       <x:c r="BL43" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM43" t="str"/>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -17367,6 +17423,7 @@
       <x:c r="BL44" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM44" t="str"/>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -17549,6 +17606,7 @@
       <x:c r="BL45" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM45" t="str"/>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -17733,6 +17791,7 @@
       <x:c r="BL46" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM46" t="str"/>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -17917,6 +17976,7 @@
       <x:c r="BL47" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM47" t="str"/>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -18101,6 +18161,7 @@
       <x:c r="BL48" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM48" t="str"/>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -18285,6 +18346,7 @@
       <x:c r="BL49" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM49" t="str"/>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -18469,6 +18531,7 @@
       <x:c r="BL50" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM50" t="str"/>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -18653,6 +18716,7 @@
       <x:c r="BL51" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM51" t="str"/>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -18837,6 +18901,7 @@
       <x:c r="BL52" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM52" t="str"/>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -19021,6 +19086,7 @@
       <x:c r="BL53" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM53" t="str"/>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -19205,6 +19271,7 @@
       <x:c r="BL54" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM54" t="str"/>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -19389,6 +19456,7 @@
       <x:c r="BL55" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM55" t="str"/>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -19573,6 +19641,7 @@
       <x:c r="BL56" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM56" t="str"/>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -19757,6 +19826,7 @@
       <x:c r="BL57" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM57" t="str"/>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -19947,6 +20017,7 @@
       <x:c r="BL58" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM58" t="str"/>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -20137,6 +20208,7 @@
       <x:c r="BL59" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM59" t="str"/>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -20325,6 +20397,7 @@
       <x:c r="BL60" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM60" t="str"/>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -20515,6 +20588,7 @@
       <x:c r="BL61" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM61" t="str"/>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -20705,6 +20779,7 @@
       <x:c r="BL62" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM62" t="str"/>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -20895,6 +20970,7 @@
       <x:c r="BL63" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM63" t="str"/>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -21085,6 +21161,7 @@
       <x:c r="BL64" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM64" t="str"/>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -21275,6 +21352,7 @@
       <x:c r="BL65" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM65" t="str"/>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -21465,6 +21543,7 @@
       <x:c r="BL66" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM66" t="str"/>
     </x:row>
     <x:row r="67" ht="58" customHeight="1">
       <x:c r="A67" t="str">
@@ -21655,6 +21734,7 @@
       <x:c r="BL67" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM67" t="str"/>
     </x:row>
     <x:row r="68" ht="58" customHeight="1">
       <x:c r="A68" t="str">
@@ -21843,6 +21923,7 @@
       <x:c r="BL68" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM68" t="str"/>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
       <x:c r="A69" t="str">
@@ -22033,6 +22114,7 @@
       <x:c r="BL69" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM69" t="str"/>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" t="str">
@@ -22223,6 +22305,7 @@
       <x:c r="BL70" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM70" t="str"/>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" t="str">
@@ -22413,6 +22496,7 @@
       <x:c r="BL71" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM71" t="str"/>
     </x:row>
     <x:row r="72" ht="58" customHeight="1">
       <x:c r="A72" t="str">
@@ -22603,6 +22687,7 @@
       <x:c r="BL72" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM72" t="str"/>
     </x:row>
     <x:row r="73" ht="58" customHeight="1">
       <x:c r="A73" t="str">
@@ -22793,6 +22878,7 @@
       <x:c r="BL73" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM73" t="str"/>
     </x:row>
     <x:row r="74" ht="58" customHeight="1">
       <x:c r="A74" t="str">
@@ -22983,6 +23069,7 @@
       <x:c r="BL74" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM74" t="str"/>
     </x:row>
     <x:row r="75" ht="58" customHeight="1">
       <x:c r="A75" t="str">
@@ -23173,6 +23260,7 @@
       <x:c r="BL75" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM75" t="str"/>
     </x:row>
     <x:row r="76" ht="58" customHeight="1">
       <x:c r="A76" t="str">
@@ -23359,6 +23447,7 @@
       <x:c r="BL76" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM76" t="str"/>
     </x:row>
     <x:row r="77" ht="58" customHeight="1">
       <x:c r="A77" t="str">
@@ -23545,6 +23634,7 @@
       <x:c r="BL77" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM77" t="str"/>
     </x:row>
     <x:row r="78" ht="58" customHeight="1">
       <x:c r="A78" t="str">
@@ -23731,6 +23821,7 @@
       <x:c r="BL78" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM78" t="str"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -23923,6 +24014,7 @@
       <x:c r="BL79" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BM79" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
@@ -23944,7 +24036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R546fae1cb2be4f0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95465e0d0a6042d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24255,6 +24347,9 @@
       <x:c r="CE1" t="str">
         <x:v>Deep Enrichment Completed</x:v>
       </x:c>
+      <x:c r="CF1" t="str">
+        <x:v>Queue Status</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="58" customHeight="1">
       <x:c r="A2" t="str">
@@ -24496,6 +24591,7 @@
       <x:c r="CE2" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF2" t="str"/>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -24737,6 +24833,7 @@
       <x:c r="CE3" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF3" t="str"/>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -24978,6 +25075,7 @@
       <x:c r="CE4" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF4" t="str"/>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -25219,6 +25317,7 @@
       <x:c r="CE5" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF5" t="str"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -25460,6 +25559,7 @@
       <x:c r="CE6" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF6" t="str"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -25701,6 +25801,7 @@
       <x:c r="CE7" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF7" t="str"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -25942,6 +26043,7 @@
       <x:c r="CE8" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF8" t="str"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -26181,6 +26283,7 @@
       <x:c r="CE9" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF9" t="str"/>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -26426,6 +26529,7 @@
       <x:c r="CE10" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF10" t="str"/>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -26673,6 +26777,7 @@
       <x:c r="CE11" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF11" t="str"/>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -26920,6 +27025,7 @@
       <x:c r="CE12" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF12" t="str"/>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -27167,6 +27273,7 @@
       <x:c r="CE13" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF13" t="str"/>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -27414,6 +27521,7 @@
       <x:c r="CE14" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF14" t="str"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -27661,6 +27769,7 @@
       <x:c r="CE15" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF15" t="str"/>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" t="str">
@@ -27906,6 +28015,7 @@
       <x:c r="CE16" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF16" t="str"/>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -28153,6 +28263,7 @@
       <x:c r="CE17" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF17" t="str"/>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -28400,6 +28511,7 @@
       <x:c r="CE18" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF18" t="str"/>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -28647,6 +28759,7 @@
       <x:c r="CE19" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF19" t="str"/>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -28894,6 +29007,7 @@
       <x:c r="CE20" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF20" t="str"/>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -29143,6 +29257,7 @@
       <x:c r="CE21" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF21" t="str"/>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -29392,6 +29507,7 @@
       <x:c r="CE22" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF22" t="str"/>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -29641,6 +29757,7 @@
       <x:c r="CE23" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF23" t="str"/>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -29890,6 +30007,7 @@
       <x:c r="CE24" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF24" t="str"/>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -30139,6 +30257,7 @@
       <x:c r="CE25" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF25" t="str"/>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -30388,6 +30507,7 @@
       <x:c r="CE26" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF26" t="str"/>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -30637,6 +30757,7 @@
       <x:c r="CE27" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF27" t="str"/>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -30886,6 +31007,7 @@
       <x:c r="CE28" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF28" t="str"/>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -31135,6 +31257,7 @@
       <x:c r="CE29" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF29" t="str"/>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -31384,6 +31507,7 @@
       <x:c r="CE30" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF30" t="str"/>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -31633,6 +31757,7 @@
       <x:c r="CE31" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF31" t="str"/>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -31882,6 +32007,7 @@
       <x:c r="CE32" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF32" t="str"/>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -32131,6 +32257,7 @@
       <x:c r="CE33" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF33" t="str"/>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -32380,6 +32507,7 @@
       <x:c r="CE34" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF34" t="str"/>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -32629,6 +32757,7 @@
       <x:c r="CE35" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF35" t="str"/>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -32878,6 +33007,7 @@
       <x:c r="CE36" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF36" t="str"/>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -33127,6 +33257,7 @@
       <x:c r="CE37" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF37" t="str"/>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -33376,6 +33507,7 @@
       <x:c r="CE38" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF38" t="str"/>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -33625,6 +33757,7 @@
       <x:c r="CE39" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF39" t="str"/>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -33874,6 +34007,7 @@
       <x:c r="CE40" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF40" t="str"/>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -34123,6 +34257,7 @@
       <x:c r="CE41" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF41" t="str"/>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -34372,6 +34507,7 @@
       <x:c r="CE42" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF42" t="str"/>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -34621,6 +34757,7 @@
       <x:c r="CE43" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF43" t="str"/>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -34870,6 +35007,7 @@
       <x:c r="CE44" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF44" t="str"/>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -35119,6 +35257,7 @@
       <x:c r="CE45" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF45" t="str"/>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -35368,6 +35507,7 @@
       <x:c r="CE46" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF46" t="str"/>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -35617,6 +35757,7 @@
       <x:c r="CE47" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF47" t="str"/>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -35866,6 +36007,7 @@
       <x:c r="CE48" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF48" t="str"/>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -36115,6 +36257,7 @@
       <x:c r="CE49" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF49" t="str"/>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -36364,6 +36507,7 @@
       <x:c r="CE50" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF50" t="str"/>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -36613,6 +36757,7 @@
       <x:c r="CE51" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF51" t="str"/>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -36862,6 +37007,7 @@
       <x:c r="CE52" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF52" t="str"/>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -37111,6 +37257,7 @@
       <x:c r="CE53" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF53" t="str"/>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -37360,6 +37507,7 @@
       <x:c r="CE54" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF54" t="str"/>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -37609,6 +37757,7 @@
       <x:c r="CE55" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF55" t="str"/>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -37858,6 +38007,7 @@
       <x:c r="CE56" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF56" t="str"/>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -38107,6 +38257,7 @@
       <x:c r="CE57" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF57" t="str"/>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -38356,6 +38507,7 @@
       <x:c r="CE58" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF58" t="str"/>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -38605,6 +38757,7 @@
       <x:c r="CE59" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF59" t="str"/>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -38854,6 +39007,7 @@
       <x:c r="CE60" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF60" t="str"/>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -39103,6 +39257,7 @@
       <x:c r="CE61" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF61" t="str"/>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -39352,6 +39507,7 @@
       <x:c r="CE62" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF62" t="str"/>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -39601,6 +39757,7 @@
       <x:c r="CE63" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF63" t="str"/>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -39850,6 +40007,7 @@
       <x:c r="CE64" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF64" t="str"/>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -40099,6 +40257,7 @@
       <x:c r="CE65" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF65" t="str"/>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -40348,6 +40507,7 @@
       <x:c r="CE66" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF66" t="str"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
@@ -40597,6 +40757,7 @@
       <x:c r="CE67" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="CF67" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="10">
@@ -40633,7 +40794,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4b0842603324a9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ea64be2c924395"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40898,6 +41059,9 @@
       <x:c r="BT1" t="str">
         <x:v>Deep Enrichment Completed</x:v>
       </x:c>
+      <x:c r="BU1" t="str">
+        <x:v>Queue Status</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="62" customHeight="1">
       <x:c r="A2" t="str">
@@ -41114,6 +41278,7 @@
       <x:c r="BT2" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU2" t="str"/>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" t="str">
@@ -41330,6 +41495,7 @@
       <x:c r="BT3" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU3" t="str"/>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" t="str">
@@ -41546,6 +41712,7 @@
       <x:c r="BT4" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU4" t="str"/>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" t="str">
@@ -41762,6 +41929,7 @@
       <x:c r="BT5" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU5" t="str"/>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" t="str">
@@ -41978,6 +42146,7 @@
       <x:c r="BT6" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU6" t="str"/>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" t="str">
@@ -42194,6 +42363,7 @@
       <x:c r="BT7" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU7" t="str"/>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" t="str">
@@ -42410,6 +42580,7 @@
       <x:c r="BT8" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU8" t="str"/>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" t="str">
@@ -42626,6 +42797,7 @@
       <x:c r="BT9" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU9" t="str"/>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" t="str">
@@ -42842,6 +43014,7 @@
       <x:c r="BT10" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU10" t="str"/>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" t="str">
@@ -43036,6 +43209,7 @@
       <x:c r="BT11" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU11" t="str"/>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" t="str">
@@ -43226,6 +43400,7 @@
       <x:c r="BT12" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU12" t="str"/>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" t="str">
@@ -43416,6 +43591,7 @@
       <x:c r="BT13" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU13" t="str"/>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" t="str">
@@ -43606,6 +43782,7 @@
       <x:c r="BT14" t="str">
         <x:v>false</x:v>
       </x:c>
+      <x:c r="BU14" t="str"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
@@ -43624,7 +43801,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad226df4586d4d02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3968b3ff70f04d19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct batch 04 read statuses
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R088f20caa81c4d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R79c228a70d0e482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R32ac521297054fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R1051e123e15c4ddd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Rd6933891c3d94d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Ree6cb4209d1f4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R2480683c407b4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R41c2cee264f74f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R564b5dae00024532"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rb62e65650a4b4772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R0fa3c7d61e984fbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R69289114541541b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R7052b95f5b0a490d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R25b09cb8c1fa4afe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="52" name="PapersTable" displayName="PapersTable" ref="A1:BR5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="PapersTable" displayName="PapersTable" ref="A1:BR5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="70">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -423,7 +423,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="53" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BM79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="57" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BM79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="65">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -496,7 +496,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="54" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CF67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="58" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CF67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="84">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -588,7 +588,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="55" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BU14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BU14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="73">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1313,7 +1313,7 @@
       <x:c r="BQ2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BR2" t="str"/>
+      <x:c r="BR2"/>
     </x:row>
     <x:row r="3" ht="150" customHeight="1">
       <x:c r="A3" t="str">
@@ -1489,7 +1489,7 @@
       <x:c r="BQ3" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BR3" t="str"/>
+      <x:c r="BR3"/>
     </x:row>
     <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" t="str">
@@ -1665,7 +1665,7 @@
       <x:c r="BQ4" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BR4" t="str"/>
+      <x:c r="BR4"/>
     </x:row>
     <x:row r="5" ht="150" customHeight="1">
       <x:c r="A5" t="str">
@@ -1841,7 +1841,7 @@
       <x:c r="BQ5" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BR5" t="str"/>
+      <x:c r="BR5"/>
     </x:row>
     <x:row r="6">
       <x:c r="AC6" s="7"/>
@@ -4854,7 +4854,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d56b28395454f48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5753606751f4e58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8150,7 +8150,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ed45e795c4b4da1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a7614ef9b646ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8501,7 +8501,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36fe4e66a443490e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8501099a1a4f77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9247,7 +9247,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe8d92f56e3b4a6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89abe657fca74772"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9667,7 +9667,7 @@
       <x:c r="BL2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM2" t="str"/>
+      <x:c r="BM2"/>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -9852,7 +9852,7 @@
       <x:c r="BL3" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM3" t="str"/>
+      <x:c r="BM3"/>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -10037,7 +10037,7 @@
       <x:c r="BL4" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM4" t="str"/>
+      <x:c r="BM4"/>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -10224,7 +10224,7 @@
       <x:c r="BL5" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM5" t="str"/>
+      <x:c r="BM5"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -10409,7 +10409,7 @@
       <x:c r="BL6" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM6" t="str"/>
+      <x:c r="BM6"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -10594,7 +10594,7 @@
       <x:c r="BL7" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM7" t="str"/>
+      <x:c r="BM7"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -10777,7 +10777,7 @@
       <x:c r="BL8" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM8" t="str"/>
+      <x:c r="BM8"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -10962,7 +10962,7 @@
       <x:c r="BL9" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM9" t="str"/>
+      <x:c r="BM9"/>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -11145,7 +11145,7 @@
       <x:c r="BL10" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM10" t="str"/>
+      <x:c r="BM10"/>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -11332,7 +11332,7 @@
       <x:c r="BL11" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM11" t="str"/>
+      <x:c r="BM11"/>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -11519,7 +11519,7 @@
       <x:c r="BL12" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM12" t="str"/>
+      <x:c r="BM12"/>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -11706,7 +11706,7 @@
       <x:c r="BL13" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM13" t="str"/>
+      <x:c r="BM13"/>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -11891,7 +11891,7 @@
       <x:c r="BL14" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM14" t="str"/>
+      <x:c r="BM14"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -12078,7 +12078,7 @@
       <x:c r="BL15" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM15" t="str"/>
+      <x:c r="BM15"/>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" t="str">
@@ -12261,7 +12261,7 @@
       <x:c r="BL16" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM16" t="str"/>
+      <x:c r="BM16"/>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -12444,7 +12444,7 @@
       <x:c r="BL17" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM17" t="str"/>
+      <x:c r="BM17"/>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -12627,7 +12627,7 @@
       <x:c r="BL18" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM18" t="str"/>
+      <x:c r="BM18"/>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -12812,7 +12812,7 @@
       <x:c r="BL19" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM19" t="str"/>
+      <x:c r="BM19"/>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -12995,7 +12995,7 @@
       <x:c r="BL20" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM20" t="str"/>
+      <x:c r="BM20"/>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -13180,7 +13180,7 @@
       <x:c r="BL21" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM21" t="str"/>
+      <x:c r="BM21"/>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -13365,7 +13365,7 @@
       <x:c r="BL22" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM22" t="str"/>
+      <x:c r="BM22"/>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -13550,7 +13550,7 @@
       <x:c r="BL23" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM23" t="str"/>
+      <x:c r="BM23"/>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -13735,7 +13735,7 @@
       <x:c r="BL24" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM24" t="str"/>
+      <x:c r="BM24"/>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -13918,7 +13918,7 @@
       <x:c r="BL25" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM25" t="str"/>
+      <x:c r="BM25"/>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -14103,7 +14103,7 @@
       <x:c r="BL26" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM26" t="str"/>
+      <x:c r="BM26"/>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -14288,7 +14288,7 @@
       <x:c r="BL27" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM27" t="str"/>
+      <x:c r="BM27"/>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -14473,7 +14473,7 @@
       <x:c r="BL28" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM28" t="str"/>
+      <x:c r="BM28"/>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -14658,7 +14658,7 @@
       <x:c r="BL29" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM29" t="str"/>
+      <x:c r="BM29"/>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -14843,7 +14843,7 @@
       <x:c r="BL30" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM30" t="str"/>
+      <x:c r="BM30"/>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -15028,7 +15028,7 @@
       <x:c r="BL31" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM31" t="str"/>
+      <x:c r="BM31"/>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -15213,7 +15213,7 @@
       <x:c r="BL32" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM32" t="str"/>
+      <x:c r="BM32"/>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -15398,7 +15398,7 @@
       <x:c r="BL33" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM33" t="str"/>
+      <x:c r="BM33"/>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -15583,7 +15583,7 @@
       <x:c r="BL34" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM34" t="str"/>
+      <x:c r="BM34"/>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -15768,7 +15768,7 @@
       <x:c r="BL35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM35" t="str"/>
+      <x:c r="BM35"/>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -15953,7 +15953,7 @@
       <x:c r="BL36" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM36" t="str"/>
+      <x:c r="BM36"/>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -16138,7 +16138,7 @@
       <x:c r="BL37" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM37" t="str"/>
+      <x:c r="BM37"/>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -16323,7 +16323,7 @@
       <x:c r="BL38" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM38" t="str"/>
+      <x:c r="BM38"/>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -16508,7 +16508,7 @@
       <x:c r="BL39" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM39" t="str"/>
+      <x:c r="BM39"/>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -16691,7 +16691,7 @@
       <x:c r="BL40" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM40" t="str"/>
+      <x:c r="BM40"/>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -16874,7 +16874,7 @@
       <x:c r="BL41" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM41" t="str"/>
+      <x:c r="BM41"/>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -17057,7 +17057,7 @@
       <x:c r="BL42" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM42" t="str"/>
+      <x:c r="BM42"/>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -17240,7 +17240,7 @@
       <x:c r="BL43" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM43" t="str"/>
+      <x:c r="BM43"/>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -17423,7 +17423,7 @@
       <x:c r="BL44" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM44" t="str"/>
+      <x:c r="BM44"/>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -17606,7 +17606,7 @@
       <x:c r="BL45" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM45" t="str"/>
+      <x:c r="BM45"/>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -17791,7 +17791,7 @@
       <x:c r="BL46" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM46" t="str"/>
+      <x:c r="BM46"/>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -17976,7 +17976,7 @@
       <x:c r="BL47" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM47" t="str"/>
+      <x:c r="BM47"/>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -18161,7 +18161,7 @@
       <x:c r="BL48" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM48" t="str"/>
+      <x:c r="BM48"/>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -18346,7 +18346,7 @@
       <x:c r="BL49" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM49" t="str"/>
+      <x:c r="BM49"/>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -18531,7 +18531,7 @@
       <x:c r="BL50" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM50" t="str"/>
+      <x:c r="BM50"/>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -18716,7 +18716,7 @@
       <x:c r="BL51" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM51" t="str"/>
+      <x:c r="BM51"/>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -18901,7 +18901,7 @@
       <x:c r="BL52" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM52" t="str"/>
+      <x:c r="BM52"/>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -19086,7 +19086,7 @@
       <x:c r="BL53" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM53" t="str"/>
+      <x:c r="BM53"/>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -19271,7 +19271,7 @@
       <x:c r="BL54" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM54" t="str"/>
+      <x:c r="BM54"/>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -19456,7 +19456,7 @@
       <x:c r="BL55" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM55" t="str"/>
+      <x:c r="BM55"/>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -19641,7 +19641,7 @@
       <x:c r="BL56" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM56" t="str"/>
+      <x:c r="BM56"/>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -19826,7 +19826,7 @@
       <x:c r="BL57" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM57" t="str"/>
+      <x:c r="BM57"/>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -20017,7 +20017,7 @@
       <x:c r="BL58" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM58" t="str"/>
+      <x:c r="BM58"/>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -20208,7 +20208,7 @@
       <x:c r="BL59" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM59" t="str"/>
+      <x:c r="BM59"/>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -20397,7 +20397,7 @@
       <x:c r="BL60" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM60" t="str"/>
+      <x:c r="BM60"/>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -20588,7 +20588,7 @@
       <x:c r="BL61" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM61" t="str"/>
+      <x:c r="BM61"/>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -20779,7 +20779,7 @@
       <x:c r="BL62" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM62" t="str"/>
+      <x:c r="BM62"/>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -20970,7 +20970,7 @@
       <x:c r="BL63" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM63" t="str"/>
+      <x:c r="BM63"/>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -21161,7 +21161,7 @@
       <x:c r="BL64" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM64" t="str"/>
+      <x:c r="BM64"/>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -21352,7 +21352,7 @@
       <x:c r="BL65" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM65" t="str"/>
+      <x:c r="BM65"/>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -21543,7 +21543,7 @@
       <x:c r="BL66" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM66" t="str"/>
+      <x:c r="BM66"/>
     </x:row>
     <x:row r="67" ht="58" customHeight="1">
       <x:c r="A67" t="str">
@@ -21734,7 +21734,7 @@
       <x:c r="BL67" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM67" t="str"/>
+      <x:c r="BM67"/>
     </x:row>
     <x:row r="68" ht="58" customHeight="1">
       <x:c r="A68" t="str">
@@ -21923,7 +21923,7 @@
       <x:c r="BL68" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM68" t="str"/>
+      <x:c r="BM68"/>
     </x:row>
     <x:row r="69" ht="58" customHeight="1">
       <x:c r="A69" t="str">
@@ -22114,7 +22114,7 @@
       <x:c r="BL69" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM69" t="str"/>
+      <x:c r="BM69"/>
     </x:row>
     <x:row r="70" ht="58" customHeight="1">
       <x:c r="A70" t="str">
@@ -22305,7 +22305,7 @@
       <x:c r="BL70" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM70" t="str"/>
+      <x:c r="BM70"/>
     </x:row>
     <x:row r="71" ht="58" customHeight="1">
       <x:c r="A71" t="str">
@@ -22496,7 +22496,7 @@
       <x:c r="BL71" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM71" t="str"/>
+      <x:c r="BM71"/>
     </x:row>
     <x:row r="72" ht="58" customHeight="1">
       <x:c r="A72" t="str">
@@ -22687,7 +22687,7 @@
       <x:c r="BL72" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM72" t="str"/>
+      <x:c r="BM72"/>
     </x:row>
     <x:row r="73" ht="58" customHeight="1">
       <x:c r="A73" t="str">
@@ -22878,7 +22878,7 @@
       <x:c r="BL73" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM73" t="str"/>
+      <x:c r="BM73"/>
     </x:row>
     <x:row r="74" ht="58" customHeight="1">
       <x:c r="A74" t="str">
@@ -23069,7 +23069,7 @@
       <x:c r="BL74" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM74" t="str"/>
+      <x:c r="BM74"/>
     </x:row>
     <x:row r="75" ht="58" customHeight="1">
       <x:c r="A75" t="str">
@@ -23260,7 +23260,7 @@
       <x:c r="BL75" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM75" t="str"/>
+      <x:c r="BM75"/>
     </x:row>
     <x:row r="76" ht="58" customHeight="1">
       <x:c r="A76" t="str">
@@ -23447,7 +23447,7 @@
       <x:c r="BL76" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM76" t="str"/>
+      <x:c r="BM76"/>
     </x:row>
     <x:row r="77" ht="58" customHeight="1">
       <x:c r="A77" t="str">
@@ -23634,7 +23634,7 @@
       <x:c r="BL77" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM77" t="str"/>
+      <x:c r="BM77"/>
     </x:row>
     <x:row r="78" ht="58" customHeight="1">
       <x:c r="A78" t="str">
@@ -23821,7 +23821,7 @@
       <x:c r="BL78" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM78" t="str"/>
+      <x:c r="BM78"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
@@ -24014,7 +24014,7 @@
       <x:c r="BL79" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BM79" t="str"/>
+      <x:c r="BM79"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="5">
@@ -24036,7 +24036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95465e0d0a6042d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2550f3c675ef4ff1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24591,7 +24591,7 @@
       <x:c r="CE2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF2" t="str"/>
+      <x:c r="CF2"/>
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" t="str">
@@ -24833,7 +24833,7 @@
       <x:c r="CE3" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF3" t="str"/>
+      <x:c r="CF3"/>
     </x:row>
     <x:row r="4" ht="58" customHeight="1">
       <x:c r="A4" t="str">
@@ -25075,7 +25075,7 @@
       <x:c r="CE4" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF4" t="str"/>
+      <x:c r="CF4"/>
     </x:row>
     <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" t="str">
@@ -25317,7 +25317,7 @@
       <x:c r="CE5" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF5" t="str"/>
+      <x:c r="CF5"/>
     </x:row>
     <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" t="str">
@@ -25559,7 +25559,7 @@
       <x:c r="CE6" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF6" t="str"/>
+      <x:c r="CF6"/>
     </x:row>
     <x:row r="7" ht="58" customHeight="1">
       <x:c r="A7" t="str">
@@ -25801,7 +25801,7 @@
       <x:c r="CE7" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF7" t="str"/>
+      <x:c r="CF7"/>
     </x:row>
     <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" t="str">
@@ -26043,7 +26043,7 @@
       <x:c r="CE8" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF8" t="str"/>
+      <x:c r="CF8"/>
     </x:row>
     <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" t="str">
@@ -26283,7 +26283,7 @@
       <x:c r="CE9" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF9" t="str"/>
+      <x:c r="CF9"/>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" t="str">
@@ -26529,7 +26529,7 @@
       <x:c r="CE10" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF10" t="str"/>
+      <x:c r="CF10"/>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" t="str">
@@ -26777,7 +26777,7 @@
       <x:c r="CE11" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF11" t="str"/>
+      <x:c r="CF11"/>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" t="str">
@@ -27025,7 +27025,7 @@
       <x:c r="CE12" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF12" t="str"/>
+      <x:c r="CF12"/>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" t="str">
@@ -27273,7 +27273,7 @@
       <x:c r="CE13" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF13" t="str"/>
+      <x:c r="CF13"/>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" t="str">
@@ -27521,7 +27521,7 @@
       <x:c r="CE14" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF14" t="str"/>
+      <x:c r="CF14"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" t="str">
@@ -27769,7 +27769,7 @@
       <x:c r="CE15" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF15" t="str"/>
+      <x:c r="CF15"/>
     </x:row>
     <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" t="str">
@@ -28015,7 +28015,7 @@
       <x:c r="CE16" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF16" t="str"/>
+      <x:c r="CF16"/>
     </x:row>
     <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" t="str">
@@ -28263,7 +28263,7 @@
       <x:c r="CE17" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF17" t="str"/>
+      <x:c r="CF17"/>
     </x:row>
     <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" t="str">
@@ -28511,7 +28511,7 @@
       <x:c r="CE18" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF18" t="str"/>
+      <x:c r="CF18"/>
     </x:row>
     <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" t="str">
@@ -28759,7 +28759,7 @@
       <x:c r="CE19" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF19" t="str"/>
+      <x:c r="CF19"/>
     </x:row>
     <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" t="str">
@@ -29007,7 +29007,7 @@
       <x:c r="CE20" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF20" t="str"/>
+      <x:c r="CF20"/>
     </x:row>
     <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" t="str">
@@ -29257,7 +29257,7 @@
       <x:c r="CE21" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF21" t="str"/>
+      <x:c r="CF21"/>
     </x:row>
     <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" t="str">
@@ -29507,7 +29507,7 @@
       <x:c r="CE22" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF22" t="str"/>
+      <x:c r="CF22"/>
     </x:row>
     <x:row r="23" ht="58" customHeight="1">
       <x:c r="A23" t="str">
@@ -29757,7 +29757,7 @@
       <x:c r="CE23" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF23" t="str"/>
+      <x:c r="CF23"/>
     </x:row>
     <x:row r="24" ht="58" customHeight="1">
       <x:c r="A24" t="str">
@@ -30007,7 +30007,7 @@
       <x:c r="CE24" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF24" t="str"/>
+      <x:c r="CF24"/>
     </x:row>
     <x:row r="25" ht="58" customHeight="1">
       <x:c r="A25" t="str">
@@ -30257,7 +30257,7 @@
       <x:c r="CE25" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF25" t="str"/>
+      <x:c r="CF25"/>
     </x:row>
     <x:row r="26" ht="58" customHeight="1">
       <x:c r="A26" t="str">
@@ -30507,7 +30507,7 @@
       <x:c r="CE26" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF26" t="str"/>
+      <x:c r="CF26"/>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
       <x:c r="A27" t="str">
@@ -30757,7 +30757,7 @@
       <x:c r="CE27" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF27" t="str"/>
+      <x:c r="CF27"/>
     </x:row>
     <x:row r="28" ht="58" customHeight="1">
       <x:c r="A28" t="str">
@@ -31007,7 +31007,7 @@
       <x:c r="CE28" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF28" t="str"/>
+      <x:c r="CF28"/>
     </x:row>
     <x:row r="29" ht="58" customHeight="1">
       <x:c r="A29" t="str">
@@ -31257,7 +31257,7 @@
       <x:c r="CE29" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF29" t="str"/>
+      <x:c r="CF29"/>
     </x:row>
     <x:row r="30" ht="58" customHeight="1">
       <x:c r="A30" t="str">
@@ -31507,7 +31507,7 @@
       <x:c r="CE30" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF30" t="str"/>
+      <x:c r="CF30"/>
     </x:row>
     <x:row r="31" ht="58" customHeight="1">
       <x:c r="A31" t="str">
@@ -31757,7 +31757,7 @@
       <x:c r="CE31" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF31" t="str"/>
+      <x:c r="CF31"/>
     </x:row>
     <x:row r="32" ht="58" customHeight="1">
       <x:c r="A32" t="str">
@@ -32007,7 +32007,7 @@
       <x:c r="CE32" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF32" t="str"/>
+      <x:c r="CF32"/>
     </x:row>
     <x:row r="33" ht="58" customHeight="1">
       <x:c r="A33" t="str">
@@ -32257,7 +32257,7 @@
       <x:c r="CE33" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF33" t="str"/>
+      <x:c r="CF33"/>
     </x:row>
     <x:row r="34" ht="58" customHeight="1">
       <x:c r="A34" t="str">
@@ -32507,7 +32507,7 @@
       <x:c r="CE34" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF34" t="str"/>
+      <x:c r="CF34"/>
     </x:row>
     <x:row r="35" ht="58" customHeight="1">
       <x:c r="A35" t="str">
@@ -32757,7 +32757,7 @@
       <x:c r="CE35" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF35" t="str"/>
+      <x:c r="CF35"/>
     </x:row>
     <x:row r="36" ht="58" customHeight="1">
       <x:c r="A36" t="str">
@@ -33007,7 +33007,7 @@
       <x:c r="CE36" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF36" t="str"/>
+      <x:c r="CF36"/>
     </x:row>
     <x:row r="37" ht="58" customHeight="1">
       <x:c r="A37" t="str">
@@ -33257,7 +33257,7 @@
       <x:c r="CE37" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF37" t="str"/>
+      <x:c r="CF37"/>
     </x:row>
     <x:row r="38" ht="58" customHeight="1">
       <x:c r="A38" t="str">
@@ -33507,7 +33507,7 @@
       <x:c r="CE38" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF38" t="str"/>
+      <x:c r="CF38"/>
     </x:row>
     <x:row r="39" ht="58" customHeight="1">
       <x:c r="A39" t="str">
@@ -33757,7 +33757,7 @@
       <x:c r="CE39" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF39" t="str"/>
+      <x:c r="CF39"/>
     </x:row>
     <x:row r="40" ht="58" customHeight="1">
       <x:c r="A40" t="str">
@@ -34007,7 +34007,7 @@
       <x:c r="CE40" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF40" t="str"/>
+      <x:c r="CF40"/>
     </x:row>
     <x:row r="41" ht="58" customHeight="1">
       <x:c r="A41" t="str">
@@ -34257,7 +34257,7 @@
       <x:c r="CE41" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF41" t="str"/>
+      <x:c r="CF41"/>
     </x:row>
     <x:row r="42" ht="58" customHeight="1">
       <x:c r="A42" t="str">
@@ -34507,7 +34507,7 @@
       <x:c r="CE42" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF42" t="str"/>
+      <x:c r="CF42"/>
     </x:row>
     <x:row r="43" ht="58" customHeight="1">
       <x:c r="A43" t="str">
@@ -34757,7 +34757,7 @@
       <x:c r="CE43" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF43" t="str"/>
+      <x:c r="CF43"/>
     </x:row>
     <x:row r="44" ht="58" customHeight="1">
       <x:c r="A44" t="str">
@@ -35007,7 +35007,7 @@
       <x:c r="CE44" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF44" t="str"/>
+      <x:c r="CF44"/>
     </x:row>
     <x:row r="45" ht="58" customHeight="1">
       <x:c r="A45" t="str">
@@ -35257,7 +35257,7 @@
       <x:c r="CE45" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF45" t="str"/>
+      <x:c r="CF45"/>
     </x:row>
     <x:row r="46" ht="58" customHeight="1">
       <x:c r="A46" t="str">
@@ -35507,7 +35507,7 @@
       <x:c r="CE46" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF46" t="str"/>
+      <x:c r="CF46"/>
     </x:row>
     <x:row r="47" ht="58" customHeight="1">
       <x:c r="A47" t="str">
@@ -35757,7 +35757,7 @@
       <x:c r="CE47" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF47" t="str"/>
+      <x:c r="CF47"/>
     </x:row>
     <x:row r="48" ht="58" customHeight="1">
       <x:c r="A48" t="str">
@@ -36007,7 +36007,7 @@
       <x:c r="CE48" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF48" t="str"/>
+      <x:c r="CF48"/>
     </x:row>
     <x:row r="49" ht="58" customHeight="1">
       <x:c r="A49" t="str">
@@ -36257,7 +36257,7 @@
       <x:c r="CE49" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF49" t="str"/>
+      <x:c r="CF49"/>
     </x:row>
     <x:row r="50" ht="58" customHeight="1">
       <x:c r="A50" t="str">
@@ -36507,7 +36507,7 @@
       <x:c r="CE50" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF50" t="str"/>
+      <x:c r="CF50"/>
     </x:row>
     <x:row r="51" ht="58" customHeight="1">
       <x:c r="A51" t="str">
@@ -36757,7 +36757,7 @@
       <x:c r="CE51" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF51" t="str"/>
+      <x:c r="CF51"/>
     </x:row>
     <x:row r="52" ht="58" customHeight="1">
       <x:c r="A52" t="str">
@@ -37007,7 +37007,7 @@
       <x:c r="CE52" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF52" t="str"/>
+      <x:c r="CF52"/>
     </x:row>
     <x:row r="53" ht="58" customHeight="1">
       <x:c r="A53" t="str">
@@ -37257,7 +37257,7 @@
       <x:c r="CE53" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF53" t="str"/>
+      <x:c r="CF53"/>
     </x:row>
     <x:row r="54" ht="58" customHeight="1">
       <x:c r="A54" t="str">
@@ -37507,7 +37507,7 @@
       <x:c r="CE54" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF54" t="str"/>
+      <x:c r="CF54"/>
     </x:row>
     <x:row r="55" ht="58" customHeight="1">
       <x:c r="A55" t="str">
@@ -37757,7 +37757,7 @@
       <x:c r="CE55" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF55" t="str"/>
+      <x:c r="CF55"/>
     </x:row>
     <x:row r="56" ht="58" customHeight="1">
       <x:c r="A56" t="str">
@@ -38007,7 +38007,7 @@
       <x:c r="CE56" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF56" t="str"/>
+      <x:c r="CF56"/>
     </x:row>
     <x:row r="57" ht="58" customHeight="1">
       <x:c r="A57" t="str">
@@ -38257,7 +38257,7 @@
       <x:c r="CE57" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF57" t="str"/>
+      <x:c r="CF57"/>
     </x:row>
     <x:row r="58" ht="58" customHeight="1">
       <x:c r="A58" t="str">
@@ -38507,7 +38507,7 @@
       <x:c r="CE58" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF58" t="str"/>
+      <x:c r="CF58"/>
     </x:row>
     <x:row r="59" ht="58" customHeight="1">
       <x:c r="A59" t="str">
@@ -38757,7 +38757,7 @@
       <x:c r="CE59" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF59" t="str"/>
+      <x:c r="CF59"/>
     </x:row>
     <x:row r="60" ht="58" customHeight="1">
       <x:c r="A60" t="str">
@@ -39007,7 +39007,7 @@
       <x:c r="CE60" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF60" t="str"/>
+      <x:c r="CF60"/>
     </x:row>
     <x:row r="61" ht="58" customHeight="1">
       <x:c r="A61" t="str">
@@ -39257,7 +39257,7 @@
       <x:c r="CE61" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF61" t="str"/>
+      <x:c r="CF61"/>
     </x:row>
     <x:row r="62" ht="58" customHeight="1">
       <x:c r="A62" t="str">
@@ -39507,7 +39507,7 @@
       <x:c r="CE62" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF62" t="str"/>
+      <x:c r="CF62"/>
     </x:row>
     <x:row r="63" ht="58" customHeight="1">
       <x:c r="A63" t="str">
@@ -39757,7 +39757,7 @@
       <x:c r="CE63" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF63" t="str"/>
+      <x:c r="CF63"/>
     </x:row>
     <x:row r="64" ht="58" customHeight="1">
       <x:c r="A64" t="str">
@@ -40007,7 +40007,7 @@
       <x:c r="CE64" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF64" t="str"/>
+      <x:c r="CF64"/>
     </x:row>
     <x:row r="65" ht="58" customHeight="1">
       <x:c r="A65" t="str">
@@ -40257,7 +40257,7 @@
       <x:c r="CE65" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF65" t="str"/>
+      <x:c r="CF65"/>
     </x:row>
     <x:row r="66" ht="58" customHeight="1">
       <x:c r="A66" t="str">
@@ -40507,7 +40507,7 @@
       <x:c r="CE66" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF66" t="str"/>
+      <x:c r="CF66"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" t="str">
@@ -40757,7 +40757,7 @@
       <x:c r="CE67" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="CF67" t="str"/>
+      <x:c r="CF67"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="10">
@@ -40794,7 +40794,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5ea64be2c924395"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961ca2f95ee544b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41278,7 +41278,7 @@
       <x:c r="BT2" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU2" t="str"/>
+      <x:c r="BU2"/>
     </x:row>
     <x:row r="3" ht="62" customHeight="1">
       <x:c r="A3" t="str">
@@ -41495,7 +41495,7 @@
       <x:c r="BT3" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU3" t="str"/>
+      <x:c r="BU3"/>
     </x:row>
     <x:row r="4" ht="62" customHeight="1">
       <x:c r="A4" t="str">
@@ -41712,7 +41712,7 @@
       <x:c r="BT4" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU4" t="str"/>
+      <x:c r="BU4"/>
     </x:row>
     <x:row r="5" ht="62" customHeight="1">
       <x:c r="A5" t="str">
@@ -41929,7 +41929,7 @@
       <x:c r="BT5" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU5" t="str"/>
+      <x:c r="BU5"/>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
       <x:c r="A6" t="str">
@@ -42146,7 +42146,7 @@
       <x:c r="BT6" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU6" t="str"/>
+      <x:c r="BU6"/>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
       <x:c r="A7" t="str">
@@ -42363,7 +42363,7 @@
       <x:c r="BT7" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU7" t="str"/>
+      <x:c r="BU7"/>
     </x:row>
     <x:row r="8" ht="62" customHeight="1">
       <x:c r="A8" t="str">
@@ -42580,7 +42580,7 @@
       <x:c r="BT8" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU8" t="str"/>
+      <x:c r="BU8"/>
     </x:row>
     <x:row r="9" ht="62" customHeight="1">
       <x:c r="A9" t="str">
@@ -42797,7 +42797,7 @@
       <x:c r="BT9" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU9" t="str"/>
+      <x:c r="BU9"/>
     </x:row>
     <x:row r="10" ht="62" customHeight="1">
       <x:c r="A10" t="str">
@@ -43014,7 +43014,7 @@
       <x:c r="BT10" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU10" t="str"/>
+      <x:c r="BU10"/>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
       <x:c r="A11" t="str">
@@ -43209,7 +43209,7 @@
       <x:c r="BT11" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU11" t="str"/>
+      <x:c r="BU11"/>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" t="str">
@@ -43400,7 +43400,7 @@
       <x:c r="BT12" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU12" t="str"/>
+      <x:c r="BU12"/>
     </x:row>
     <x:row r="13" ht="62" customHeight="1">
       <x:c r="A13" t="str">
@@ -43591,7 +43591,7 @@
       <x:c r="BT13" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU13" t="str"/>
+      <x:c r="BU13"/>
     </x:row>
     <x:row r="14" ht="62" customHeight="1">
       <x:c r="A14" t="str">
@@ -43782,7 +43782,7 @@
       <x:c r="BT14" t="str">
         <x:v>false</x:v>
       </x:c>
-      <x:c r="BU14" t="str"/>
+      <x:c r="BU14"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
@@ -43801,7 +43801,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3968b3ff70f04d19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39291e5246964ba3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add and deep-enrich SayCan
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R41c2cee264f74f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R564b5dae00024532"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rb62e65650a4b4772"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R0fa3c7d61e984fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R69289114541541b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R7052b95f5b0a490d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R25b09cb8c1fa4afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R86f01c6dad0e4415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rb991b7fdee134239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rdd3ba6f2361044fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rfc90709385e342e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Ra1faf7c021804116"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc96f7f93fef2443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rfd09c41558954595"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="56" name="PapersTable" displayName="PapersTable" ref="A1:BR5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="60" name="PapersTable" displayName="PapersTable" ref="A1:BR6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="70">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -588,7 +588,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="59" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BU14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="61" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:BU15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="73">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1276,7 +1276,7 @@
       <x:c r="BD2" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BE2" t="str"/>
+      <x:c r="BE2"/>
       <x:c r="BF2" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -1452,7 +1452,7 @@
       <x:c r="BD3" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BE3" t="str"/>
+      <x:c r="BE3"/>
       <x:c r="BF3" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -1628,7 +1628,7 @@
       <x:c r="BD4" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BE4" t="str"/>
+      <x:c r="BE4"/>
       <x:c r="BF4" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -1804,7 +1804,7 @@
       <x:c r="BD5" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BE5" t="str"/>
+      <x:c r="BE5"/>
       <x:c r="BF5" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -1844,7 +1844,216 @@
       <x:c r="BR5"/>
     </x:row>
     <x:row r="6">
-      <x:c r="AC6" s="7"/>
+      <x:c r="A6" t="str">
+        <x:v>P0005</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Do As I Can, Not As I Say: Grounding Language in Robotic Affordances</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>CoRL</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Not CCF A</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>VLA / Robot Manipulation / Language Grounding</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Language-conditioned planning / affordance grounding</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>LLMs lack embodiment and execution grounding for long-horizon robot instructions.</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Text-only planning can propose infeasible skills; prior systems do not jointly score usefulness and current-state feasibility.</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>SayCan multiplies LLM skill usefulness with affordance/value feasibility and replans after every executed skill.</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Interpretable language-conditioned skill composition grounded by learned value functions; 101-task real/mock kitchen evaluation.</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Everyday Robots mobile manipulator; two-finger gripper</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>Single arm</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>RGB observation plus language instruction and robot state</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>Skill-level pick/place/navigation/drawer actions; low-level 7-DoF arm and gripper control</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>68k demonstrations + 12k successful autonomous episodes (official blog/project report); SayCan dataset v0</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
+        <x:v>101 natural-language instructions; Mock Kitchen and Real Kitchen; 7 instruction families</x:v>
+      </x:c>
+      <x:c r="S6" t="str">
+        <x:v>https://research.google/pubs/do-as-i-can-not-as-i-say-grounding-language-in-robotic-affordances/</x:v>
+      </x:c>
+      <x:c r="T6" t="str">
+        <x:v>https://say-can.github.io/</x:v>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>Partial - official tabletop simulation released</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
+        <x:v>https://github.com/google-research/google-research/tree/master/saycan</x:v>
+      </x:c>
+      <x:c r="W6" t="str">
+        <x:v>Not released as complete PaLM/Everyday Robots stack</x:v>
+      </x:c>
+      <x:c r="X6" t="str">
+        <x:v>Partial - SayCan dataset v0; full training dump not confirmed</x:v>
+      </x:c>
+      <x:c r="Y6" t="str">
+        <x:v>Official tabletop environment available; original kitchen stack not fully reproducible</x:v>
+      </x:c>
+      <x:c r="Z6" t="str">
+        <x:v>L1</x:v>
+      </x:c>
+      <x:c r="AA6" t="str">
+        <x:v>L1 / foundational; direct inspiration for feasibility scoring, bimanual joint affordance and recovery</x:v>
+      </x:c>
+      <x:c r="AB6" t="str">
+        <x:v>Full-text Evidence A. 551 skills, 7 families, 17 objects; Table 2 Mock 84/74 and Real 81/60.</x:v>
+      </x:c>
+      <x:c r="AC6" s="7" t="str">
+        <x:v>2026-09-22</x:v>
+      </x:c>
+      <x:c r="AD6" t="str">
+        <x:v>VLA</x:v>
+      </x:c>
+      <x:c r="AE6" t="str">
+        <x:v>02_Papers/01_VLA/SayCan.md</x:v>
+      </x:c>
+      <x:c r="AF6" t="n">
+        <x:v>523</x:v>
+      </x:c>
+      <x:c r="AG6" t="str">
+        <x:v>OpenAlex</x:v>
+      </x:c>
+      <x:c r="AH6" t="str">
+        <x:v>2026-09-22</x:v>
+      </x:c>
+      <x:c r="AI6" t="str">
+        <x:v>LLMs have semantic knowledge but no embodiment or current-state grounding.</x:v>
+      </x:c>
+      <x:c r="AJ6" t="str">
+        <x:v>Long-horizon abstract instructions require both useful decomposition and physically feasible execution.</x:v>
+      </x:c>
+      <x:c r="AK6" t="str">
+        <x:v>SayCan: p(cπ|s,ℓπ) × p(ℓπ|i), receding-horizon skill selection.</x:v>
+      </x:c>
+      <x:c r="AL6" t="str">
+        <x:v>101 instructions across 7 families; mock and real office kitchens; 15 objects/5 locations.</x:v>
+      </x:c>
+      <x:c r="AM6" t="str">
+        <x:v>No VF; Generative; FLAN-SayCan; BC NL; BC USE; PaLM scale ablations.</x:v>
+      </x:c>
+      <x:c r="AN6" t="str">
+        <x:v>Affordance-grounded interpretable LLM planning over pretrained skills.</x:v>
+      </x:c>
+      <x:c r="AO6" t="str">
+        <x:v>Everyday Robots mobile manipulator; 551 candidate skills; PaLM 540B; Mock/Real Kitchen.</x:v>
+      </x:c>
+      <x:c r="AP6" t="str">
+        <x:v>Mock 84% plan / 74% execute; Real 81% / 60%; FLAN 70% / 61%; drawer 100% / 33%.</x:v>
+      </x:c>
+      <x:c r="AQ6" t="str">
+        <x:v>Fixed skill library; value-function/current-step feedback; low-level execution and recovery remain limited.</x:v>
+      </x:c>
+      <x:c r="AR6" t="str">
+        <x:v>Open-ended skill synthesis, continuous/contact grounding, closed-loop verification/recovery, bimanual joint feasibility.</x:v>
+      </x:c>
+      <x:c r="AS6" t="str">
+        <x:v>Use dual language-usefulness and joint-arm feasibility scoring; add post-action verification and replanning for NERO.</x:v>
+      </x:c>
+      <x:c r="AT6" t="str">
+        <x:v>VLA; Robot Manipulation; Language Grounding; Affordance; Long-horizon; Planning; RL; IL; Sim2Real</x:v>
+      </x:c>
+      <x:c r="AU6" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="AV6" t="str">
+        <x:v>Joint-affordance SayCan; VLA feasibility veto; failure-aware receding-horizon recovery; affordance-calibrated sim2real library.</x:v>
+      </x:c>
+      <x:c r="AW6" t="str">
+        <x:v>No VF, Generative, BC NL/USE, PaLM 8B/62B/540B, FLAN 137B; drawer/CoT/multilingual appendices.</x:v>
+      </x:c>
+      <x:c r="AX6" t="str">
+        <x:v>Plan-execute gap; wrong object/negation; drawer manipulation and incomplete close; embodiment-specific failures.</x:v>
+      </x:c>
+      <x:c r="AY6" t="str">
+        <x:v>OpenAlex Work W4224912544</x:v>
+      </x:c>
+      <x:c r="AZ6" t="str">
+        <x:v>Google Research publication; arXiv HTML 2204.01691; CoRL/PMLR; say-can.github.io; Google Research blog; official google-research/saycan</x:v>
+      </x:c>
+      <x:c r="BA6" t="str">
+        <x:v>A-Upgraded</x:v>
+      </x:c>
+      <x:c r="BB6" t="str">
+        <x:v>Available - Verified</x:v>
+      </x:c>
+      <x:c r="BC6" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BD6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BE6" t="str">
+        <x:v>https://arxiv.org/html/2204.01691</x:v>
+      </x:c>
+      <x:c r="BF6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BG6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BH6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BI6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BJ6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BK6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BL6" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BM6" t="str">
+        <x:v>OpenAlex matched</x:v>
+      </x:c>
+      <x:c r="BN6" t="str">
+        <x:v>Verified - 10.48550/arXiv.2204.01691</x:v>
+      </x:c>
+      <x:c r="BO6" t="str">
+        <x:v>Verified - 2204.01691</x:v>
+      </x:c>
+      <x:c r="BP6" t="str">
+        <x:v>Completed - Full text read</x:v>
+      </x:c>
+      <x:c r="BQ6" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="BR6" t="str">
+        <x:v>Completed-A</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="AC7" s="7"/>
@@ -4854,7 +5063,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5753606751f4e58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8b9cc21c0e4685"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8150,7 +8359,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a7614ef9b646ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24875c2dbfc745b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8501,7 +8710,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8501099a1a4f77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae14747bf124552"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9247,7 +9456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89abe657fca74772"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148d6e9fc32646c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24036,7 +24245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2550f3c675ef4ff1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref9e2238cf614bf0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -40794,7 +41003,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R961ca2f95ee544b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1420b6b070443d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41241,7 +41450,7 @@
       <x:c r="BG2" t="str">
         <x:v>Multiple real-world setups are shown; exact hardware inventory not extracted at abstract/project level</x:v>
       </x:c>
-      <x:c r="BH2" t="str"/>
+      <x:c r="BH2"/>
       <x:c r="BI2" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -41458,7 +41667,7 @@
       <x:c r="BG3" t="str">
         <x:v>Dual robot arms; exact platform pending full-paper check</x:v>
       </x:c>
-      <x:c r="BH3" t="str"/>
+      <x:c r="BH3"/>
       <x:c r="BI3" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -41675,7 +41884,7 @@
       <x:c r="BG4" t="str">
         <x:v>Bimanual gripper system; exact model pending full-paper check</x:v>
       </x:c>
-      <x:c r="BH4" t="str"/>
+      <x:c r="BH4"/>
       <x:c r="BI4" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -41892,7 +42101,7 @@
       <x:c r="BG5" t="str">
         <x:v>Dexterous robotic hand</x:v>
       </x:c>
-      <x:c r="BH5" t="str"/>
+      <x:c r="BH5"/>
       <x:c r="BI5" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -42109,7 +42318,7 @@
       <x:c r="BG6" t="str">
         <x:v>Simulation plus real-world replication</x:v>
       </x:c>
-      <x:c r="BH6" t="str"/>
+      <x:c r="BH6"/>
       <x:c r="BI6" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -42326,7 +42535,7 @@
       <x:c r="BG7" t="str">
         <x:v>Dual robot arms; exact model pending full-paper check</x:v>
       </x:c>
-      <x:c r="BH7" t="str"/>
+      <x:c r="BH7"/>
       <x:c r="BI7" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -42543,7 +42752,7 @@
       <x:c r="BG8" t="str">
         <x:v>Robot arm with visuotactile end effector</x:v>
       </x:c>
-      <x:c r="BH8" t="str"/>
+      <x:c r="BH8"/>
       <x:c r="BI8" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -42760,7 +42969,7 @@
       <x:c r="BG9" t="str">
         <x:v>Multiple robotic arms</x:v>
       </x:c>
-      <x:c r="BH9" t="str"/>
+      <x:c r="BH9"/>
       <x:c r="BI9" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -42977,7 +43186,7 @@
       <x:c r="BG10" t="str">
         <x:v>Multiple hand geometries</x:v>
       </x:c>
-      <x:c r="BH10" t="str"/>
+      <x:c r="BH10"/>
       <x:c r="BI10" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -43172,7 +43381,7 @@
       <x:c r="BG11" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BH11" t="str"/>
+      <x:c r="BH11"/>
       <x:c r="BI11" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -43363,7 +43572,7 @@
       <x:c r="BG12" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BH12" t="str"/>
+      <x:c r="BH12"/>
       <x:c r="BI12" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -43554,7 +43763,7 @@
       <x:c r="BG13" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BH13" t="str"/>
+      <x:c r="BH13"/>
       <x:c r="BI13" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -43745,7 +43954,7 @@
       <x:c r="BG14" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BH14" t="str"/>
+      <x:c r="BH14"/>
       <x:c r="BI14" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -43783,6 +43992,227 @@
         <x:v>false</x:v>
       </x:c>
       <x:c r="BU14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>R014</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Do As I Can, Not As I Say: Grounding Language in Robotic Affordances</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Michael Ahn et al.</x:v>
+      </x:c>
+      <x:c r="D15" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>CoRL</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Robotics Core Venue</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Full Conference Paper; PMLR 205</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Not CCF A</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>VLA / Robot Manipulation / Language Grounding</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Language-conditioned planning / affordance grounding</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>VLA; Affordance; Long-horizon; Planning; Robot Learning</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>LLMs lack embodiment and execution grounding.</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>Multiplicative language-usefulness and affordance-feasibility scoring over skills.</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>Say + Can; receding-horizon selection.</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>https://research.google/pubs/do-as-i-can-not-as-i-say-grounding-language-in-robotic-affordances/</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>https://say-can.github.io/</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>https://github.com/google-research/google-research/tree/master/saycan</x:v>
+      </x:c>
+      <x:c r="R15" t="str">
+        <x:v>Partial - official tabletop simulation</x:v>
+      </x:c>
+      <x:c r="S15" t="str">
+        <x:v>Not released as complete original stack</x:v>
+      </x:c>
+      <x:c r="T15" t="str">
+        <x:v>SayCan dataset v0; 68k demos/12k successful episodes reported by official sources</x:v>
+      </x:c>
+      <x:c r="U15" t="str">
+        <x:v>Everyday Robots mobile manipulator</x:v>
+      </x:c>
+      <x:c r="V15" t="str">
+        <x:v>Single arm / two-finger gripper</x:v>
+      </x:c>
+      <x:c r="W15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X15" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="Y15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z15" t="str">
+        <x:v>Official full paper, project page, PMLR and code entry verified</x:v>
+      </x:c>
+      <x:c r="AA15" t="str">
+        <x:v>2026-09-22</x:v>
+      </x:c>
+      <x:c r="AB15" t="str">
+        <x:v>Full-text Evidence A; Table 2: Mock 84/74, Real 81/60; 551 skills, 7 families, 17 objects.</x:v>
+      </x:c>
+      <x:c r="AC15" t="str">
+        <x:v>02_Papers/01_VLA/SayCan.md</x:v>
+      </x:c>
+      <x:c r="AD15" t="str">
+        <x:v>Robotics Core / VLA</x:v>
+      </x:c>
+      <x:c r="AE15" t="str">
+        <x:v>Google Research; arXiv HTML; CoRL/PMLR; SayCan project page; official repository</x:v>
+      </x:c>
+      <x:c r="AF15" t="str">
+        <x:v>Full paper + appendices</x:v>
+      </x:c>
+      <x:c r="AG15" t="str">
+        <x:v>101 instructions; mock and real office kitchens; 7 families</x:v>
+      </x:c>
+      <x:c r="AH15" t="str">
+        <x:v>Feasibility scoring, joint-arm affordance and verification/replanning inspirations</x:v>
+      </x:c>
+      <x:c r="AI15" t="str">
+        <x:v>Current CCF check: no CCF-A assignment recorded</x:v>
+      </x:c>
+      <x:c r="AJ15" t="str">
+        <x:v>VLA</x:v>
+      </x:c>
+      <x:c r="AK15" t="n">
+        <x:v>523</x:v>
+      </x:c>
+      <x:c r="AL15" t="str">
+        <x:v>OpenAlex</x:v>
+      </x:c>
+      <x:c r="AM15" t="str">
+        <x:v>2026-09-22</x:v>
+      </x:c>
+      <x:c r="AN15" t="str">
+        <x:v>LLMs have semantic knowledge but no embodiment grounding.</x:v>
+      </x:c>
+      <x:c r="AO15" t="str">
+        <x:v>Useful decomposition and feasible execution were not jointly scored.</x:v>
+      </x:c>
+      <x:c r="AP15" t="str">
+        <x:v>SayCan p(cπ|s,ℓπ) × p(ℓπ|i), skill-level receding horizon.</x:v>
+      </x:c>
+      <x:c r="AQ15" t="str">
+        <x:v>101 instructions, 7 families, mock/real kitchens.</x:v>
+      </x:c>
+      <x:c r="AR15" t="str">
+        <x:v>No VF; Generative; FLAN-SayCan; BC NL/USE.</x:v>
+      </x:c>
+      <x:c r="AS15" t="str">
+        <x:v>Interpretable grounded skill composition.</x:v>
+      </x:c>
+      <x:c r="AT15" t="str">
+        <x:v>Mobile manipulator, PaLM 540B, 551 skills.</x:v>
+      </x:c>
+      <x:c r="AU15" t="str">
+        <x:v>Mock 84/74; Real 81/60; FLAN 70/61; drawer 100/33.</x:v>
+      </x:c>
+      <x:c r="AV15" t="str">
+        <x:v>Fixed skill library, current-step value feedback, execution/recovery gaps.</x:v>
+      </x:c>
+      <x:c r="AW15" t="str">
+        <x:v>Skill synthesis, contact-level grounding, recovery, bimanual joint feasibility.</x:v>
+      </x:c>
+      <x:c r="AX15" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="AY15" t="str">
+        <x:v>Joint affordance; VLA feasibility veto; recovery/replanning; sim2real calibration.</x:v>
+      </x:c>
+      <x:c r="AZ15" t="str">
+        <x:v>No VF/Generative/BC; LLM size; drawer/CoT/multilingual.</x:v>
+      </x:c>
+      <x:c r="BA15" t="str">
+        <x:v>Planning errors, low-level execution, drawer manipulation, embodiment limits.</x:v>
+      </x:c>
+      <x:c r="BB15" t="str">
+        <x:v>OpenAlex Work W4224912544</x:v>
+      </x:c>
+      <x:c r="BC15" t="str">
+        <x:v>Google Research; arXiv; CoRL/PMLR; project page; official repository</x:v>
+      </x:c>
+      <x:c r="BD15" t="str">
+        <x:v>A-Upgraded</x:v>
+      </x:c>
+      <x:c r="BE15" t="str">
+        <x:v>Available - Verified</x:v>
+      </x:c>
+      <x:c r="BF15" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="BG15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BH15" t="str">
+        <x:v>https://arxiv.org/html/2204.01691</x:v>
+      </x:c>
+      <x:c r="BI15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BJ15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BK15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BL15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BM15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BN15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BO15" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="BP15" t="str">
+        <x:v>OpenAlex matched</x:v>
+      </x:c>
+      <x:c r="BQ15" t="str">
+        <x:v>Verified - 10.48550/arXiv.2204.01691</x:v>
+      </x:c>
+      <x:c r="BR15" t="str">
+        <x:v>Verified - 2204.01691</x:v>
+      </x:c>
+      <x:c r="BS15" t="str">
+        <x:v>Completed - Full text read</x:v>
+      </x:c>
+      <x:c r="BT15" t="str">
+        <x:v>true</x:v>
+      </x:c>
+      <x:c r="BU15" t="str">
+        <x:v>Completed-A</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
@@ -43801,7 +44231,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39291e5246964ba3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b540e7d6f794333"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete citation metrics pass
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R86f01c6dad0e4415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Rb991b7fdee134239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="Rdd3ba6f2361044fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rfc90709385e342e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="Ra1faf7c021804116"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rc96f7f93fef2443e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rfd09c41558954595"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rc736cc22804a4b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Re4602d75c7c141a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R67f546b2a2a7407e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rba32f92ab29c43ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R859d166c580e4cf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rfe0cb00ad062490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rcd0c832da3134a21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1201,14 +1201,14 @@
       <x:c r="AE2" t="str">
         <x:v>02_Papers/02_Robot_Manipulation/ManipLLM.md</x:v>
       </x:c>
-      <x:c r="AF2" t="str">
+      <x:c r="AF2" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="AG2" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AH2" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AI2" t="str">
         <x:v>研究主题为 `Multimodal / Generali</x:v>
@@ -1259,7 +1259,7 @@
         <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
       </x:c>
       <x:c r="AY2" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4402727730</x:v>
+        <x:v>https://openalex.org/W4402727730</x:v>
       </x:c>
       <x:c r="AZ2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -1377,14 +1377,14 @@
       <x:c r="AE3" t="str">
         <x:v>02_Papers/03_Bimanual/ManipTrans.md</x:v>
       </x:c>
-      <x:c r="AF3" t="str">
+      <x:c r="AF3" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="AG3" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AH3" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AI3" t="str">
         <x:v>研究主题为 `Residual Learning / Sim-to-Real`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -1435,7 +1435,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY3" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413145126</x:v>
       </x:c>
       <x:c r="AZ3" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -1553,14 +1553,14 @@
       <x:c r="AE4" t="str">
         <x:v>02_Papers/04_Dexterous/DexHandDiff.md</x:v>
       </x:c>
-      <x:c r="AF4" t="str">
+      <x:c r="AF4" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AG4" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AH4" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AI4" t="str">
         <x:v>研究主题为 `Diffusion / Contact-rich Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -1611,7 +1611,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY4" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413146641</x:v>
       </x:c>
       <x:c r="AZ4" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
@@ -1729,14 +1729,14 @@
       <x:c r="AE5" t="str">
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/AR-VRM.md</x:v>
       </x:c>
-      <x:c r="AF5" t="str">
+      <x:c r="AF5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AG5" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AH5" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AI5" t="str">
         <x:v>研究主题为 `Human Video / VLM`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -1787,7 +1787,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AY5" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4416242580</x:v>
       </x:c>
       <x:c r="AZ5" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -1944,7 +1944,7 @@
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AH6" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AI6" t="str">
         <x:v>LLMs have semantic knowledge but no embodiment or current-state grounding.</x:v>
@@ -1995,7 +1995,7 @@
         <x:v>Plan-execute gap; wrong object/negation; drawer manipulation and incomplete close; embodiment-specific failures.</x:v>
       </x:c>
       <x:c r="AY6" t="str">
-        <x:v>OpenAlex Work W4224912544</x:v>
+        <x:v>https://openalex.org/W4224912544</x:v>
       </x:c>
       <x:c r="AZ6" t="str">
         <x:v>Google Research publication; arXiv HTML 2204.01691; CoRL/PMLR; say-can.github.io; Google Research blog; official google-research/saycan</x:v>
@@ -5063,7 +5063,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c8b9cc21c0e4685"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf752ab12745d489f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8359,7 +8359,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24875c2dbfc745b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a7ef36493ad4994"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8710,7 +8710,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae14747bf124552"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d42fab89b1a4f3c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9456,7 +9456,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R148d6e9fc32646c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R411e0dc3c962411a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9768,10 +9768,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB2" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC2" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD2" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -9949,14 +9949,14 @@
       <x:c r="Z3" t="str">
         <x:v>02_Papers/03_Bimanual/Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework.md</x:v>
       </x:c>
-      <x:c r="AA3" t="str">
+      <x:c r="AA3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB3" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC3" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD3" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Bimanual`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -10007,7 +10007,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT3" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415101881</x:v>
       </x:c>
       <x:c r="AU3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -10134,14 +10134,14 @@
       <x:c r="Z4" t="str">
         <x:v>02_Papers/03_Bimanual/Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation.md</x:v>
       </x:c>
-      <x:c r="AA4" t="str">
+      <x:c r="AA4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB4" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC4" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD4" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Bimanual`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -10192,7 +10192,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT4" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414754983</x:v>
       </x:c>
       <x:c r="AU4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -10325,10 +10325,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB5" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC5" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD5" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -10506,14 +10506,14 @@
       <x:c r="Z6" t="str">
         <x:v>02_Papers/04_Dexterous/Cross-Embodiment_Dexterous_Grasping_with_Reinforcement_Learning.md</x:v>
       </x:c>
-      <x:c r="AA6" t="str">
+      <x:c r="AA6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB6" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC6" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD6" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -10564,7 +10564,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT6" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4403883977</x:v>
       </x:c>
       <x:c r="AU6" t="str">
         <x:v>Unknown</x:v>
@@ -10695,10 +10695,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB7" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC7" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD7" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -10874,14 +10874,14 @@
       <x:c r="Z8" t="str">
         <x:v>02_Papers/04_Dexterous/DexTrack.md</x:v>
       </x:c>
-      <x:c r="AA8" t="str">
+      <x:c r="AA8" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB8" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC8" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD8" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -10932,7 +10932,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT8" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4407590583</x:v>
       </x:c>
       <x:c r="AU8" t="str">
         <x:v>Unknown</x:v>
@@ -11063,10 +11063,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB9" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD9" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -11242,14 +11242,14 @@
       <x:c r="Z10" t="str">
         <x:v>02_Papers/10_Benchmark_Dataset/AdaManip.md</x:v>
       </x:c>
-      <x:c r="AA10" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA10" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB10" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC10" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD10" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -11300,7 +11300,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT10" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4407690282</x:v>
       </x:c>
       <x:c r="AU10" t="str">
         <x:v>Unknown</x:v>
@@ -11429,14 +11429,14 @@
       <x:c r="Z11" t="str">
         <x:v>02_Papers/07_Generalization_LongHorizon/HAMSTER.md</x:v>
       </x:c>
-      <x:c r="AA11" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA11" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB11" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC11" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD11" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -11487,7 +11487,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT11" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4407384835</x:v>
       </x:c>
       <x:c r="AU11" t="str">
         <x:v>Unknown</x:v>
@@ -11616,14 +11616,14 @@
       <x:c r="Z12" t="str">
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/ET-SEED.md</x:v>
       </x:c>
-      <x:c r="AA12" t="str">
+      <x:c r="AA12" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB12" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC12" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD12" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -11674,7 +11674,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT12" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4404371741</x:v>
       </x:c>
       <x:c r="AU12" t="str">
         <x:v>Unknown</x:v>
@@ -11804,13 +11804,13 @@
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/Bidirectional_Decoding.md</x:v>
       </x:c>
       <x:c r="AA13" t="str">
-        <x:v>0</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB13" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC13" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD13" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -11992,10 +11992,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB14" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC14" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD14" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -12176,13 +12176,13 @@
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/Demystifying_Robot_Diffusion_Policies_Action_Memorization_and_a_Simple_Lookup_Table_Altern.md</x:v>
       </x:c>
       <x:c r="AA15" t="str">
-        <x:v>0</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB15" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC15" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD15" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -12358,14 +12358,14 @@
       <x:c r="Z16" t="str">
         <x:v>02_Papers/01_VLA/SP-VLA.md</x:v>
       </x:c>
-      <x:c r="AA16" t="str">
+      <x:c r="AA16" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB16" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC16" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD16" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -12416,7 +12416,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT16" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4417536563</x:v>
       </x:c>
       <x:c r="AU16" t="str">
         <x:v>Unknown</x:v>
@@ -12545,10 +12545,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB17" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC17" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD17" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -12724,14 +12724,14 @@
       <x:c r="Z18" t="str">
         <x:v>02_Papers/01_VLA/Actions_as_Language.md</x:v>
       </x:c>
-      <x:c r="AA18" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA18" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AB18" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC18" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD18" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -12782,7 +12782,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT18" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7083676685</x:v>
       </x:c>
       <x:c r="AU18" t="str">
         <x:v>Unknown</x:v>
@@ -12913,10 +12913,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB19" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC19" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD19" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -13096,10 +13096,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB20" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC20" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD20" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -13281,10 +13281,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB21" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC21" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD21" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -13466,10 +13466,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB22" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC22" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD22" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -13651,10 +13651,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB23" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC23" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD23" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -13836,10 +13836,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB24" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC24" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD24" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -14019,10 +14019,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB25" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC25" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD25" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -14204,10 +14204,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB26" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC26" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD26" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -14385,14 +14385,14 @@
       <x:c r="Z27" t="str">
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/Learning_Robotic_Manipulation_Policies_from_Point_Clouds_with_Conditional_Flow_Matching.md</x:v>
       </x:c>
-      <x:c r="AA27" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA27" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB27" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC27" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD27" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -14443,7 +14443,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT27" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4403622102</x:v>
       </x:c>
       <x:c r="AU27" t="str">
         <x:v>Unknown</x:v>
@@ -14570,14 +14570,14 @@
       <x:c r="Z28" t="str">
         <x:v>02_Papers/07_Generalization_LongHorizon/SPIRE.md</x:v>
       </x:c>
-      <x:c r="AA28" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA28" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB28" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC28" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD28" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -14628,7 +14628,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT28" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4404308601</x:v>
       </x:c>
       <x:c r="AU28" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
@@ -14755,14 +14755,14 @@
       <x:c r="Z29" t="str">
         <x:v>02_Papers/08_Data_Teleoperation/OPEN_TEACH.md</x:v>
       </x:c>
-      <x:c r="AA29" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA29" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AB29" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC29" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD29" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -14813,7 +14813,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT29" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4392781441</x:v>
       </x:c>
       <x:c r="AU29" t="str">
         <x:v>Unknown</x:v>
@@ -14940,14 +14940,14 @@
       <x:c r="Z30" t="str">
         <x:v>02_Papers/07_Generalization_LongHorizon/RAM.md</x:v>
       </x:c>
-      <x:c r="AA30" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA30" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="AB30" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC30" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD30" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -14998,7 +14998,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT30" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400435236</x:v>
       </x:c>
       <x:c r="AU30" t="str">
         <x:v>Unknown</x:v>
@@ -15125,14 +15125,14 @@
       <x:c r="Z31" t="str">
         <x:v>02_Papers/08_Data_Teleoperation/ManiWAV.md</x:v>
       </x:c>
-      <x:c r="AA31" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA31" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AB31" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC31" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD31" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -15183,7 +15183,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT31" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400222297</x:v>
       </x:c>
       <x:c r="AU31" t="str">
         <x:v>Unknown</x:v>
@@ -15310,14 +15310,14 @@
       <x:c r="Z32" t="str">
         <x:v>02_Papers/02_Robot_Manipulation/Dreamitate.md</x:v>
       </x:c>
-      <x:c r="AA32" t="str">
+      <x:c r="AA32" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB32" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC32" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD32" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -15368,7 +15368,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT32" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400024954</x:v>
       </x:c>
       <x:c r="AU32" t="str">
         <x:v>Unknown</x:v>
@@ -15499,10 +15499,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB33" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC33" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD33" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -15680,14 +15680,14 @@
       <x:c r="Z34" t="str">
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/EquiBot.md</x:v>
       </x:c>
-      <x:c r="AA34" t="str">
+      <x:c r="AA34" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB34" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC34" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD34" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -15738,7 +15738,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT34" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400373516</x:v>
       </x:c>
       <x:c r="AU34" t="str">
         <x:v>Unknown</x:v>
@@ -15865,14 +15865,14 @@
       <x:c r="Z35" t="str">
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/3D_Diffuser_Actor.md</x:v>
       </x:c>
-      <x:c r="AA35" t="str">
+      <x:c r="AA35" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AB35" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC35" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD35" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -15923,7 +15923,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT35" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4391949089</x:v>
       </x:c>
       <x:c r="AU35" t="str">
         <x:v>Unknown</x:v>
@@ -16050,14 +16050,14 @@
       <x:c r="Z36" t="str">
         <x:v>02_Papers/10_Benchmark_Dataset/BiGym.md</x:v>
       </x:c>
-      <x:c r="AA36" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA36" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AB36" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC36" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD36" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -16108,7 +16108,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT36" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400611211</x:v>
       </x:c>
       <x:c r="AU36" t="str">
         <x:v>Unknown</x:v>
@@ -16235,14 +16235,14 @@
       <x:c r="Z37" t="str">
         <x:v>02_Papers/03_Bimanual/VoxAct-B.md</x:v>
       </x:c>
-      <x:c r="AA37" t="str">
+      <x:c r="AA37" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB37" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC37" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD37" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -16293,7 +16293,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT37" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4400434472</x:v>
       </x:c>
       <x:c r="AU37" t="str">
         <x:v>Unknown</x:v>
@@ -16421,13 +16421,13 @@
         <x:v>02_Papers/03_Bimanual/Mobile_ALOHA.md</x:v>
       </x:c>
       <x:c r="AA38" t="str">
-        <x:v>31</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB38" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC38" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD38" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -16605,14 +16605,14 @@
       <x:c r="Z39" t="str">
         <x:v>02_Papers/03_Bimanual/ALOHA_Unleashed.md</x:v>
       </x:c>
-      <x:c r="AA39" t="str">
+      <x:c r="AA39" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AB39" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC39" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD39" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -16663,7 +16663,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT39" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4403579180</x:v>
       </x:c>
       <x:c r="AU39" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
@@ -16792,10 +16792,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB40" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC40" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD40" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -16975,10 +16975,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB41" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC41" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD41" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17154,14 +17154,14 @@
       <x:c r="Z42" t="str">
         <x:v>02_Papers/03_Bimanual/COMBO-Grasp.md</x:v>
       </x:c>
-      <x:c r="AA42" t="str">
+      <x:c r="AA42" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB42" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC42" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD42" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17212,7 +17212,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT42" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4407569722</x:v>
       </x:c>
       <x:c r="AU42" t="str">
         <x:v>Unknown</x:v>
@@ -17341,10 +17341,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB43" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC43" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD43" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17520,14 +17520,14 @@
       <x:c r="Z44" t="str">
         <x:v>02_Papers/04_Dexterous/DexUMI.md</x:v>
       </x:c>
-      <x:c r="AA44" t="str">
+      <x:c r="AA44" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB44" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC44" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD44" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17578,7 +17578,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT44" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4416623172</x:v>
       </x:c>
       <x:c r="AU44" t="str">
         <x:v>Unknown</x:v>
@@ -17707,10 +17707,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB45" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC45" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD45" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17888,14 +17888,14 @@
       <x:c r="Z46" t="str">
         <x:v>02_Papers/09_Survey_Review/A_Survey_on_Vision-Language-Action_Models_for_Embodied_AI.md</x:v>
       </x:c>
-      <x:c r="AA46" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA46" t="n">
+        <x:v>29</x:v>
       </x:c>
       <x:c r="AB46" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC46" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD46" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -17946,7 +17946,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT46" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4398796510</x:v>
       </x:c>
       <x:c r="AU46" t="str">
         <x:v>Unknown</x:v>
@@ -18077,10 +18077,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB47" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC47" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD47" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -18258,14 +18258,14 @@
       <x:c r="Z48" t="str">
         <x:v>02_Papers/09_Survey_Review/What_Foundation_Models_can_Bring_for_Robot_Learning_in_Manipulation_A_Survey.md</x:v>
       </x:c>
-      <x:c r="AA48" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA48" t="n">
+        <x:v>6</x:v>
       </x:c>
       <x:c r="AB48" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC48" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD48" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -18316,7 +18316,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT48" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4416422407</x:v>
       </x:c>
       <x:c r="AU48" t="str">
         <x:v>Unknown</x:v>
@@ -18443,14 +18443,14 @@
       <x:c r="Z49" t="str">
         <x:v>02_Papers/09_Survey_Review/A_Survey_on_Robotics_with_Foundation_Models_Toward_Embodied_AI.md</x:v>
       </x:c>
-      <x:c r="AA49" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA49" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AB49" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC49" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD49" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -18501,7 +18501,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT49" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4391590994</x:v>
       </x:c>
       <x:c r="AU49" t="str">
         <x:v>Unknown</x:v>
@@ -18632,10 +18632,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB50" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC50" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD50" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -18813,14 +18813,14 @@
       <x:c r="Z51" t="str">
         <x:v>02_Papers/09_Survey_Review/Survey_of_Learning-Based_Approaches_for_Robotic_In-Hand_Manipulation.md</x:v>
       </x:c>
-      <x:c r="AA51" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA51" t="n">
+        <x:v>28</x:v>
       </x:c>
       <x:c r="AB51" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC51" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD51" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -18871,7 +18871,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT51" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4404085362</x:v>
       </x:c>
       <x:c r="AU51" t="str">
         <x:v>Unknown</x:v>
@@ -18998,14 +18998,14 @@
       <x:c r="Z52" t="str">
         <x:v>02_Papers/09_Survey_Review/Dexterous_Hand_towards_Intelligent_Manufacturing_A_Review_of_Technologies,_Trends,_and_Pot.md</x:v>
       </x:c>
-      <x:c r="AA52" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA52" t="n">
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AB52" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC52" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD52" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19056,7 +19056,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT52" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4409168415</x:v>
       </x:c>
       <x:c r="AU52" t="str">
         <x:v>Unknown</x:v>
@@ -19183,14 +19183,14 @@
       <x:c r="Z53" t="str">
         <x:v>02_Papers/09_Survey_Review/A_Survey_of_Embodied_Learning_for_Object-Centric_Robotic_Manipulation.md</x:v>
       </x:c>
-      <x:c r="AA53" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA53" t="n">
+        <x:v>16</x:v>
       </x:c>
       <x:c r="AB53" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC53" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD53" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19241,7 +19241,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT53" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4405426927</x:v>
       </x:c>
       <x:c r="AU53" t="str">
         <x:v>Unknown</x:v>
@@ -19368,14 +19368,14 @@
       <x:c r="Z54" t="str">
         <x:v>02_Papers/09_Survey_Review/Interactive_Imitation_Learning_for_Dexterous_Robotic_Manipulation_Challenges_and_Perspecti.md</x:v>
       </x:c>
-      <x:c r="AA54" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA54" t="n">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="AB54" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC54" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD54" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19426,7 +19426,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT54" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4417483688</x:v>
       </x:c>
       <x:c r="AU54" t="str">
         <x:v>Unknown</x:v>
@@ -19557,10 +19557,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB55" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC55" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD55" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19742,10 +19742,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB56" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC56" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD56" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19923,14 +19923,14 @@
       <x:c r="Z57" t="str">
         <x:v>02_Papers/09_Survey_Review/A_Survey_of_Demonstration_Learning.md</x:v>
       </x:c>
-      <x:c r="AA57" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA57" t="n">
+        <x:v>32</x:v>
       </x:c>
       <x:c r="AB57" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC57" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD57" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -19981,7 +19981,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT57" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402510263</x:v>
       </x:c>
       <x:c r="AU57" t="str">
         <x:v>Unknown</x:v>
@@ -20115,13 +20115,13 @@
         <x:v>02_Papers/03_Bimanual/RDT-1B.md</x:v>
       </x:c>
       <x:c r="AA58" t="str">
-        <x:v>5</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB58" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC58" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD58" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -20305,14 +20305,14 @@
       <x:c r="Z59" t="str">
         <x:v>02_Papers/03_Bimanual/TwinVLA.md</x:v>
       </x:c>
-      <x:c r="AA59" t="str">
+      <x:c r="AA59" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB59" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC59" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD59" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -20363,7 +20363,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT59" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7104816971</x:v>
       </x:c>
       <x:c r="AU59" t="str">
         <x:v>Unknown</x:v>
@@ -20498,10 +20498,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB60" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC60" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD60" t="str">
         <x:v>研究主题为 `Bimanual; Dataset / Benchmark`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -20685,14 +20685,14 @@
       <x:c r="Z61" t="str">
         <x:v>02_Papers/01_VLA/BridgeVLA.md</x:v>
       </x:c>
-      <x:c r="AA61" t="str">
+      <x:c r="AA61" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB61" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC61" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD61" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -20743,7 +20743,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT61" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415272059</x:v>
       </x:c>
       <x:c r="AU61" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -20876,14 +20876,14 @@
       <x:c r="Z62" t="str">
         <x:v>02_Papers/01_VLA/VLA-Cache.md</x:v>
       </x:c>
-      <x:c r="AA62" t="str">
+      <x:c r="AA62" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="AB62" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC62" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD62" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -20934,7 +20934,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT62" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196930033</x:v>
       </x:c>
       <x:c r="AU62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -21071,10 +21071,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB63" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC63" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD63" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -21258,14 +21258,14 @@
       <x:c r="Z64" t="str">
         <x:v>02_Papers/01_VLA/3D-VLA.md</x:v>
       </x:c>
-      <x:c r="AA64" t="str">
+      <x:c r="AA64" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="AB64" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC64" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD64" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models; Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -21316,7 +21316,7 @@
         <x:v>Not Explicitly Reported in the accessible proceedings page.</x:v>
       </x:c>
       <x:c r="AT64" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4392886475</x:v>
+        <x:v>https://openalex.org/W4392886475</x:v>
       </x:c>
       <x:c r="AU64" t="str">
         <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
@@ -21449,14 +21449,14 @@
       <x:c r="Z65" t="str">
         <x:v>02_Papers/01_VLA/RoboMamba.md</x:v>
       </x:c>
-      <x:c r="AA65" t="str">
+      <x:c r="AA65" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="AB65" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC65" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD65" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -21507,7 +21507,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT65" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415797921</x:v>
       </x:c>
       <x:c r="AU65" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
@@ -21641,13 +21641,13 @@
         <x:v>02_Papers/01_VLA/TraceVLA.md</x:v>
       </x:c>
       <x:c r="AA66" t="str">
-        <x:v>1</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB66" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AC66" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD66" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -21835,10 +21835,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB67" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC67" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD67" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -22021,13 +22021,13 @@
         <x:v>02_Papers/06_Diffusion_Flow_IL_RL/FlowPolicy.md</x:v>
       </x:c>
       <x:c r="AA68" t="str">
-        <x:v>16</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB68" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC68" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD68" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -22211,14 +22211,14 @@
       <x:c r="Z69" t="str">
         <x:v>02_Papers/04_Dexterous/UniGraspTransformer.md</x:v>
       </x:c>
-      <x:c r="AA69" t="str">
+      <x:c r="AA69" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="AB69" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC69" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD69" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -22269,7 +22269,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT69" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413145029</x:v>
       </x:c>
       <x:c r="AU69" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -22402,14 +22402,14 @@
       <x:c r="Z70" t="str">
         <x:v>02_Papers/04_Dexterous/Scaffolding_Dexterous_Manipulation_with_Vision-Language_Models.md</x:v>
       </x:c>
-      <x:c r="AA70" t="str">
+      <x:c r="AA70" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB70" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC70" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD70" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -22460,7 +22460,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT70" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414683599</x:v>
       </x:c>
       <x:c r="AU70" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -22593,14 +22593,14 @@
       <x:c r="Z71" t="str">
         <x:v>02_Papers/01_VLA/VideoVLA.md</x:v>
       </x:c>
-      <x:c r="AA71" t="str">
+      <x:c r="AA71" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AB71" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC71" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD71" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -22651,7 +22651,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT71" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196952124</x:v>
       </x:c>
       <x:c r="AU71" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -22784,14 +22784,14 @@
       <x:c r="Z72" t="str">
         <x:v>02_Papers/04_Dexterous/DextER.md</x:v>
       </x:c>
-      <x:c r="AA72" t="str">
+      <x:c r="AA72" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB72" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC72" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD72" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -22842,7 +22842,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT72" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7125566978</x:v>
       </x:c>
       <x:c r="AU72" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -22975,14 +22975,14 @@
       <x:c r="Z73" t="str">
         <x:v>02_Papers/01_VLA/SpatialVLA.md</x:v>
       </x:c>
-      <x:c r="AA73" t="str">
+      <x:c r="AA73" t="n">
         <x:v>41</x:v>
       </x:c>
       <x:c r="AB73" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC73" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD73" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -23033,7 +23033,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT73" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414051092</x:v>
       </x:c>
       <x:c r="AU73" t="str">
         <x:v>Unknown</x:v>
@@ -23166,14 +23166,14 @@
       <x:c r="Z74" t="str">
         <x:v>02_Papers/01_VLA/OpenVLA.md</x:v>
       </x:c>
-      <x:c r="AA74" t="str">
+      <x:c r="AA74" t="n">
         <x:v>43</x:v>
       </x:c>
       <x:c r="AB74" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC74" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD74" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -23224,7 +23224,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT74" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4399695759</x:v>
       </x:c>
       <x:c r="AU74" t="str">
         <x:v>Unknown</x:v>
@@ -23357,14 +23357,14 @@
       <x:c r="Z75" t="str">
         <x:v>02_Papers/01_VLA/Octo.md</x:v>
       </x:c>
-      <x:c r="AA75" t="str">
+      <x:c r="AA75" t="n">
         <x:v>102</x:v>
       </x:c>
       <x:c r="AB75" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC75" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD75" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -23415,7 +23415,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT75" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402353985</x:v>
       </x:c>
       <x:c r="AU75" t="str">
         <x:v>Unknown</x:v>
@@ -23548,10 +23548,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB76" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC76" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD76" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -23731,14 +23731,14 @@
       <x:c r="Z77" t="str">
         <x:v>02_Papers/10_Benchmark_Dataset/RoboCasa.md</x:v>
       </x:c>
-      <x:c r="AA77" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AA77" t="n">
+        <x:v>44</x:v>
       </x:c>
       <x:c r="AB77" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC77" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD77" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -23789,7 +23789,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT77" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402354126</x:v>
       </x:c>
       <x:c r="AU77" t="str">
         <x:v>Unknown</x:v>
@@ -23922,10 +23922,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AB78" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AC78" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD78" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -24111,14 +24111,14 @@
       <x:c r="Z79" t="str">
         <x:v>02_Papers/01_VLA/ReconVLA.md</x:v>
       </x:c>
-      <x:c r="AA79" t="str">
+      <x:c r="AA79" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AB79" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AC79" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AD79" t="str">
         <x:v>现有 VLA 在执行操作时对任务目标区域的视觉注意力往往过于分散，可能关注错误对象，影响精确操作。</x:v>
@@ -24169,7 +24169,7 @@
         <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
       </x:c>
       <x:c r="AT79" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W7137985120</x:v>
+        <x:v>https://openalex.org/W7137985120</x:v>
       </x:c>
       <x:c r="AU79" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
@@ -24245,7 +24245,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref9e2238cf614bf0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51f5e2fd390a42b8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24695,10 +24695,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV2" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AW2" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX2" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -24933,14 +24933,14 @@
       <x:c r="AT3" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU3" t="str">
+      <x:c r="AU3" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV3" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW3" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX3" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Bimanual`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -24988,7 +24988,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM3" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415101881</x:v>
       </x:c>
       <x:c r="BN3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -25175,14 +25175,14 @@
       <x:c r="AT4" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU4" t="str">
+      <x:c r="AU4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV4" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW4" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX4" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Bimanual`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -25230,7 +25230,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM4" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414754983</x:v>
       </x:c>
       <x:c r="BN4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -25421,10 +25421,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV5" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW5" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX5" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -25663,10 +25663,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV6" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW6" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX6" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -25905,10 +25905,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV7" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW7" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX7" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -26147,10 +26147,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV8" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW8" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX8" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -26387,10 +26387,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV9" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX9" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -26633,10 +26633,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV10" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW10" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX10" t="str">
         <x:v>研究主题为 `Bimanual; Dataset / Benchmark`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -26877,14 +26877,14 @@
       <x:c r="AT11" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU11" t="str">
+      <x:c r="AU11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV11" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW11" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX11" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -26932,7 +26932,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM11" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415272059</x:v>
       </x:c>
       <x:c r="BN11" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -27125,14 +27125,14 @@
       <x:c r="AT12" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU12" t="str">
+      <x:c r="AU12" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="AV12" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW12" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX12" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -27180,7 +27180,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM12" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196930033</x:v>
       </x:c>
       <x:c r="BN12" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/f062da1973ac9ac61fc6d44dd7fa309f-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -27377,10 +27377,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV13" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW13" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX13" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -27621,14 +27621,14 @@
       <x:c r="AT14" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU14" t="str">
+      <x:c r="AU14" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="AV14" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW14" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX14" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models; Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -27676,7 +27676,7 @@
         <x:v>Not Explicitly Reported in the accessible proceedings page.</x:v>
       </x:c>
       <x:c r="BM14" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4392886475</x:v>
+        <x:v>https://openalex.org/W4392886475</x:v>
       </x:c>
       <x:c r="BN14" t="str">
         <x:v>https://proceedings.mlr.press/v235/zhen24a.html；官方摘要/论文集元数据</x:v>
@@ -27869,14 +27869,14 @@
       <x:c r="AT15" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU15" t="str">
+      <x:c r="AU15" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="AV15" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW15" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX15" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -27924,7 +27924,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM15" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415797921</x:v>
       </x:c>
       <x:c r="BN15" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
@@ -28116,13 +28116,13 @@
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
       <x:c r="AU16" t="str">
-        <x:v>16</x:v>
+        <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV16" t="str">
-        <x:v>OpenAlex</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW16" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX16" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -28363,14 +28363,14 @@
       <x:c r="AT17" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU17" t="str">
+      <x:c r="AU17" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="AV17" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW17" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX17" t="str">
         <x:v>研究主题为 `Robot Manipulation / IL / Diffusion; Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -28418,7 +28418,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM17" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413145029</x:v>
       </x:c>
       <x:c r="BN17" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -28611,14 +28611,14 @@
       <x:c r="AT18" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU18" t="str">
+      <x:c r="AU18" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV18" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW18" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX18" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -28666,7 +28666,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM18" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414683599</x:v>
       </x:c>
       <x:c r="BN18" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -28859,14 +28859,14 @@
       <x:c r="AT19" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU19" t="str">
+      <x:c r="AU19" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AV19" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW19" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX19" t="str">
         <x:v>研究主题为 `VLA / Robot Foundation Models`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -28914,7 +28914,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM19" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196952124</x:v>
       </x:c>
       <x:c r="BN19" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -29107,14 +29107,14 @@
       <x:c r="AT20" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU20" t="str">
+      <x:c r="AU20" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV20" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW20" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX20" t="str">
         <x:v>研究主题为 `Dexterous Hand / Dexterous Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -29162,7 +29162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM20" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7125566978</x:v>
       </x:c>
       <x:c r="BN20" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -29357,14 +29357,14 @@
       <x:c r="AT21" t="str">
         <x:v>Robot Manipulation</x:v>
       </x:c>
-      <x:c r="AU21" t="str">
+      <x:c r="AU21" t="n">
         <x:v>82</x:v>
       </x:c>
       <x:c r="AV21" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW21" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX21" t="str">
         <x:v>研究主题为 `Multimodal / Generali</x:v>
@@ -29412,7 +29412,7 @@
         <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
       </x:c>
       <x:c r="BM21" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4402727730</x:v>
+        <x:v>https://openalex.org/W4402727730</x:v>
       </x:c>
       <x:c r="BN21" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -29607,14 +29607,14 @@
       <x:c r="AT22" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU22" t="str">
+      <x:c r="AU22" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="AV22" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW22" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX22" t="str">
         <x:v>研究主题为 `Residual Learning / Sim-to-Real`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -29662,7 +29662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM22" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413145126</x:v>
       </x:c>
       <x:c r="BN22" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -29857,14 +29857,14 @@
       <x:c r="AT23" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU23" t="str">
+      <x:c r="AU23" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV23" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW23" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX23" t="str">
         <x:v>研究主题为 `Diffusion / Contact-rich Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -29912,7 +29912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM23" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413146641</x:v>
       </x:c>
       <x:c r="BN23" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
@@ -30107,14 +30107,14 @@
       <x:c r="AT24" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU24" t="str">
+      <x:c r="AU24" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV24" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW24" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX24" t="str">
         <x:v>研究主题为 `Human Video / VLM`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -30162,7 +30162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM24" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4416242580</x:v>
       </x:c>
       <x:c r="BN24" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -30357,14 +30357,14 @@
       <x:c r="AT25" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU25" t="str">
+      <x:c r="AU25" t="n">
         <x:v>29</x:v>
       </x:c>
       <x:c r="AV25" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW25" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX25" t="str">
         <x:v>研究主题为 `Dexterous Grasping`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -30412,7 +30412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM25" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402816741</x:v>
       </x:c>
       <x:c r="BN25" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Xu_Dexterous_Grasp_Transformer_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -30607,14 +30607,14 @@
       <x:c r="AT26" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU26" t="str">
+      <x:c r="AU26" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="AV26" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW26" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX26" t="str">
         <x:v>研究主题为 `Mobile Manipulation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -30662,7 +30662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM26" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413147465</x:v>
       </x:c>
       <x:c r="BN26" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wu_MoManipVLA_Transferring_Vision-language-action_Models_for_General_Mobile_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -30857,14 +30857,14 @@
       <x:c r="AT27" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU27" t="str">
+      <x:c r="AU27" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="AV27" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW27" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX27" t="str">
         <x:v>研究主题为 `Action Chunking / Multi-task Policy`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -30912,7 +30912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM27" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415800339</x:v>
       </x:c>
       <x:c r="BN27" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/ff887781480973bd3cb6026feb378d1e-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -31107,14 +31107,14 @@
       <x:c r="AT28" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AU28" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU28" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AV28" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW28" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX28" t="str">
         <x:v>研究主题为 `Surgical Robotics`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -31162,7 +31162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM28" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415796959</x:v>
       </x:c>
       <x:c r="BN28" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/74c4f2b87b7499d365422152c76fd916-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -31357,14 +31357,14 @@
       <x:c r="AT29" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU29" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU29" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AV29" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW29" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX29" t="str">
         <x:v>研究主题为 `Video Demonstration / Reward Learning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -31412,7 +31412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM29" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415795570</x:v>
       </x:c>
       <x:c r="BN29" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/dcd297696d0bb304ba426b3c5a679c37-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -31607,14 +31607,14 @@
       <x:c r="AT30" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU30" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU30" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="AV30" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW30" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX30" t="str">
         <x:v>研究主题为 `Long-Hori</x:v>
@@ -31662,7 +31662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM30" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415800541</x:v>
       </x:c>
       <x:c r="BN30" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/fad8962279154544ed69bb63eb14d677-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -31857,14 +31857,14 @@
       <x:c r="AT31" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AU31" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU31" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="AV31" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW31" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX31" t="str">
         <x:v>研究主题为 `3D Observation / Contact-rich`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -31912,7 +31912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM31" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415797227</x:v>
       </x:c>
       <x:c r="BN31" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/8e5dc5969a6174fcaaececd890c7f59b-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -32107,14 +32107,14 @@
       <x:c r="AT32" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU32" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU32" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AV32" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW32" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX32" t="str">
         <x:v>研究主题为 `Text-conditioned Reward`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -32162,7 +32162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM32" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415797662</x:v>
       </x:c>
       <x:c r="BN32" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/5227ce00add5aa0a12d1c4ee92fcd2dc-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -32361,10 +32361,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV33" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW33" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX33" t="str">
         <x:v>研究主题为 `Human-Robot Domain Adaptation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -32607,14 +32607,14 @@
       <x:c r="AT34" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU34" t="str">
+      <x:c r="AU34" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="AV34" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW34" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX34" t="str">
         <x:v>研究主题为 `Grounding / Synthetic Data`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -32662,7 +32662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM34" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413147462</x:v>
       </x:c>
       <x:c r="BN34" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Huang_RoboGround_Robotic_Manipulation_with_Grounded_Vision-Language_Priors_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -32857,14 +32857,14 @@
       <x:c r="AT35" t="str">
         <x:v>Data / Teleoperation</x:v>
       </x:c>
-      <x:c r="AU35" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU35" t="n">
+        <x:v>6</x:v>
       </x:c>
       <x:c r="AV35" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW35" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX35" t="str">
         <x:v>研究主题为 `Synthetic Data / Scene Generation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -32912,7 +32912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM35" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413147695</x:v>
       </x:c>
       <x:c r="BN35" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -33111,10 +33111,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV36" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AW36" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX36" t="str">
         <x:v>研究主题为 `Lifelong Learning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -33361,10 +33361,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV37" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW37" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX37" t="str">
         <x:v>研究主题为 `Failure Recovery / 3D Gaussian Splatting`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -33611,10 +33611,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV38" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW38" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX38" t="str">
         <x:v>研究主题为 `Articulated Object / Affordance`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -33861,10 +33861,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV39" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW39" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX39" t="str">
         <x:v>研究主题为 `Long-Hori</x:v>
@@ -34107,14 +34107,14 @@
       <x:c r="AT40" t="str">
         <x:v>Robot Manipulation</x:v>
       </x:c>
-      <x:c r="AU40" t="str">
-        <x:v>0</x:v>
+      <x:c r="AU40" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AV40" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW40" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX40" t="str">
         <x:v>研究主题为 `World Model / Video Diffusion`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -34162,7 +34162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM40" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7103754590</x:v>
       </x:c>
       <x:c r="BN40" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/481c70828a4ff20d31a646cc6cc95f3d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -34357,14 +34357,14 @@
       <x:c r="AT41" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU41" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU41" t="n">
+        <x:v>8</x:v>
       </x:c>
       <x:c r="AV41" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW41" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX41" t="str">
         <x:v>研究主题为 `Human Video / 3D Affordance`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -34412,7 +34412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM41" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413144616</x:v>
       </x:c>
       <x:c r="BN41" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generali</x:v>
@@ -34607,14 +34607,14 @@
       <x:c r="AT42" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU42" t="str">
+      <x:c r="AU42" t="n">
         <x:v>57</x:v>
       </x:c>
       <x:c r="AV42" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW42" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX42" t="str">
         <x:v>研究主题为 `Visual Chain-of-Thought`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -34662,7 +34662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM42" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413156213</x:v>
       </x:c>
       <x:c r="BN42" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -34857,14 +34857,14 @@
       <x:c r="AT43" t="str">
         <x:v>Sim2Real</x:v>
       </x:c>
-      <x:c r="AU43" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU43" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV43" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW43" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX43" t="str">
         <x:v>研究主题为 `Sim-to-Real / Behavior Cloning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -34912,7 +34912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM43" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415251366</x:v>
       </x:c>
       <x:c r="BN43" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1185c89347a3f21ffc48c9d083c9437c-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -35107,14 +35107,14 @@
       <x:c r="AT44" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU44" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU44" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV44" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW44" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX44" t="str">
         <x:v>研究主题为 `Long-Hori</x:v>
@@ -35162,7 +35162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM44" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196926233</x:v>
       </x:c>
       <x:c r="BN44" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b94310e1c7ecb79f1a24adc757f1b89b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -35357,14 +35357,14 @@
       <x:c r="AT45" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU45" t="str">
+      <x:c r="AU45" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV45" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW45" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX45" t="str">
         <x:v>研究主题为 `Stochastic Interpolant / Efficiency`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -35412,7 +35412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM45" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196975408</x:v>
       </x:c>
       <x:c r="BN45" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/49eadcc4a329fc6b74b9f8a82b78cbc3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -35607,14 +35607,14 @@
       <x:c r="AT46" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU46" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU46" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AV46" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW46" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX46" t="str">
         <x:v>研究主题为 `Mobile Manipulation / Agent`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -35662,7 +35662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM46" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7197036842</x:v>
       </x:c>
       <x:c r="BN46" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/bc97207e3979d1cc23109db0be0e8ed2-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -35857,14 +35857,14 @@
       <x:c r="AT47" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU47" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU47" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV47" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW47" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX47" t="str">
         <x:v>研究主题为 `Flow Matching / Visuomotor Policy`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -35912,7 +35912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM47" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4417258107</x:v>
       </x:c>
       <x:c r="BN47" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/282c3318be1b047b7bb5ba94fa4f3231-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36107,14 +36107,14 @@
       <x:c r="AT48" t="str">
         <x:v>Robot Manipulation</x:v>
       </x:c>
-      <x:c r="AU48" t="str">
+      <x:c r="AU48" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV48" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW48" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX48" t="str">
         <x:v>研究主题为 `Tool Use / Generative Design`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -36162,7 +36162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM48" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4415312722</x:v>
       </x:c>
       <x:c r="BN48" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/9fc291fef2f9607a46777d367f900a15-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36357,14 +36357,14 @@
       <x:c r="AT49" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AU49" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU49" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV49" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW49" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX49" t="str">
         <x:v>研究主题为 `3D Manipulation / Multimodal Policy`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -36412,7 +36412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM49" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4417082659</x:v>
       </x:c>
       <x:c r="BN49" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/eacc8ae341d15d2c13c02fef88189db3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36607,14 +36607,14 @@
       <x:c r="AT50" t="str">
         <x:v>Data / Teleoperation</x:v>
       </x:c>
-      <x:c r="AU50" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU50" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV50" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW50" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX50" t="str">
         <x:v>研究主题为 `Robot Data / Spatial Reasoning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -36662,7 +36662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM50" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196982428</x:v>
       </x:c>
       <x:c r="BN50" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1f467c3e37abf9f86c78f44c6a27ee7c-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -36857,14 +36857,14 @@
       <x:c r="AT51" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU51" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU51" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV51" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW51" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX51" t="str">
         <x:v>研究主题为 `Task Planning / Demonstrations`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -36912,7 +36912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM51" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7196933803</x:v>
       </x:c>
       <x:c r="BN51" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b8358a00e5b870194b974ddf8dd415c3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -37107,14 +37107,14 @@
       <x:c r="AT52" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AU52" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AU52" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AV52" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW52" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX52" t="str">
         <x:v>研究主题为 `Human-to-Robot Handover / Teleoperation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -37162,7 +37162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM52" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7160048141</x:v>
       </x:c>
       <x:c r="BN52" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Wang_DexH2R_A_Benchmark_for_Dynamic_Dexterous_Grasping_in_Human-to-Robot_Handover_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -37357,14 +37357,14 @@
       <x:c r="AT53" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU53" t="str">
+      <x:c r="AU53" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="AV53" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW53" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX53" t="str">
         <x:v>研究主题为 `3D Hand-Object Interaction / Articulated Objects`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -37412,7 +37412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM53" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413145043</x:v>
       </x:c>
       <x:c r="BN53" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -37607,14 +37607,14 @@
       <x:c r="AT54" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU54" t="str">
+      <x:c r="AU54" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV54" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW54" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX54" t="str">
         <x:v>研究主题为 `Vision-Language-Grasp / Flow Matching`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -37662,7 +37662,7 @@
         <x:v>The reported setting focuses on tabletop part-aligned grasps; broader clutter, occlusion and multi-step manipulation are not established by the cited results.</x:v>
       </x:c>
       <x:c r="BM54" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4417183400</x:v>
+        <x:v>https://openalex.org/W4417183400</x:v>
       </x:c>
       <x:c r="BN54" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/He_DexVLG_Dexterous_Vision-Language-Grasp_Model_at_Scale_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -37857,14 +37857,14 @@
       <x:c r="AT55" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU55" t="str">
+      <x:c r="AU55" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="AV55" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW55" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX55" t="str">
         <x:v>研究主题为 `Hand-Object Motion / Generali</x:v>
@@ -37912,7 +37912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM55" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4413146191</x:v>
       </x:c>
       <x:c r="BN55" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generali</x:v>
@@ -38111,10 +38111,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV56" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AW56" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX56" t="str">
         <x:v>研究主题为 `Tool-Action-Object Understanding`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -38357,14 +38357,14 @@
       <x:c r="AT57" t="str">
         <x:v>Robot Manipulation</x:v>
       </x:c>
-      <x:c r="AU57" t="str">
+      <x:c r="AU57" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="AV57" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW57" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX57" t="str">
         <x:v>研究主题为 `Mobile Manipulation / Navigation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -38412,7 +38412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM57" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402772268</x:v>
       </x:c>
       <x:c r="BN57" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Uppal_SPIN_Simultaneous_Perception_Interaction_and_Navigation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -38607,14 +38607,14 @@
       <x:c r="AT58" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU58" t="str">
+      <x:c r="AU58" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV58" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW58" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX58" t="str">
         <x:v>研究主题为 `Policy Transfer / Generali</x:v>
@@ -38662,7 +38662,7 @@
         <x:v>The paper identifies observation discrepancy between unimanual and bimanual systems as a transfer risk; detailed failure cases require appendix extraction.</x:v>
       </x:c>
       <x:c r="BM58" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W4405254485</x:v>
+        <x:v>https://openalex.org/W4405254485</x:v>
       </x:c>
       <x:c r="BN58" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Lu_AnyBimanual_Transferring_Unimanual_Policy_for_General_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -38857,14 +38857,14 @@
       <x:c r="AT59" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU59" t="str">
+      <x:c r="AU59" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV59" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW59" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX59" t="str">
         <x:v>研究主题为 `Cross-Embodiment / Human Video`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -38912,7 +38912,7 @@
         <x:v>Cross-hand and retargeting edge cases are not detailed in the accessible abstract; full supplementary review is needed.</x:v>
       </x:c>
       <x:c r="BM59" t="str">
-        <x:v>OpenAlex Work: Unknown</x:v>
+        <x:v>https://openalex.org/W7140345735</x:v>
       </x:c>
       <x:c r="BN59" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Zhang_UniDex_A_Robot_Foundation_Suite_for_Universal_Dexterous_Hand_Control_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -39111,10 +39111,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AV60" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AW60" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX60" t="str">
         <x:v>研究主题为 `Video Generation / Hand-Object Interaction`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -39357,14 +39357,14 @@
       <x:c r="AT61" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU61" t="str">
+      <x:c r="AU61" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV61" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW61" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX61" t="str">
         <x:v>研究主题为 `Human Video / Motion Retargeting`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -39412,7 +39412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM61" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7138113519</x:v>
       </x:c>
       <x:c r="BN61" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38874；官方摘要/论文集元数据</x:v>
@@ -39607,14 +39607,14 @@
       <x:c r="AT62" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU62" t="str">
+      <x:c r="AU62" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV62" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW62" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX62" t="str">
         <x:v>研究主题为 `Humanoid / Synthetic Demonstrations / LLM Planning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -39662,7 +39662,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM62" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4417041439</x:v>
       </x:c>
       <x:c r="BN62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/e4ef7454447baa15a424314e6284441b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -39857,14 +39857,14 @@
       <x:c r="AT63" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU63" t="str">
+      <x:c r="AU63" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV63" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW63" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX63" t="str">
         <x:v>研究主题为 `Affordance / Policy Distillation`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -39912,7 +39912,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM63" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7138302344</x:v>
       </x:c>
       <x:c r="BN63" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38313；官方摘要/论文集元数据</x:v>
@@ -40107,14 +40107,14 @@
       <x:c r="AT64" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU64" t="str">
+      <x:c r="AU64" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV64" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW64" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX64" t="str">
         <x:v>研究主题为 `Human Demonstrations / Reinforcement Learning`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -40162,7 +40162,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM64" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W7138037195</x:v>
       </x:c>
       <x:c r="BN64" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/40127；官方摘要/论文集元数据</x:v>
@@ -40357,14 +40357,14 @@
       <x:c r="AT65" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU65" t="str">
+      <x:c r="AU65" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV65" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW65" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX65" t="str">
         <x:v>研究主题为 `Motion Forecasting / Hand-Object Contact`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -40412,7 +40412,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM65" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4393158202</x:v>
       </x:c>
       <x:c r="BN65" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28266；官方摘要/论文集元数据</x:v>
@@ -40607,14 +40607,14 @@
       <x:c r="AT66" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AU66" t="str">
+      <x:c r="AU66" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="AV66" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW66" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX66" t="str">
         <x:v>研究主题为 `Human Video / Affordance`；本卡仅按官方摘要级证据整理，未替代全文审阅。</x:v>
@@ -40662,7 +40662,7 @@
         <x:v>The paper notes ambiguity/multi-modality of valid interaction regions; exact failure examples require figure-level review.</x:v>
       </x:c>
       <x:c r="BM66" t="str">
-        <x:v>OpenAlex Work: Unknown</x:v>
+        <x:v>https://openalex.org/W4416031407</x:v>
       </x:c>
       <x:c r="BN66" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Heidinger_2HandedAfforder_Learning_Precise_Actionable_Bimanual_Affordances_from_Human_Videos_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -40857,14 +40857,14 @@
       <x:c r="AT67" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AU67" t="str">
+      <x:c r="AU67" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="AV67" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AW67" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AX67" t="str">
         <x:v>现有 VLA 在执行操作时对任务目标区域的视觉注意力往往过于分散，可能关注错误对象，影响精确操作。</x:v>
@@ -40912,7 +40912,7 @@
         <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
       </x:c>
       <x:c r="BM67" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W7137985120</x:v>
+        <x:v>https://openalex.org/W7137985120</x:v>
       </x:c>
       <x:c r="BN67" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
@@ -41003,7 +41003,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1420b6b070443d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d79457ce1774232"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41385,10 +41385,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL2" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AM2" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN2" t="str">
         <x:v>Synthetic-only VLA training usually transfers unreliably to real manipulation.</x:v>
@@ -41433,7 +41433,7 @@
         <x:v>Domain-gap evaluation explicitly tests background, object, table and combined shifts; exact failure cases require full-paper appendix extraction.</x:v>
       </x:c>
       <x:c r="BB2" t="str">
-        <x:v>OpenAlex Work: https://openalex.org/W? title match was not high-confidence for this title; Citation Count remains Unknown.</x:v>
+        <x:v>Unknown (no high-confidence match)</x:v>
       </x:c>
       <x:c r="BC2" t="str">
         <x:v>Official ICLR Downloads/Proceedings; accepted OpenReview PDF; official project page; official EmbodiChain repository; author publication list; current official CCF directory</x:v>
@@ -41598,14 +41598,14 @@
       <x:c r="AJ3" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AK3" t="str">
+      <x:c r="AK3" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="AL3" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM3" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN3" t="str">
         <x:v>Learning coordinated bimanual skills with low demonstration cost.</x:v>
@@ -41650,7 +41650,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB3" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414050937</x:v>
       </x:c>
       <x:c r="BC3" t="str">
         <x:v>https://www.roboticsproceedings.org/rss21/p149.html; https://hnu</x:v>
@@ -41815,14 +41815,14 @@
       <x:c r="AJ4" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AK4" t="str">
+      <x:c r="AK4" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="AL4" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM4" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN4" t="str">
         <x:v>Bimanual policies must combine spatial locali</x:v>
@@ -41867,7 +41867,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB4" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4414050727</x:v>
       </x:c>
       <x:c r="BC4" t="str">
         <x:v>RSS official proceedings abstract</x:v>
@@ -42036,10 +42036,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL5" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity ambiguous)</x:v>
       </x:c>
       <x:c r="AM5" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN5" t="str">
         <x:v>Collecting detailed, portable human-hand demonstrations for dexterous robot learning.</x:v>
@@ -42253,10 +42253,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL6" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AM6" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN6" t="str">
         <x:v>Manipulation policies are often evaluated too close to training conditions.</x:v>
@@ -42466,14 +42466,14 @@
       <x:c r="AJ7" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AK7" t="str">
+      <x:c r="AK7" t="n">
         <x:v>11</x:v>
       </x:c>
       <x:c r="AL7" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM7" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN7" t="str">
         <x:v>Planning while maintaining a fixed transform between two end effectors creates difficult equality constraints.</x:v>
@@ -42518,7 +42518,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB7" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4401415458</x:v>
       </x:c>
       <x:c r="BC7" t="str">
         <x:v>IEEE Xplore abstract; official project page</x:v>
@@ -42683,14 +42683,14 @@
       <x:c r="AJ8" t="str">
         <x:v>Diffusion / Flow / IL / RL</x:v>
       </x:c>
-      <x:c r="AK8" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AK8" t="n">
+        <x:v>14</x:v>
       </x:c>
       <x:c r="AL8" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM8" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN8" t="str">
         <x:v>Contact-rich imitation must reproduce forces and switch sensing/control modes reliably.</x:v>
@@ -42735,7 +42735,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB8" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4405753615</x:v>
       </x:c>
       <x:c r="BC8" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -42900,14 +42900,14 @@
       <x:c r="AJ9" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AK9" t="str">
+      <x:c r="AK9" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="AL9" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM9" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN9" t="str">
         <x:v>Multiple arms need online trajectory adaptation and collision avoidance in shared workspaces.</x:v>
@@ -42952,7 +42952,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB9" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4404520558</x:v>
       </x:c>
       <x:c r="BC9" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -43121,10 +43121,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL10" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AM10" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN10" t="str">
         <x:v>State and action representations may not transfer across reality gaps or hand geometries.</x:v>
@@ -43312,14 +43312,14 @@
       <x:c r="AJ11" t="str">
         <x:v>VLA</x:v>
       </x:c>
-      <x:c r="AK11" t="str">
+      <x:c r="AK11" t="n">
         <x:v>102</x:v>
       </x:c>
       <x:c r="AL11" t="str">
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM11" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN11" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -43364,7 +43364,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB11" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402353985</x:v>
       </x:c>
       <x:c r="BC11" t="str">
         <x:v>Unknown</x:v>
@@ -43507,10 +43507,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL12" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AM12" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN12" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -43694,14 +43694,14 @@
       <x:c r="AJ13" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AK13" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="AK13" t="n">
+        <x:v>44</x:v>
       </x:c>
       <x:c r="AL13" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM13" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN13" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -43746,7 +43746,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB13" t="str">
-        <x:v>Unknown (no high-confidence match)</x:v>
+        <x:v>https://openalex.org/W4402354126</x:v>
       </x:c>
       <x:c r="BC13" t="str">
         <x:v>Unknown</x:v>
@@ -43889,10 +43889,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="AL14" t="str">
-        <x:v>OpenAlex (no high-confidence title match)</x:v>
+        <x:v>OpenAlex (identity unmatched)</x:v>
       </x:c>
       <x:c r="AM14" t="str">
-        <x:v>2026-09-21</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN14" t="str">
         <x:v>Unknown / Needs Full-Paper Verification</x:v>
@@ -44109,7 +44109,7 @@
         <x:v>OpenAlex</x:v>
       </x:c>
       <x:c r="AM15" t="str">
-        <x:v>2026-09-22</x:v>
+        <x:v>2026-09-23</x:v>
       </x:c>
       <x:c r="AN15" t="str">
         <x:v>LLMs have semantic knowledge but no embodiment grounding.</x:v>
@@ -44154,7 +44154,7 @@
         <x:v>Planning errors, low-level execution, drawer manipulation, embodiment limits.</x:v>
       </x:c>
       <x:c r="BB15" t="str">
-        <x:v>OpenAlex Work W4224912544</x:v>
+        <x:v>https://openalex.org/W4224912544</x:v>
       </x:c>
       <x:c r="BC15" t="str">
         <x:v>Google Research; arXiv; CoRL/PMLR; project page; official repository</x:v>
@@ -44231,7 +44231,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b540e7d6f794333"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reac433e9ea2f47c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Correct RoboCasa fulltext source metadata
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="Rf34e3ef76b4247fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R72e1a1bcb5f740e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R81f52f8342df421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R82d4680386654c31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R06b05290bbbe48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rf1c22db630ed47e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rb1f17bc3bb304c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R0692eb68bb314a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="Ra523ac2a0d98410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R2663c1e840cc4fd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rc9a5428bbbb4414d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R481916f3a87340d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R0a70830d5045435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="R0f837519acb64b12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -300,7 +300,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="74" name="PapersTable" displayName="PapersTable" ref="A1:CE6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="78" name="PapersTable" displayName="PapersTable" ref="A1:CE6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="83">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -436,7 +436,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="75" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BZ79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="79" name="DiscoveryTable" displayName="DiscoveryTable" ref="A1:BZ79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="78">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -522,7 +522,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="76" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CS67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="80" name="CCFALibraryTable" displayName="CCFALibraryTable" ref="A1:CS67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="97">
     <x:tableColumn id="1" name="编号 ID"/>
     <x:tableColumn id="2" name="论文标题 Title"/>
@@ -627,7 +627,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="77" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:CH15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="81" name="RoboticsCoreLibraryTable" displayName="RoboticsCoreLibraryTable" ref="A1:CH15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="86">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -5331,7 +5331,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f302552a21844f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ef4e32889f440e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8627,7 +8627,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f032058dcc948d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f9c45a596a24bf1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8978,7 +8978,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R785ce104cd4d4572"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R395670ce787f406d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9724,7 +9724,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af23533ecd0437a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84dd079b53594eaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26596,7 +26596,9 @@
       <x:c r="AY77" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="AZ77"/>
+      <x:c r="AZ77" t="str">
+        <x:v>https://www.roboticsproceedings.org/rss20/p050.pdf</x:v>
+      </x:c>
       <x:c r="BA77" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -26622,10 +26624,10 @@
         <x:v>Not Checked</x:v>
       </x:c>
       <x:c r="BI77" t="str">
-        <x:v>Not Found After Verification</x:v>
+        <x:v>Verified DOI</x:v>
       </x:c>
       <x:c r="BJ77" t="str">
-        <x:v>Not Found After Verification</x:v>
+        <x:v>Verified - 2406.02523</x:v>
       </x:c>
       <x:c r="BK77" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
@@ -27142,7 +27144,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbf8d6f51f124fa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc28476572740b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -46159,7 +46161,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74c9fd2cd0fb4e26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd374438b095542f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49327,7 +49329,9 @@
       <x:c r="BG13" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="BH13"/>
+      <x:c r="BH13" t="str">
+        <x:v>https://www.roboticsproceedings.org/rss20/p050.pdf</x:v>
+      </x:c>
       <x:c r="BI13" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -49353,10 +49357,10 @@
         <x:v>Not Checked</x:v>
       </x:c>
       <x:c r="BQ13" t="str">
-        <x:v>Not Found After Verification</x:v>
+        <x:v>Verified DOI</x:v>
       </x:c>
       <x:c r="BR13" t="str">
-        <x:v>Not Found After Verification</x:v>
+        <x:v>Verified - 2406.02523</x:v>
       </x:c>
       <x:c r="BS13" t="str">
         <x:v>Audit logged - deep extraction pending</x:v>
@@ -49902,7 +49906,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b6f9198ed0e4d4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa19e8e776f4a68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add verified citation provenance and Crossref matches
</commit_message>
<xml_diff>
--- a/00_Paper_Pool/Paper_Pool.xlsx
+++ b/00_Paper_Pool/Paper_Pool.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R455e651720dc49ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R2c325815a6814582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R6c1f97ee8ee84a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R3e423bf7e23340ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R7611a26cf679499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="R85d867a1d6ff4ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rb9ade8676bc74cde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Papers" sheetId="1" r:id="R4fff0bbbd5524283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejected" sheetId="2" r:id="R0a35edba35584f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="3" r:id="R17e394ab109844dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="Rda2a3df3953148e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery" sheetId="5" r:id="R9935fa90070b4ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CCF_A_Library" sheetId="6" r:id="Rb5e3b09fca084827"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robotics_Core_Library" sheetId="7" r:id="Rffe694cc3ed04401"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -352,7 +352,7 @@
     <x:tableColumn id="48" name="Idea Clues"/>
     <x:tableColumn id="49" name="Ablation Study"/>
     <x:tableColumn id="50" name="Failure Cases"/>
-    <x:tableColumn id="51" name="Citation Source Identifier"/>
+    <x:tableColumn id="51" name="引用量来源链接"/>
     <x:tableColumn id="52" name="Evidence Sources"/>
     <x:tableColumn id="53" name="Evidence Upgrade Status"/>
     <x:tableColumn id="54" name="Supplement Status"/>
@@ -483,7 +483,7 @@
     <x:tableColumn id="43" name="Idea Clues"/>
     <x:tableColumn id="44" name="Ablation Study"/>
     <x:tableColumn id="45" name="Failure Cases"/>
-    <x:tableColumn id="46" name="Citation Source Identifier"/>
+    <x:tableColumn id="46" name="引用量来源链接"/>
     <x:tableColumn id="47" name="Evidence Sources"/>
     <x:tableColumn id="48" name="Evidence Upgrade Status"/>
     <x:tableColumn id="49" name="Supplement Status"/>
@@ -588,7 +588,7 @@
     <x:tableColumn id="62" name="Idea Clues"/>
     <x:tableColumn id="63" name="Ablation Study"/>
     <x:tableColumn id="64" name="Failure Cases"/>
-    <x:tableColumn id="65" name="Citation Source Identifier"/>
+    <x:tableColumn id="65" name="引用量来源链接"/>
     <x:tableColumn id="66" name="Evidence Sources"/>
     <x:tableColumn id="67" name="Evidence Upgrade Status"/>
     <x:tableColumn id="68" name="Supplement Status"/>
@@ -682,7 +682,7 @@
     <x:tableColumn id="51" name="Idea Clues"/>
     <x:tableColumn id="52" name="Ablation Study"/>
     <x:tableColumn id="53" name="Failure Cases"/>
-    <x:tableColumn id="54" name="Citation Source Identifier"/>
+    <x:tableColumn id="54" name="引用量来源链接"/>
     <x:tableColumn id="55" name="Evidence Sources"/>
     <x:tableColumn id="56" name="Evidence Upgrade Status"/>
     <x:tableColumn id="57" name="Supplement Status"/>
@@ -1100,7 +1100,7 @@
         <x:v>Failure Cases</x:v>
       </x:c>
       <x:c r="AY1" t="str">
-        <x:v>Citation Source Identifier</x:v>
+        <x:v>引用量来源链接</x:v>
       </x:c>
       <x:c r="AZ1" t="str">
         <x:v>Evidence Sources</x:v>
@@ -1349,9 +1349,8 @@
       <x:c r="AX2" t="str">
         <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
       </x:c>
-      <x:c r="AY2" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402727730","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402727730, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AY2" t="str">
+        <x:v>https://openalex.org/W4402727730</x:v>
       </x:c>
       <x:c r="AZ2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -1565,9 +1564,8 @@
       <x:c r="AX3" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AY3" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145126","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145126, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AY3" t="str">
+        <x:v>https://openalex.org/W4413145126</x:v>
       </x:c>
       <x:c r="AZ3" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -1777,9 +1775,8 @@
       <x:c r="AX4" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AY4" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413146641","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413146641, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AY4" t="str">
+        <x:v>https://openalex.org/W4413146641</x:v>
       </x:c>
       <x:c r="AZ4" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
@@ -1989,9 +1986,8 @@
       <x:c r="AX5" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AY5" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4416242580","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4416242580, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AY5" t="str">
+        <x:v>https://openalex.org/W4416242580</x:v>
       </x:c>
       <x:c r="AZ5" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -2233,9 +2229,8 @@
       <x:c r="AX6" t="str">
         <x:v>Plan-execute gap; wrong object/negation; drawer manipulation and incomplete close; embodiment-specific failures.</x:v>
       </x:c>
-      <x:c r="AY6" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4224912544","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4224912544, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AY6" t="str">
+        <x:v>https://openalex.org/W4224912544</x:v>
       </x:c>
       <x:c r="AZ6" t="str">
         <x:v>Google Research publication; arXiv HTML 2204.01691; CoRL/PMLR; say-can.github.io; Google Research blog; official google-research/saycan</x:v>
@@ -5347,7 +5342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3e2febbcb5242ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R250b431c1f83454a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8643,7 +8638,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb608bc10d0fa447a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75b6a4d8846b4732"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8994,7 +8989,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R539a3dd3fcb640f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R632ee644304a4e73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9740,7 +9735,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b0bea9668e9461b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f371f007e7c4788"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9917,7 +9912,7 @@
         <x:v>Failure Cases</x:v>
       </x:c>
       <x:c r="AT1" t="str">
-        <x:v>Citation Source Identifier</x:v>
+        <x:v>引用量来源链接</x:v>
       </x:c>
       <x:c r="AU1" t="str">
         <x:v>Evidence Sources</x:v>
@@ -10143,9 +10138,8 @@
       <x:c r="AS2" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT2" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402727783","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402727783, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT2" t="str">
+        <x:v>https://openalex.org/W4402727783</x:v>
       </x:c>
       <x:c r="AU2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -10365,9 +10359,8 @@
       <x:c r="AS3" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT3" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415101881","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415101881, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT3" t="str">
+        <x:v>https://openalex.org/W4415101881</x:v>
       </x:c>
       <x:c r="AU3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -10587,9 +10580,8 @@
       <x:c r="AS4" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT4" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414754983","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414754983, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT4" t="str">
+        <x:v>https://openalex.org/W4414754983</x:v>
       </x:c>
       <x:c r="AU4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -10897,7 +10889,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2025/hash/e19b6f65791e350347bcff8a3955cb5b-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX5" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY5" t="n">
         <x:v>0</x:v>
@@ -11033,9 +11025,8 @@
       <x:c r="AS6" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT6" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4403883977","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4403883977, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT6" t="str">
+        <x:v>https://openalex.org/W4403883977</x:v>
       </x:c>
       <x:c r="AU6" t="str">
         <x:v>Unknown</x:v>
@@ -11340,7 +11331,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2025/hash/e68274fc4f158dbcbd4dddc672f7ee9c-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX7" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY7" t="n">
         <x:v>0</x:v>
@@ -11474,9 +11465,8 @@
       <x:c r="AS8" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT8" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4407590583","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4407590583, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT8" t="str">
+        <x:v>https://openalex.org/W4407590583</x:v>
       </x:c>
       <x:c r="AU8" t="str">
         <x:v>Unknown</x:v>
@@ -11781,7 +11771,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2025/hash/6eed1e1d5ed52deee53234786998245e-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX9" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY9" t="n">
         <x:v>0</x:v>
@@ -12000,7 +11990,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2025/hash/9cd0c57170f48520749d5ae62838241f-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX10" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY10" t="n">
         <x:v>0</x:v>
@@ -12139,9 +12129,8 @@
       <x:c r="AS11" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT11" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4407384835","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4407384835, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT11" t="str">
+        <x:v>https://openalex.org/W4407384835</x:v>
       </x:c>
       <x:c r="AU11" t="str">
         <x:v>Unknown</x:v>
@@ -12364,9 +12353,8 @@
       <x:c r="AS12" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT12" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4404371741","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4404371741, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT12" t="str">
+        <x:v>https://openalex.org/W4404371741</x:v>
       </x:c>
       <x:c r="AU12" t="str">
         <x:v>Unknown</x:v>
@@ -12589,9 +12577,8 @@
       <x:c r="AS13" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT13" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4403525052","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4403525052, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT13" t="str">
+        <x:v>https://openalex.org/W4403525052</x:v>
       </x:c>
       <x:c r="AU13" t="str">
         <x:v>Unknown</x:v>
@@ -12811,9 +12798,8 @@
       <x:c r="AS14" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT14" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4405626335","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4405626335, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT14" t="str">
+        <x:v>https://openalex.org/W4405626335</x:v>
       </x:c>
       <x:c r="AU14" t="str">
         <x:v>Unknown</x:v>
@@ -13121,7 +13107,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2026/hash/122ea6470232ee5e79a2649243348005-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX15" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY15" t="n">
         <x:v>0</x:v>
@@ -13255,9 +13241,8 @@
       <x:c r="AS16" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT16" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417536563","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417536563, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT16" t="str">
+        <x:v>https://openalex.org/W4417536563</x:v>
       </x:c>
       <x:c r="AU16" t="str">
         <x:v>Unknown</x:v>
@@ -13560,7 +13545,7 @@
         <x:v>官方摘要/论文页; https://arxiv.org/html/2509.09674; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX17" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY17" t="n">
         <x:v>6</x:v>
@@ -13779,7 +13764,7 @@
         <x:v>官方摘要/论文页; https://arxiv.org/html/2509.22195; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX18" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY18" t="n">
         <x:v>8</x:v>
@@ -13915,9 +13900,8 @@
       <x:c r="AS19" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT19" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7126041108","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7126041108, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT19" t="str">
+        <x:v>https://openalex.org/W7126041108</x:v>
       </x:c>
       <x:c r="AU19" t="str">
         <x:v>Unknown</x:v>
@@ -14220,7 +14204,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2026/hash/cd96cb9a239c37b39dbf34f3f5a4c56f-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX20" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY20" t="n">
         <x:v>0</x:v>
@@ -14356,9 +14340,8 @@
       <x:c r="AS21" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT21" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138268695","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138268695, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT21" t="str">
+        <x:v>https://openalex.org/W7138268695</x:v>
       </x:c>
       <x:c r="AU21" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
@@ -14578,9 +14561,8 @@
       <x:c r="AS22" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT22" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138377383","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138377383, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT22" t="str">
+        <x:v>https://openalex.org/W7138377383</x:v>
       </x:c>
       <x:c r="AU22" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
@@ -14800,9 +14782,8 @@
       <x:c r="AS23" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT23" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138167694","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138167694, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT23" t="str">
+        <x:v>https://openalex.org/W7138167694</x:v>
       </x:c>
       <x:c r="AU23" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
@@ -15022,9 +15003,8 @@
       <x:c r="AS24" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT24" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4416716605","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4416716605, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT24" t="str">
+        <x:v>https://openalex.org/W4416716605</x:v>
       </x:c>
       <x:c r="AU24" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
@@ -15187,11 +15167,11 @@
       <x:c r="Z25" t="str">
         <x:v>02_Papers/04_Dexterous/Learning_Object-Centric_Motion_Priors_from_Human_for_Robotic_Dexterous_Manipulation.md</x:v>
       </x:c>
-      <x:c r="AA25" t="str">
-        <x:v>—</x:v>
+      <x:c r="AA25" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AB25" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AC25" t="str">
         <x:v>2026-09-25</x:v>
@@ -15243,7 +15223,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT25" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1609/aaai.v40i22.38892</x:v>
       </x:c>
       <x:c r="AU25" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
@@ -15285,7 +15265,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BH25" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BI25" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -15327,7 +15307,7 @@
         <x:v>官方摘要/论文页：https://ojs.aaai.org/index.php/AAAI/article/view/38892；核验于 2026-09-23。仅为摘要级速读，原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX25" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="BY25" t="n">
         <x:v>0</x:v>
@@ -15463,9 +15443,8 @@
       <x:c r="AS26" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT26" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4404312247","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4404312247, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT26" t="str">
+        <x:v>https://openalex.org/W4404312247</x:v>
       </x:c>
       <x:c r="AU26" t="str">
         <x:v>Unknown</x:v>
@@ -15685,9 +15664,8 @@
       <x:c r="AS27" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT27" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4403622102","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4403622102, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT27" t="str">
+        <x:v>https://openalex.org/W4403622102</x:v>
       </x:c>
       <x:c r="AU27" t="str">
         <x:v>Unknown</x:v>
@@ -15907,9 +15885,8 @@
       <x:c r="AS28" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT28" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4404308601","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4404308601, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT28" t="str">
+        <x:v>https://openalex.org/W4404308601</x:v>
       </x:c>
       <x:c r="AU28" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
@@ -16129,9 +16106,8 @@
       <x:c r="AS29" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT29" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4392781441","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4392781441, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT29" t="str">
+        <x:v>https://openalex.org/W4392781441</x:v>
       </x:c>
       <x:c r="AU29" t="str">
         <x:v>Unknown</x:v>
@@ -16351,9 +16327,8 @@
       <x:c r="AS30" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT30" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400435236","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400435236, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT30" t="str">
+        <x:v>https://openalex.org/W4400435236</x:v>
       </x:c>
       <x:c r="AU30" t="str">
         <x:v>Unknown</x:v>
@@ -16658,7 +16633,7 @@
         <x:v>OpenAlex 索引摘要; https://api.openalex.org/works/W4400222297; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX31" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY31" t="n">
         <x:v>0</x:v>
@@ -16794,9 +16769,8 @@
       <x:c r="AS32" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT32" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400024954","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400024954, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT32" t="str">
+        <x:v>https://openalex.org/W4400024954</x:v>
       </x:c>
       <x:c r="AU32" t="str">
         <x:v>Unknown</x:v>
@@ -17016,9 +16990,8 @@
       <x:c r="AS33" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT33" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400377647","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400377647, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT33" t="str">
+        <x:v>https://openalex.org/W4400377647</x:v>
       </x:c>
       <x:c r="AU33" t="str">
         <x:v>Unknown</x:v>
@@ -17238,9 +17211,8 @@
       <x:c r="AS34" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT34" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400373516","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400373516, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT34" t="str">
+        <x:v>https://openalex.org/W4400373516</x:v>
       </x:c>
       <x:c r="AU34" t="str">
         <x:v>Unknown</x:v>
@@ -17460,9 +17432,8 @@
       <x:c r="AS35" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT35" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4391949089","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4391949089, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT35" t="str">
+        <x:v>https://openalex.org/W4391949089</x:v>
       </x:c>
       <x:c r="AU35" t="str">
         <x:v>Unknown</x:v>
@@ -17682,9 +17653,8 @@
       <x:c r="AS36" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT36" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400611211","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400611211, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT36" t="str">
+        <x:v>https://openalex.org/W4400611211</x:v>
       </x:c>
       <x:c r="AU36" t="str">
         <x:v>Unknown</x:v>
@@ -17904,9 +17874,8 @@
       <x:c r="AS37" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT37" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4400434472","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4400434472, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT37" t="str">
+        <x:v>https://openalex.org/W4400434472</x:v>
       </x:c>
       <x:c r="AU37" t="str">
         <x:v>Unknown</x:v>
@@ -18211,7 +18180,7 @@
         <x:v>官方摘要/论文页; https://proceedings.mlr.press/v270/fu25b.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX38" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY38" t="n">
         <x:v>0</x:v>
@@ -18347,9 +18316,8 @@
       <x:c r="AS39" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT39" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4403579180","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4403579180, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT39" t="str">
+        <x:v>https://openalex.org/W4403579180</x:v>
       </x:c>
       <x:c r="AU39" t="str">
         <x:v>https://proceedings.mlr.press/v270/</x:v>
@@ -18567,9 +18535,8 @@
       <x:c r="AS40" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT40" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414991924","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414991924, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT40" t="str">
+        <x:v>https://openalex.org/W4414991924</x:v>
       </x:c>
       <x:c r="AU40" t="str">
         <x:v>Unknown</x:v>
@@ -18872,7 +18839,7 @@
         <x:v>官方摘要/论文页; https://proceedings.mlr.press/v305/deng25c.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX41" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY41" t="n">
         <x:v>0</x:v>
@@ -19006,9 +18973,8 @@
       <x:c r="AS42" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT42" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4407569722","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4407569722, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT42" t="str">
+        <x:v>https://openalex.org/W4407569722</x:v>
       </x:c>
       <x:c r="AU42" t="str">
         <x:v>Unknown</x:v>
@@ -19311,7 +19277,7 @@
         <x:v>官方摘要/论文页; https://proceedings.mlr.press/v305/lin25c.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX43" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY43" t="n">
         <x:v>0</x:v>
@@ -19530,7 +19496,7 @@
         <x:v>OpenAlex 索引摘要; https://api.openalex.org/works/W4416623172; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX44" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY44" t="n">
         <x:v>0</x:v>
@@ -19749,7 +19715,7 @@
         <x:v>官方摘要/论文页; https://arxiv.org/html/2506.17811; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX45" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY45" t="n">
         <x:v>5</x:v>
@@ -19885,9 +19851,8 @@
       <x:c r="AS46" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT46" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/ae9a2bcd460354c706aaea8797b1c2c15841a6b6","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/ae9a2bcd460354c706aaea8797b1c2c15841a6b6, friendlyName=Semantic Scholar</x:v>
+      <x:c r="AT46" t="str">
+        <x:v>https://www.semanticscholar.org/paper/ae9a2bcd460354c706aaea8797b1c2c15841a6b6</x:v>
       </x:c>
       <x:c r="AU46" t="str">
         <x:v>Unknown</x:v>
@@ -20107,9 +20072,8 @@
       <x:c r="AS47" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT47" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417042701","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417042701, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT47" t="str">
+        <x:v>https://openalex.org/W4417042701</x:v>
       </x:c>
       <x:c r="AU47" t="str">
         <x:v>Unknown</x:v>
@@ -20274,11 +20238,11 @@
       <x:c r="Z48" t="str">
         <x:v>02_Papers/09_Survey_Review/What_Foundation_Models_can_Bring_for_Robot_Learning_in_Manipulation_A_Survey.md</x:v>
       </x:c>
-      <x:c r="AA48" t="str">
-        <x:v>—</x:v>
+      <x:c r="AA48" t="n">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="AB48" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AC48" t="str">
         <x:v>2026-09-25</x:v>
@@ -20330,7 +20294,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT48" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1177/02783649251390579</x:v>
       </x:c>
       <x:c r="AU48" t="str">
         <x:v>Unknown</x:v>
@@ -20372,7 +20336,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BH48" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BI48" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -20414,7 +20378,7 @@
         <x:v>OpenAlex 索引摘要; https://api.openalex.org/works/W4416422407; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX48" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="BY48" t="n">
         <x:v>0</x:v>
@@ -20550,9 +20514,8 @@
       <x:c r="AS49" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT49" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4391590994","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4391590994, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT49" t="str">
+        <x:v>https://openalex.org/W4391590994</x:v>
       </x:c>
       <x:c r="AU49" t="str">
         <x:v>Unknown</x:v>
@@ -20772,9 +20735,8 @@
       <x:c r="AS50" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT50" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4391800778","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4391800778, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT50" t="str">
+        <x:v>https://openalex.org/W4391800778</x:v>
       </x:c>
       <x:c r="AU50" t="str">
         <x:v>Unknown</x:v>
@@ -20994,9 +20956,8 @@
       <x:c r="AS51" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT51" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4390962508","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4390962508, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT51" t="str">
+        <x:v>https://openalex.org/W4390962508</x:v>
       </x:c>
       <x:c r="AU51" t="str">
         <x:v>Unknown</x:v>
@@ -21299,7 +21260,7 @@
         <x:v>OpenAlex 索引摘要; https://api.openalex.org/works/W4409168415; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX52" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY52" t="n">
         <x:v>1</x:v>
@@ -21380,11 +21341,11 @@
       <x:c r="Z53" t="str">
         <x:v>02_Papers/09_Survey_Review/A_Survey_of_Embodied_Learning_for_Object-Centric_Robotic_Manipulation.md</x:v>
       </x:c>
-      <x:c r="AA53" t="str">
-        <x:v>—</x:v>
+      <x:c r="AA53" t="n">
+        <x:v>20</x:v>
       </x:c>
       <x:c r="AB53" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AC53" t="str">
         <x:v>2026-09-25</x:v>
@@ -21436,7 +21397,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT53" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1007/s11633-025-1542-8</x:v>
       </x:c>
       <x:c r="AU53" t="str">
         <x:v>Unknown</x:v>
@@ -21478,7 +21439,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BH53" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BI53" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -21520,7 +21481,7 @@
         <x:v>官方摘要/论文页; https://link.springer.com/article/10.1007/s11633-025-1542-8; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX53" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="BY53" t="n">
         <x:v>3</x:v>
@@ -21656,9 +21617,8 @@
       <x:c r="AS54" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT54" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414888151","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414888151, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT54" t="str">
+        <x:v>https://openalex.org/W4414888151</x:v>
       </x:c>
       <x:c r="AU54" t="str">
         <x:v>Unknown</x:v>
@@ -21961,7 +21921,7 @@
         <x:v>Existing canonical card and official-paper metadata; abstract unavailable; https://github.com/Destiny000621/awesome-bimanual-robot-learning/blob/main/SURVEY.md; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：证据有限；不得视为全文核验</x:v>
       </x:c>
       <x:c r="BX55" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY55" t="n">
         <x:v>0</x:v>
@@ -22097,9 +22057,8 @@
       <x:c r="AS56" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT56" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/9702a6cce93fbff83dbdad83ae74a3180eb47622","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/9702a6cce93fbff83dbdad83ae74a3180eb47622, friendlyName=Semantic Scholar</x:v>
+      <x:c r="AT56" t="str">
+        <x:v>https://www.semanticscholar.org/paper/9702a6cce93fbff83dbdad83ae74a3180eb47622</x:v>
       </x:c>
       <x:c r="AU56" t="str">
         <x:v>Unknown</x:v>
@@ -22319,9 +22278,8 @@
       <x:c r="AS57" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT57" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402510263","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402510263, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT57" t="str">
+        <x:v>https://openalex.org/W4402510263</x:v>
       </x:c>
       <x:c r="AU57" t="str">
         <x:v>Unknown</x:v>
@@ -22549,9 +22507,8 @@
       <x:c r="AS58" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT58" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4403364995","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4403364995, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT58" t="str">
+        <x:v>https://openalex.org/W4403364995</x:v>
       </x:c>
       <x:c r="AU58" t="str">
         <x:v>Unknown</x:v>
@@ -22779,9 +22736,8 @@
       <x:c r="AS59" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT59" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7104616842","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7104616842, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT59" t="str">
+        <x:v>https://openalex.org/W7104616842</x:v>
       </x:c>
       <x:c r="AU59" t="str">
         <x:v>Unknown</x:v>
@@ -22952,11 +22908,11 @@
       <x:c r="Z60" t="str">
         <x:v>02_Papers/10_Benchmark_Dataset/RoboTwin.md</x:v>
       </x:c>
-      <x:c r="AA60" t="str">
-        <x:v>—</x:v>
+      <x:c r="AA60" t="n">
+        <x:v>28</x:v>
       </x:c>
       <x:c r="AB60" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AC60" t="str">
         <x:v>2026-09-25</x:v>
@@ -23008,7 +22964,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="AT60" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52734.2025.02575</x:v>
       </x:c>
       <x:c r="AU60" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -23050,7 +23006,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BH60" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BI60" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -23092,7 +23048,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX60" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="BY60" t="n">
         <x:v>0</x:v>
@@ -23236,9 +23192,8 @@
       <x:c r="AS61" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT61" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415272059","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415272059, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT61" t="str">
+        <x:v>https://openalex.org/W4415272059</x:v>
       </x:c>
       <x:c r="AU61" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -23471,9 +23426,8 @@
       <x:c r="AS62" t="str">
         <x:v>背景动态使基线 PickPot SR 95→80%；VLA-Cache 在动态条件保持80%且降低FLOPs/延迟；PickPot 真机SR 95→90%（Table 5,7）。</x:v>
       </x:c>
-      <x:c r="AT62" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196930033","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196930033, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT62" t="str">
+        <x:v>https://openalex.org/W7196930033</x:v>
       </x:c>
       <x:c r="AU62" t="str">
         <x:v>NeurIPS 正式论文页；arXiv PDF §1–6、Appendix A–F、Tables 1–5、7–11；NeurIPS Supplemental zip 与作者 GitHub。</x:v>
@@ -23789,7 +23743,7 @@
         <x:v>官方摘要/论文页; https://proceedings.mlr.press/v267/wen25g.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX63" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY63" t="n">
         <x:v>8</x:v>
@@ -23938,9 +23892,8 @@
       <x:c r="AS64" t="str">
         <x:v>§6：目标生成可能改变纹理/形状、令物体消失、预测不相关的未来或状态无变化；小物体精细操作失败。</x:v>
       </x:c>
-      <x:c r="AT64" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4392886475","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4392886475, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT64" t="str">
+        <x:v>https://openalex.org/W4392886475</x:v>
       </x:c>
       <x:c r="AU64" t="str">
         <x:v>PMLR 官方 PDF：§3.1–3.3、§4.1–4.3、§5.1–5.3、§6–7；Figures 2–3、5–6；Tables 1–6、Appendix Tables 7–9。https://raw.githubusercontent.com/mlresearch/v235/main/assets/zhen24a/zhen24a.pdf</x:v>
@@ -24175,9 +24128,8 @@
       <x:c r="AS65" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT65" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415797921","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415797921, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT65" t="str">
+        <x:v>https://openalex.org/W4415797921</x:v>
       </x:c>
       <x:c r="AU65" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
@@ -24405,9 +24357,8 @@
       <x:c r="AS66" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT66" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4405434146","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4405434146, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT66" t="str">
+        <x:v>https://openalex.org/W4405434146</x:v>
       </x:c>
       <x:c r="AU66" t="str">
         <x:v>Unknown</x:v>
@@ -24720,7 +24671,7 @@
         <x:v>官方摘要/论文页; https://proceedings.iclr.cc/paper_files/paper/2025/hash/45d74e190008c7bff2845ffc8e3facd3-Abstract-Conference.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="BX67" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="BY67" t="n">
         <x:v>0</x:v>
@@ -24861,9 +24812,8 @@
       <x:c r="AS68" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT68" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4409365031","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4409365031, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT68" t="str">
+        <x:v>https://openalex.org/W4409365031</x:v>
       </x:c>
       <x:c r="AU68" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
@@ -25091,9 +25041,8 @@
       <x:c r="AS69" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT69" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145029","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145029, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT69" t="str">
+        <x:v>https://openalex.org/W4413145029</x:v>
       </x:c>
       <x:c r="AU69" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -25321,9 +25270,8 @@
       <x:c r="AS70" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT70" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414683599","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414683599, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT70" t="str">
+        <x:v>https://openalex.org/W4414683599</x:v>
       </x:c>
       <x:c r="AU70" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -25551,9 +25499,8 @@
       <x:c r="AS71" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT71" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196952124","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196952124, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT71" t="str">
+        <x:v>https://openalex.org/W7196952124</x:v>
       </x:c>
       <x:c r="AU71" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -25781,9 +25728,8 @@
       <x:c r="AS72" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT72" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7125566978","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7125566978, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT72" t="str">
+        <x:v>https://openalex.org/W7125566978</x:v>
       </x:c>
       <x:c r="AU72" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -26011,9 +25957,8 @@
       <x:c r="AS73" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT73" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414051092","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414051092, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT73" t="str">
+        <x:v>https://openalex.org/W4414051092</x:v>
       </x:c>
       <x:c r="AU73" t="str">
         <x:v>Unknown</x:v>
@@ -26241,9 +26186,8 @@
       <x:c r="AS74" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT74" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4399695759","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4399695759, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT74" t="str">
+        <x:v>https://openalex.org/W4399695759</x:v>
       </x:c>
       <x:c r="AU74" t="str">
         <x:v>Unknown</x:v>
@@ -26471,9 +26415,8 @@
       <x:c r="AS75" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT75" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402353985","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402353985, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT75" t="str">
+        <x:v>https://openalex.org/W4402353985</x:v>
       </x:c>
       <x:c r="AU75" t="str">
         <x:v>Unknown</x:v>
@@ -26696,9 +26639,8 @@
       <x:c r="AS76" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT76" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402354047","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402354047, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT76" t="str">
+        <x:v>https://openalex.org/W4402354047</x:v>
       </x:c>
       <x:c r="AU76" t="str">
         <x:v>Unknown</x:v>
@@ -26927,9 +26869,8 @@
       <x:c r="AS77" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT77" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632, friendlyName=Semantic Scholar</x:v>
+      <x:c r="AT77" t="str">
+        <x:v>https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632</x:v>
       </x:c>
       <x:c r="AU77" t="str">
         <x:v>Unknown</x:v>
@@ -27154,9 +27095,8 @@
       <x:c r="AS78" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="AT78" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4387764390","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4387764390, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT78" t="str">
+        <x:v>https://openalex.org/W4387764390</x:v>
       </x:c>
       <x:c r="AU78" t="str">
         <x:v>Unknown</x:v>
@@ -27389,9 +27329,8 @@
       <x:c r="AS79" t="str">
         <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
       </x:c>
-      <x:c r="AT79" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7137985120","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7137985120, friendlyName=OpenAlex Work</x:v>
+      <x:c r="AT79" t="str">
+        <x:v>https://openalex.org/W7137985120</x:v>
       </x:c>
       <x:c r="AU79" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
@@ -27508,7 +27447,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc37a0a8c536b4386"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1026b7fa96694510"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27763,7 +27702,7 @@
         <x:v>Failure Cases</x:v>
       </x:c>
       <x:c r="BM1" t="str">
-        <x:v>Citation Source Identifier</x:v>
+        <x:v>引用量来源链接</x:v>
       </x:c>
       <x:c r="BN1" t="str">
         <x:v>Evidence Sources</x:v>
@@ -28046,9 +27985,8 @@
       <x:c r="BL2" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM2" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402727783","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402727783, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM2" t="str">
+        <x:v>https://openalex.org/W4402727783</x:v>
       </x:c>
       <x:c r="BN2" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Ma_Hierarchical_Diffusion_Policy_for_Kinematics-Aware_Multi-Task_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -28325,9 +28263,8 @@
       <x:c r="BL3" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM3" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415101881","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415101881, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM3" t="str">
+        <x:v>https://openalex.org/W4415101881</x:v>
       </x:c>
       <x:c r="BN3" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Jiang_Rethinking_Bimanual_Robotic_Manipulation_Learning_with_Decoupled_Interaction_Framework_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -28604,9 +28541,8 @@
       <x:c r="BL4" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM4" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414754983","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414754983, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM4" t="str">
+        <x:v>https://openalex.org/W4414754983</x:v>
       </x:c>
       <x:c r="BN4" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Xu_Diffusion-Based_Imaginative_Coordination_for_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -28883,9 +28819,8 @@
       <x:c r="BL5" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM5" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138268695","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138268695, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM5" t="str">
+        <x:v>https://openalex.org/W7138268695</x:v>
       </x:c>
       <x:c r="BN5" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38889；官方摘要/论文集元数据</x:v>
@@ -29162,9 +29097,8 @@
       <x:c r="BL6" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM6" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138377383","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138377383, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM6" t="str">
+        <x:v>https://openalex.org/W7138377383</x:v>
       </x:c>
       <x:c r="BN6" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38911；官方摘要/论文集元数据</x:v>
@@ -29441,9 +29375,8 @@
       <x:c r="BL7" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM7" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138167694","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138167694, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM7" t="str">
+        <x:v>https://openalex.org/W7138167694</x:v>
       </x:c>
       <x:c r="BN7" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38955；官方摘要/论文集元数据</x:v>
@@ -29720,9 +29653,8 @@
       <x:c r="BL8" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM8" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4416716605","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4416716605, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM8" t="str">
+        <x:v>https://openalex.org/W4416716605</x:v>
       </x:c>
       <x:c r="BN8" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38539；官方摘要/论文集元数据</x:v>
@@ -29945,11 +29877,11 @@
       <x:c r="AT9" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AU9" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU9" t="n">
+        <x:v>0</x:v>
       </x:c>
       <x:c r="AV9" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW9" t="str">
         <x:v>2026-09-25</x:v>
@@ -29998,7 +29930,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM9" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1609/aaai.v40i22.38892</x:v>
       </x:c>
       <x:c r="BN9" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/download/38892/42854；官方摘要/论文集元数据</x:v>
@@ -30040,7 +29972,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA9" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB9" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -30082,7 +30014,7 @@
         <x:v>官方摘要/论文页：https://ojs.aaai.org/index.php/AAAI/article/view/38892；核验于 2026-09-23。仅为摘要级速读，原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ9" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR9" t="n">
         <x:v>0</x:v>
@@ -30229,11 +30161,11 @@
       <x:c r="AT10" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AU10" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU10" t="n">
+        <x:v>28</x:v>
       </x:c>
       <x:c r="AV10" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW10" t="str">
         <x:v>2026-09-25</x:v>
@@ -30282,7 +30214,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM10" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52734.2025.02575</x:v>
       </x:c>
       <x:c r="BN10" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -30324,7 +30256,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB10" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -30366,7 +30298,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Mu_RoboTwin_Dual-Arm_Robot_Benchmark_with_Generative_Digital_Twins_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ10" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR10" t="n">
         <x:v>0</x:v>
@@ -30568,9 +30500,8 @@
       <x:c r="BL11" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM11" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415272059","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415272059, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM11" t="str">
+        <x:v>https://openalex.org/W4415272059</x:v>
       </x:c>
       <x:c r="BN11" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/5c1a8aa04c1a2cf5013f28831870dafa-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -30861,9 +30792,8 @@
       <x:c r="BL12" t="str">
         <x:v>背景动态使基线 PickPot SR 95→80%；VLA-Cache 在动态条件保持80%且降低FLOPs/延迟；PickPot 真机SR 95→90%（Table 5,7）。</x:v>
       </x:c>
-      <x:c r="BM12" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196930033","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196930033, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM12" t="str">
+        <x:v>https://openalex.org/W7196930033</x:v>
       </x:c>
       <x:c r="BN12" t="str">
         <x:v>NeurIPS 正式论文页；arXiv PDF §1–6、Appendix A–F、Tables 1–5、7–11；NeurIPS Supplemental zip 与作者 GitHub。</x:v>
@@ -31236,7 +31166,7 @@
         <x:v>官方摘要/论文页; https://proceedings.mlr.press/v267/wen25g.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ13" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="CR13" t="n">
         <x:v>8</x:v>
@@ -31443,9 +31373,8 @@
       <x:c r="BL14" t="str">
         <x:v>§6：目标生成可能改变纹理/形状、令物体消失、预测不相关的未来或状态无变化；小物体精细操作失败。</x:v>
       </x:c>
-      <x:c r="BM14" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4392886475","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4392886475, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM14" t="str">
+        <x:v>https://openalex.org/W4392886475</x:v>
       </x:c>
       <x:c r="BN14" t="str">
         <x:v>PMLR 官方 PDF：§3.1–3.3、§4.1–4.3、§5.1–5.3、§6–7；Figures 2–3、5–6；Tables 1–6、Appendix Tables 7–9。https://raw.githubusercontent.com/mlresearch/v235/main/assets/zhen24a/zhen24a.pdf</x:v>
@@ -31738,9 +31667,8 @@
       <x:c r="BL15" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM15" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415797921","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415797921, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM15" t="str">
+        <x:v>https://openalex.org/W4415797921</x:v>
       </x:c>
       <x:c r="BN15" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/46a126492ea6fb87410e55a58df2e189-Abstract-Conference.html; https://sites.google.com/view/robomamba-web; https://github.com/lm</x:v>
@@ -32022,9 +31950,8 @@
       <x:c r="BL16" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM16" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4409365031","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4409365031, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM16" t="str">
+        <x:v>https://openalex.org/W4409365031</x:v>
       </x:c>
       <x:c r="BN16" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33617; https://github.com/</x:v>
@@ -32309,9 +32236,8 @@
       <x:c r="BL17" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM17" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145029","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145029, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM17" t="str">
+        <x:v>https://openalex.org/W4413145029</x:v>
       </x:c>
       <x:c r="BN17" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wang_UniGraspTransformer_Simplified_Policy_Distillation_for_Scalable_Dexterous_Robotic_Grasping_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -32597,9 +32523,8 @@
       <x:c r="BL18" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM18" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414683599","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414683599, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM18" t="str">
+        <x:v>https://openalex.org/W4414683599</x:v>
       </x:c>
       <x:c r="BN18" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/862644b156e51c35dea5a7446d640b14-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -32885,9 +32810,8 @@
       <x:c r="BL19" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM19" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196952124","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196952124, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM19" t="str">
+        <x:v>https://openalex.org/W7196952124</x:v>
       </x:c>
       <x:c r="BN19" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/89a3b655a8b68ae1c76b768152c9c19d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -33172,9 +33096,8 @@
       <x:c r="BL20" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM20" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7125566978","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7125566978, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM20" t="str">
+        <x:v>https://openalex.org/W7125566978</x:v>
       </x:c>
       <x:c r="BN20" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Lee_DextER_Language-driven_Dexterous_Grasp_Generation_with_Embodied_Reasoning_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -33463,9 +33386,8 @@
       <x:c r="BL21" t="str">
         <x:v>Position predictions are sensitive to lighting and texture domain gaps; suction cannot grasp non-smooth handles and short gripper geometry can cause collisions.</x:v>
       </x:c>
-      <x:c r="BM21" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402727730","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402727730, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM21" t="str">
+        <x:v>https://openalex.org/W4402727730</x:v>
       </x:c>
       <x:c r="BN21" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Li_ManipLLM_Embodied_Multimodal_Large_Language_Model_for_Object-Centric_Robotic_Manipulation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -33756,9 +33678,8 @@
       <x:c r="BL22" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM22" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145126","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145126, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM22" t="str">
+        <x:v>https://openalex.org/W4413145126</x:v>
       </x:c>
       <x:c r="BN22" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_ManipTrans_Efficient_Dexterous_Bimanual_Manipulation_Transfer_via_Residual_Learning_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -34045,9 +33966,8 @@
       <x:c r="BL23" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM23" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413146641","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413146641, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM23" t="str">
+        <x:v>https://openalex.org/W4413146641</x:v>
       </x:c>
       <x:c r="BN23" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Liang_DexHandDiff_Interaction-aware_Diffusion_Planning_for_Adaptive_Dexterous_Manipulation_CVPR_2025_paper.html; https://dexdiffuser.github.io/; https://github.com/Liang-</x:v>
@@ -34334,9 +34254,8 @@
       <x:c r="BL24" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM24" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4416242580","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4416242580, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM24" t="str">
+        <x:v>https://openalex.org/W4416242580</x:v>
       </x:c>
       <x:c r="BN24" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Yang_AR-VRM_Imitating_Human_Motions_for_Visual_Robot_Manipulation_with_Analogical_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -34622,9 +34541,8 @@
       <x:c r="BL25" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM25" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402816741","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402816741, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM25" t="str">
+        <x:v>https://openalex.org/W4402816741</x:v>
       </x:c>
       <x:c r="BN25" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Xu_Dexterous_Grasp_Transformer_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -34909,9 +34827,8 @@
       <x:c r="BL26" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM26" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W6967143107","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W6967143107, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM26" t="str">
+        <x:v>https://openalex.org/W6967143107</x:v>
       </x:c>
       <x:c r="BN26" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Wu_MoManipVLA_Transferring_Vision-language-action_Models_for_General_Mobile_Manipulation_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -35197,9 +35114,8 @@
       <x:c r="BL27" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM27" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415800339","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415800339, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM27" t="str">
+        <x:v>https://openalex.org/W4415800339</x:v>
       </x:c>
       <x:c r="BN27" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/ff887781480973bd3cb6026feb378d1e-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -35486,9 +35402,8 @@
       <x:c r="BL28" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM28" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/f344e82d0d4f5e97c3d6176fd4b953a8c6c72d45","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/f344e82d0d4f5e97c3d6176fd4b953a8c6c72d45, friendlyName=Semantic Scholar</x:v>
+      <x:c r="BM28" t="str">
+        <x:v>https://www.semanticscholar.org/paper/f344e82d0d4f5e97c3d6176fd4b953a8c6c72d45</x:v>
       </x:c>
       <x:c r="BN28" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/74c4f2b87b7499d365422152c76fd916-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -35775,9 +35690,8 @@
       <x:c r="BL29" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM29" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415795570","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415795570, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM29" t="str">
+        <x:v>https://openalex.org/W4415795570</x:v>
       </x:c>
       <x:c r="BN29" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/dcd297696d0bb304ba426b3c5a679c37-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36064,9 +35978,8 @@
       <x:c r="BL30" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM30" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415800541","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415800541, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM30" t="str">
+        <x:v>https://openalex.org/W4415800541</x:v>
       </x:c>
       <x:c r="BN30" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/fad8962279154544ed69bb63eb14d677-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36352,9 +36265,8 @@
       <x:c r="BL31" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM31" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415797227","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415797227, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM31" t="str">
+        <x:v>https://openalex.org/W4415797227</x:v>
       </x:c>
       <x:c r="BN31" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/8e5dc5969a6174fcaaececd890c7f59b-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -36640,9 +36552,8 @@
       <x:c r="BL32" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM32" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415797662","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415797662, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM32" t="str">
+        <x:v>https://openalex.org/W4415797662</x:v>
       </x:c>
       <x:c r="BN32" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/5227ce00add5aa0a12d1c4ee92fcd2dc-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -36927,9 +36838,8 @@
       <x:c r="BL33" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM33" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145391","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145391, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM33" t="str">
+        <x:v>https://openalex.org/W4413145391</x:v>
       </x:c>
       <x:c r="BN33" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -37214,9 +37124,8 @@
       <x:c r="BL34" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM34" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413147462","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413147462, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM34" t="str">
+        <x:v>https://openalex.org/W4413147462</x:v>
       </x:c>
       <x:c r="BN34" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Huang_RoboGround_Robotic_Manipulation_with_Grounded_Vision-Language_Priors_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -37449,11 +37358,11 @@
       <x:c r="AT35" t="str">
         <x:v>Data / Teleoperation</x:v>
       </x:c>
-      <x:c r="AU35" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU35" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AV35" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW35" t="str">
         <x:v>2026-09-25</x:v>
@@ -37502,7 +37411,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM35" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52734.2025.01136</x:v>
       </x:c>
       <x:c r="BN35" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -37544,7 +37453,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA35" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB35" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -37586,7 +37495,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Lee_DynScene_Scalable_Generation_of_Dynamic_Robotic_Manipulation_Scenes_for_Embodied_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ35" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR35" t="n">
         <x:v>0</x:v>
@@ -37735,11 +37644,11 @@
       <x:c r="AT36" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU36" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU36" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="AV36" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW36" t="str">
         <x:v>2026-09-25</x:v>
@@ -37788,7 +37697,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM36" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52734.2025.02102</x:v>
       </x:c>
       <x:c r="BN36" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Yao_Think_Small_Act_Big_Primitive_Prompt_Learning_for_Lifelong_Robot_CVPR_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -37830,7 +37739,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA36" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB36" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -37872,7 +37781,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Yao_Think_Small_Act_Big_Primitive_Prompt_Learning_for_Lifelong_Robot_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ36" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR36" t="n">
         <x:v>0</x:v>
@@ -38073,9 +37982,8 @@
       <x:c r="BL37" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM37" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4409362855","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4409362855, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM37" t="str">
+        <x:v>https://openalex.org/W4409362855</x:v>
       </x:c>
       <x:c r="BN37" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/34866；官方摘要/论文集元数据</x:v>
@@ -38360,9 +38268,8 @@
       <x:c r="BL38" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM38" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4409364627","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4409364627, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM38" t="str">
+        <x:v>https://openalex.org/W4409364627</x:v>
       </x:c>
       <x:c r="BN38" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33615；官方摘要/论文集元数据</x:v>
@@ -38647,9 +38554,8 @@
       <x:c r="BL39" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM39" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4409364594","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4409364594, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM39" t="str">
+        <x:v>https://openalex.org/W4409364594</x:v>
       </x:c>
       <x:c r="BN39" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/33610；官方摘要/论文集元数据</x:v>
@@ -38935,9 +38841,8 @@
       <x:c r="BL40" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM40" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7103754590","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7103754590, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM40" t="str">
+        <x:v>https://openalex.org/W7103754590</x:v>
       </x:c>
       <x:c r="BN40" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/481c70828a4ff20d31a646cc6cc95f3d-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -39307,7 +39212,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Chen_VidBot_Learning_Generalizable_3D_Actions_from_In-the-Wild_2D_Human_Videos_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ41" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="CR41" t="n">
         <x:v>0</x:v>
@@ -39508,9 +39413,8 @@
       <x:c r="BL42" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM42" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413156213","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413156213, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM42" t="str">
+        <x:v>https://openalex.org/W4413156213</x:v>
       </x:c>
       <x:c r="BN42" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -39796,9 +39700,8 @@
       <x:c r="BL43" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM43" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415251366","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415251366, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM43" t="str">
+        <x:v>https://openalex.org/W4415251366</x:v>
       </x:c>
       <x:c r="BN43" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1185c89347a3f21ffc48c9d083c9437c-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -40084,9 +39987,8 @@
       <x:c r="BL44" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM44" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196926233","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196926233, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM44" t="str">
+        <x:v>https://openalex.org/W7196926233</x:v>
       </x:c>
       <x:c r="BN44" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b94310e1c7ecb79f1a24adc757f1b89b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -40372,9 +40274,8 @@
       <x:c r="BL45" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM45" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7196975408","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7196975408, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM45" t="str">
+        <x:v>https://openalex.org/W7196975408</x:v>
       </x:c>
       <x:c r="BN45" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/49eadcc4a329fc6b74b9f8a82b78cbc3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -40660,9 +40561,8 @@
       <x:c r="BL46" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM46" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7197036842","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7197036842, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM46" t="str">
+        <x:v>https://openalex.org/W7197036842</x:v>
       </x:c>
       <x:c r="BN46" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/bc97207e3979d1cc23109db0be0e8ed2-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -40948,9 +40848,8 @@
       <x:c r="BL47" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM47" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417258107","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417258107, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM47" t="str">
+        <x:v>https://openalex.org/W4417258107</x:v>
       </x:c>
       <x:c r="BN47" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/282c3318be1b047b7bb5ba94fa4f3231-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -41236,9 +41135,8 @@
       <x:c r="BL48" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM48" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4415312722","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4415312722, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM48" t="str">
+        <x:v>https://openalex.org/W4415312722</x:v>
       </x:c>
       <x:c r="BN48" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/9fc291fef2f9607a46777d367f900a15-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -41524,9 +41422,8 @@
       <x:c r="BL49" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM49" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417082659","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417082659, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM49" t="str">
+        <x:v>https://openalex.org/W4417082659</x:v>
       </x:c>
       <x:c r="BN49" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/eacc8ae341d15d2c13c02fef88189db3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -41812,9 +41709,8 @@
       <x:c r="BL50" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM50" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/afeff85d95e5428eb0a36dbc58446ce42e686d1d","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/afeff85d95e5428eb0a36dbc58446ce42e686d1d, friendlyName=Semantic Scholar</x:v>
+      <x:c r="BM50" t="str">
+        <x:v>https://www.semanticscholar.org/paper/afeff85d95e5428eb0a36dbc58446ce42e686d1d</x:v>
       </x:c>
       <x:c r="BN50" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/1f467c3e37abf9f86c78f44c6a27ee7c-Abstract-Datasets_and_Benchmarks_Track.html；官方摘要/论文集元数据</x:v>
@@ -42100,9 +41996,8 @@
       <x:c r="BL51" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM51" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/31feae9cc3d888b85e1cba366c79b2c50f29c2b3","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/31feae9cc3d888b85e1cba366c79b2c50f29c2b3, friendlyName=Semantic Scholar</x:v>
+      <x:c r="BM51" t="str">
+        <x:v>https://www.semanticscholar.org/paper/31feae9cc3d888b85e1cba366c79b2c50f29c2b3</x:v>
       </x:c>
       <x:c r="BN51" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/b8358a00e5b870194b974ddf8dd415c3-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -42473,7 +42368,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/ICCV2025/html/Wang_DexH2R_A_Benchmark_for_Dynamic_Dexterous_Grasping_in_Human-to-Robot_Handover_ICCV_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ52" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="CR52" t="n">
         <x:v>0</x:v>
@@ -42674,9 +42569,8 @@
       <x:c r="BL53" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM53" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413145043","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413145043, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM53" t="str">
+        <x:v>https://openalex.org/W4413145043</x:v>
       </x:c>
       <x:c r="BN53" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -42964,9 +42858,8 @@
       <x:c r="BL54" t="str">
         <x:v>The reported setting focuses on tabletop part-aligned grasps; broader clutter, occlusion and multi-step manipulation are not established by the cited results.</x:v>
       </x:c>
-      <x:c r="BM54" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417183400","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417183400, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM54" t="str">
+        <x:v>https://openalex.org/W4417183400</x:v>
       </x:c>
       <x:c r="BN54" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/He_DexVLG_Dexterous_Vision-Language-Grasp_Model_at_Scale_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -43255,9 +43148,8 @@
       <x:c r="BL55" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM55" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4413146191","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4413146191, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM55" t="str">
+        <x:v>https://openalex.org/W4413146191</x:v>
       </x:c>
       <x:c r="BN55" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/Li_LatentHOI_On_the_Generali</x:v>
@@ -43490,11 +43382,11 @@
       <x:c r="AT56" t="str">
         <x:v>Benchmark / Dataset</x:v>
       </x:c>
-      <x:c r="AU56" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU56" t="n">
+        <x:v>37</x:v>
       </x:c>
       <x:c r="AV56" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW56" t="str">
         <x:v>2026-09-25</x:v>
@@ -43543,7 +43435,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM56" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52733.2024.02054</x:v>
       </x:c>
       <x:c r="BN56" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generali</x:v>
@@ -43585,7 +43477,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA56" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB56" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -43627,7 +43519,7 @@
         <x:v>官方摘要/论文页：https://openaccess.thecvf.com/content/CVPR2024/papers/Liu_TACO_Benchmarking_Generalizable_Bimanual_Tool-ACtion-Object_Understanding_CVPR_2024_paper.pdf；核验于 2026-09-23。仅为摘要级速读，原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ56" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR56" t="n">
         <x:v>0</x:v>
@@ -43829,9 +43721,8 @@
       <x:c r="BL57" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM57" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402772268","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402772268, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM57" t="str">
+        <x:v>https://openalex.org/W4402772268</x:v>
       </x:c>
       <x:c r="BN57" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Uppal_SPIN_Simultaneous_Perception_Interaction_and_Navigation_CVPR_2024_paper.html；官方摘要/论文集元数据</x:v>
@@ -44118,9 +44009,8 @@
       <x:c r="BL58" t="str">
         <x:v>The paper identifies observation discrepancy between unimanual and bimanual systems as a transfer risk; detailed failure cases require appendix extraction.</x:v>
       </x:c>
-      <x:c r="BM58" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4405254485","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4405254485, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM58" t="str">
+        <x:v>https://openalex.org/W4405254485</x:v>
       </x:c>
       <x:c r="BN58" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Lu_AnyBimanual_Transferring_Unimanual_Policy_for_General_Bimanual_Manipulation_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -44411,9 +44301,8 @@
       <x:c r="BL59" t="str">
         <x:v>Cross-hand and retargeting edge cases are not detailed in the accessible abstract; full supplementary review is needed.</x:v>
       </x:c>
-      <x:c r="BM59" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7140228196","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7140228196, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM59" t="str">
+        <x:v>https://openalex.org/W7140228196</x:v>
       </x:c>
       <x:c r="BN59" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2026/html/Zhang_UniDex_A_Robot_Foundation_Suite_for_Universal_Dexterous_Hand_Control_CVPR_2026_paper.html；官方摘要/论文集元数据</x:v>
@@ -44650,11 +44539,11 @@
       <x:c r="AT60" t="str">
         <x:v>Generalization / Long-Horizon</x:v>
       </x:c>
-      <x:c r="AU60" t="str">
-        <x:v>—</x:v>
+      <x:c r="AU60" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="AV60" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AW60" t="str">
         <x:v>2026-09-25</x:v>
@@ -44703,7 +44592,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BM60" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/cvpr52734.2025.02578</x:v>
       </x:c>
       <x:c r="BN60" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2025/html/</x:v>
@@ -44745,7 +44634,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="CA60" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="CB60" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -44787,7 +44676,7 @@
         <x:v>官方摘要/论文页; https://openaccess.thecvf.com/content/CVPR2025/html/Zhao_TASTE-Rob_Advancing_Video_Generation_of_Task-Oriented_Hand-Object_Interaction_for_Generalizable_CVPR_2025_paper.html; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CQ60" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-pdf-authors</x:v>
       </x:c>
       <x:c r="CR60" t="n">
         <x:v>0</x:v>
@@ -44989,9 +44878,8 @@
       <x:c r="BL61" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM61" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138113519","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138113519, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM61" t="str">
+        <x:v>https://openalex.org/W7138113519</x:v>
       </x:c>
       <x:c r="BN61" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38874；官方摘要/论文集元数据</x:v>
@@ -45278,9 +45166,8 @@
       <x:c r="BL62" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM62" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4417041439","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4417041439, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM62" t="str">
+        <x:v>https://openalex.org/W4417041439</x:v>
       </x:c>
       <x:c r="BN62" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/e4ef7454447baa15a424314e6284441b-Abstract-Conference.html；官方摘要/论文集元数据</x:v>
@@ -45566,9 +45453,8 @@
       <x:c r="BL63" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM63" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138302344","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138302344, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM63" t="str">
+        <x:v>https://openalex.org/W7138302344</x:v>
       </x:c>
       <x:c r="BN63" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38313；官方摘要/论文集元数据</x:v>
@@ -45854,9 +45740,8 @@
       <x:c r="BL64" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM64" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7138037195","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7138037195, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM64" t="str">
+        <x:v>https://openalex.org/W7138037195</x:v>
       </x:c>
       <x:c r="BN64" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/40127；官方摘要/论文集元数据</x:v>
@@ -46142,9 +46027,8 @@
       <x:c r="BL65" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BM65" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4393158202","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4393158202, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM65" t="str">
+        <x:v>https://openalex.org/W4393158202</x:v>
       </x:c>
       <x:c r="BN65" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/28266；官方摘要/论文集元数据</x:v>
@@ -46431,9 +46315,8 @@
       <x:c r="BL66" t="str">
         <x:v>The paper notes ambiguity/multi-modality of valid interaction regions; exact failure examples require figure-level review.</x:v>
       </x:c>
-      <x:c r="BM66" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4416031407","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4416031407, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM66" t="str">
+        <x:v>https://openalex.org/W4416031407</x:v>
       </x:c>
       <x:c r="BN66" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2025/html/Heidinger_2HandedAfforder_Learning_Precise_Actionable_Bimanual_Affordances_from_Human_Videos_ICCV_2025_paper.html；官方摘要/论文集元数据</x:v>
@@ -46728,9 +46611,8 @@
       <x:c r="BL67" t="str">
         <x:v>Not Explicitly Reported in the accessible official abstract/project evidence.</x:v>
       </x:c>
-      <x:c r="BM67" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W7137985120","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W7137985120, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BM67" t="str">
+        <x:v>https://openalex.org/W7137985120</x:v>
       </x:c>
       <x:c r="BN67" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/38921；https://arxiv.org/abs/2508.10333；https://zionchow.github.io/ReconVLA/；https://github.com/OpenHelix-Team/ReconVLA</x:v>
@@ -46862,7 +46744,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54b74dcd0baf4d58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6736d1e682044cbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -47071,7 +46953,7 @@
         <x:v>Failure Cases</x:v>
       </x:c>
       <x:c r="BB1" t="str">
-        <x:v>Citation Source Identifier</x:v>
+        <x:v>引用量来源链接</x:v>
       </x:c>
       <x:c r="BC1" t="str">
         <x:v>Evidence Sources</x:v>
@@ -47422,7 +47304,7 @@
         <x:v>官方摘要/论文页：https://edem-ai.github.io/sim2realvla.github.io/；核验于 2026-09-23。仅为摘要级速读，原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CF2" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>Unresolved; no reliable citation service count</x:v>
       </x:c>
       <x:c r="CG2" t="n">
         <x:v>0</x:v>
@@ -47591,9 +47473,8 @@
       <x:c r="BA3" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB3" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414050937","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414050937, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB3" t="str">
+        <x:v>https://openalex.org/W4414050937</x:v>
       </x:c>
       <x:c r="BC3" t="str">
         <x:v>https://www.roboticsproceedings.org/rss21/p149.html; https://hnu</x:v>
@@ -47846,9 +47727,8 @@
       <x:c r="BA4" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB4" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4414050727","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4414050727, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB4" t="str">
+        <x:v>https://openalex.org/W4414050727</x:v>
       </x:c>
       <x:c r="BC4" t="str">
         <x:v>RSS official proceedings abstract</x:v>
@@ -48100,9 +47980,8 @@
       <x:c r="BA5" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB5" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/84a351dcc0323aed7fac5755303eb5614fac5f46","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/84a351dcc0323aed7fac5755303eb5614fac5f46, friendlyName=Semantic Scholar</x:v>
+      <x:c r="BB5" t="str">
+        <x:v>https://www.semanticscholar.org/paper/84a351dcc0323aed7fac5755303eb5614fac5f46</x:v>
       </x:c>
       <x:c r="BC5" t="str">
         <x:v>RSS official proceedings</x:v>
@@ -48355,9 +48234,8 @@
       <x:c r="BA6" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB6" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402354166","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402354166, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB6" t="str">
+        <x:v>https://openalex.org/W4402354166</x:v>
       </x:c>
       <x:c r="BC6" t="str">
         <x:v>RSS official proceedings abstract</x:v>
@@ -48611,9 +48489,8 @@
       <x:c r="BA7" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB7" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4401415458","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4401415458, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB7" t="str">
+        <x:v>https://openalex.org/W4401415458</x:v>
       </x:c>
       <x:c r="BC7" t="str">
         <x:v>IEEE Xplore abstract; official project page</x:v>
@@ -48866,9 +48743,8 @@
       <x:c r="BA8" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB8" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4405753615","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4405753615, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB8" t="str">
+        <x:v>https://openalex.org/W4405753615</x:v>
       </x:c>
       <x:c r="BC8" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -49071,11 +48947,11 @@
       <x:c r="AJ9" t="str">
         <x:v>Bimanual</x:v>
       </x:c>
-      <x:c r="AK9" t="str">
-        <x:v>—</x:v>
+      <x:c r="AK9" t="n">
+        <x:v>10</x:v>
       </x:c>
       <x:c r="AL9" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AM9" t="str">
         <x:v>2026-09-25</x:v>
@@ -49121,7 +48997,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB9" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/tro.2024.3502223</x:v>
       </x:c>
       <x:c r="BC9" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -49161,7 +49037,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BP9" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BQ9" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -49203,7 +49079,7 @@
         <x:v>OpenAlex 索引摘要; https://api.openalex.org/works/W4404520558; 核验于 2026-09-23. 仅为摘要级速读；原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CF9" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-official-publisher</x:v>
       </x:c>
       <x:c r="CG9" t="n">
         <x:v>0</x:v>
@@ -49322,11 +49198,11 @@
       <x:c r="AJ10" t="str">
         <x:v>Dexterous</x:v>
       </x:c>
-      <x:c r="AK10" t="str">
-        <x:v>—</x:v>
+      <x:c r="AK10" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="AL10" t="str">
-        <x:v>未可靠匹配</x:v>
+        <x:v>Crossref</x:v>
       </x:c>
       <x:c r="AM10" t="str">
         <x:v>2026-09-25</x:v>
@@ -49372,7 +49248,7 @@
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
       <x:c r="BB10" t="str">
-        <x:v>—</x:v>
+        <x:v>https://api.crossref.org/works/10.1109/lra.2025.3558699</x:v>
       </x:c>
       <x:c r="BC10" t="str">
         <x:v>IEEE Xplore abstract</x:v>
@@ -49412,7 +49288,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="BP10" t="str">
-        <x:v>Unresolved</x:v>
+        <x:v>Matched</x:v>
       </x:c>
       <x:c r="BQ10" t="str">
         <x:v>Not Found After Verification</x:v>
@@ -49454,7 +49330,7 @@
         <x:v>官方摘要/论文页：https://ieeexplore.ieee.org/document/10955245/；核验于 2026-09-23。仅为摘要级速读，原 Evidence Quality 不变。 - 核验层级：摘要有可追溯来源</x:v>
       </x:c>
       <x:c r="CF10" t="str">
-        <x:v>Unresolved; insufficient identity evidence</x:v>
+        <x:v>crossref-exact-title-official-publisher</x:v>
       </x:c>
       <x:c r="CG10" t="n">
         <x:v>0</x:v>
@@ -49602,9 +49478,8 @@
       <x:c r="BA11" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB11" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402353985","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402353985, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB11" t="str">
+        <x:v>https://openalex.org/W4402353985</x:v>
       </x:c>
       <x:c r="BC11" t="str">
         <x:v>Unknown</x:v>
@@ -49831,9 +49706,8 @@
       <x:c r="BA12" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB12" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4402354047","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4402354047, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB12" t="str">
+        <x:v>https://openalex.org/W4402354047</x:v>
       </x:c>
       <x:c r="BC12" t="str">
         <x:v>Unknown</x:v>
@@ -50063,9 +49937,8 @@
       <x:c r="BA13" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB13" t="e">
-        <x:f>HYPERLINK("https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632","Semantic Scholar")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632, friendlyName=Semantic Scholar</x:v>
+      <x:c r="BB13" t="str">
+        <x:v>https://www.semanticscholar.org/paper/a294546084fda4e0f12f307caed4f9c58f051632</x:v>
       </x:c>
       <x:c r="BC13" t="str">
         <x:v>Unknown</x:v>
@@ -50294,9 +50167,8 @@
       <x:c r="BA14" t="str">
         <x:v>Unknown / Not Explicitly Reported in the currently accessible sources.</x:v>
       </x:c>
-      <x:c r="BB14" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4387764390","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4387764390, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB14" t="str">
+        <x:v>https://openalex.org/W4387764390</x:v>
       </x:c>
       <x:c r="BC14" t="str">
         <x:v>Unknown</x:v>
@@ -50550,9 +50422,8 @@
       <x:c r="BA15" t="str">
         <x:v>Planning errors, low-level execution, drawer manipulation, embodiment limits.</x:v>
       </x:c>
-      <x:c r="BB15" t="e">
-        <x:f>HYPERLINK("https://openalex.org/W4224912544","OpenAlex Work")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://openalex.org/W4224912544, friendlyName=OpenAlex Work</x:v>
+      <x:c r="BB15" t="str">
+        <x:v>https://openalex.org/W4224912544</x:v>
       </x:c>
       <x:c r="BC15" t="str">
         <x:v>Google Research; arXiv; CoRL/PMLR; project page; official repository</x:v>
@@ -50673,7 +50544,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e9107d5f17a4d56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d883dfc0d7141c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>